<commit_message>
📊 체감온도 기록: 2026-09-13 19:40 KST
</commit_message>
<xml_diff>
--- a/data/체감온도기록_2026.xlsx
+++ b/data/체감온도기록_2026.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3698" uniqueCount="403">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3714" uniqueCount="404">
   <si>
     <t>성동자이리버뷰 체감온도 기록</t>
   </si>
@@ -1223,6 +1223,9 @@
   </si>
   <si>
     <t>14:21</t>
+  </si>
+  <si>
+    <t>19:40</t>
   </si>
 </sst>
 </file>
@@ -1643,7 +1646,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G920"/>
+  <dimension ref="A1:G924"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
@@ -22800,6 +22803,98 @@
         <v>11</v>
       </c>
     </row>
+    <row r="921" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A921" s="5" t="s">
+        <v>400</v>
+      </c>
+      <c r="B921" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="C921" s="5" t="s">
+        <v>403</v>
+      </c>
+      <c r="D921" s="5">
+        <v>23.6</v>
+      </c>
+      <c r="E921" s="5">
+        <v>61</v>
+      </c>
+      <c r="F921" s="5">
+        <v>24</v>
+      </c>
+      <c r="G921" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="922" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A922" s="5" t="s">
+        <v>400</v>
+      </c>
+      <c r="B922" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="C922" s="5" t="s">
+        <v>403</v>
+      </c>
+      <c r="D922" s="5">
+        <v>23.9</v>
+      </c>
+      <c r="E922" s="5">
+        <v>56</v>
+      </c>
+      <c r="F922" s="5">
+        <v>24</v>
+      </c>
+      <c r="G922" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="923" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A923" s="5" t="s">
+        <v>400</v>
+      </c>
+      <c r="B923" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="C923" s="5" t="s">
+        <v>403</v>
+      </c>
+      <c r="D923" s="5">
+        <v>24.1</v>
+      </c>
+      <c r="E923" s="5">
+        <v>55</v>
+      </c>
+      <c r="F923" s="5">
+        <v>24</v>
+      </c>
+      <c r="G923" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="924" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A924" s="5" t="s">
+        <v>400</v>
+      </c>
+      <c r="B924" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="C924" s="5" t="s">
+        <v>403</v>
+      </c>
+      <c r="D924" s="5">
+        <v>23.9</v>
+      </c>
+      <c r="E924" s="5">
+        <v>60</v>
+      </c>
+      <c r="F924" s="5">
+        <v>24</v>
+      </c>
+      <c r="G924" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>

</xml_diff>

<commit_message>
📊 체감온도 기록: 2026-09-14 09:26 KST
</commit_message>
<xml_diff>
--- a/data/체감온도기록_2026.xlsx
+++ b/data/체감온도기록_2026.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3714" uniqueCount="404">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3722" uniqueCount="406">
   <si>
     <t>성동자이리버뷰 체감온도 기록</t>
   </si>
@@ -1226,6 +1226,12 @@
   </si>
   <si>
     <t>19:40</t>
+  </si>
+  <si>
+    <t>2026-09-14</t>
+  </si>
+  <si>
+    <t>09:26</t>
   </si>
 </sst>
 </file>
@@ -1646,7 +1652,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G924"/>
+  <dimension ref="A1:G926"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
@@ -22895,6 +22901,52 @@
         <v>11</v>
       </c>
     </row>
+    <row r="925" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A925" s="5" t="s">
+        <v>404</v>
+      </c>
+      <c r="B925" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="C925" s="5" t="s">
+        <v>405</v>
+      </c>
+      <c r="D925" s="5">
+        <v>19.7</v>
+      </c>
+      <c r="E925" s="5">
+        <v>83</v>
+      </c>
+      <c r="F925" s="5">
+        <v>22</v>
+      </c>
+      <c r="G925" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="926" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A926" s="5" t="s">
+        <v>404</v>
+      </c>
+      <c r="B926" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="C926" s="5" t="s">
+        <v>405</v>
+      </c>
+      <c r="D926" s="5">
+        <v>20.2</v>
+      </c>
+      <c r="E926" s="5">
+        <v>81</v>
+      </c>
+      <c r="F926" s="5">
+        <v>22</v>
+      </c>
+      <c r="G926" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>

</xml_diff>

<commit_message>
📊 체감온도 기록: 2026-09-14 14:27 KST
</commit_message>
<xml_diff>
--- a/data/체감온도기록_2026.xlsx
+++ b/data/체감온도기록_2026.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3722" uniqueCount="406">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3742" uniqueCount="407">
   <si>
     <t>성동자이리버뷰 체감온도 기록</t>
   </si>
@@ -1232,6 +1232,9 @@
   </si>
   <si>
     <t>09:26</t>
+  </si>
+  <si>
+    <t>14:26</t>
   </si>
 </sst>
 </file>
@@ -1652,7 +1655,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G926"/>
+  <dimension ref="A1:G931"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
@@ -22947,6 +22950,121 @@
         <v>11</v>
       </c>
     </row>
+    <row r="927" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A927" s="5" t="s">
+        <v>404</v>
+      </c>
+      <c r="B927" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="C927" s="5" t="s">
+        <v>406</v>
+      </c>
+      <c r="D927" s="5">
+        <v>22.1</v>
+      </c>
+      <c r="E927" s="5">
+        <v>72</v>
+      </c>
+      <c r="F927" s="5">
+        <v>24</v>
+      </c>
+      <c r="G927" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="928" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A928" s="5" t="s">
+        <v>404</v>
+      </c>
+      <c r="B928" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C928" s="5" t="s">
+        <v>406</v>
+      </c>
+      <c r="D928" s="5">
+        <v>23.6</v>
+      </c>
+      <c r="E928" s="5">
+        <v>63</v>
+      </c>
+      <c r="F928" s="5">
+        <v>24</v>
+      </c>
+      <c r="G928" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="929" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A929" s="5" t="s">
+        <v>404</v>
+      </c>
+      <c r="B929" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="C929" s="5" t="s">
+        <v>406</v>
+      </c>
+      <c r="D929" s="5">
+        <v>24.2</v>
+      </c>
+      <c r="E929" s="5">
+        <v>59</v>
+      </c>
+      <c r="F929" s="5">
+        <v>25</v>
+      </c>
+      <c r="G929" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="930" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A930" s="5" t="s">
+        <v>404</v>
+      </c>
+      <c r="B930" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="C930" s="5" t="s">
+        <v>406</v>
+      </c>
+      <c r="D930" s="5">
+        <v>24.6</v>
+      </c>
+      <c r="E930" s="5">
+        <v>57</v>
+      </c>
+      <c r="F930" s="5">
+        <v>25</v>
+      </c>
+      <c r="G930" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="931" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A931" s="5" t="s">
+        <v>404</v>
+      </c>
+      <c r="B931" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="C931" s="5" t="s">
+        <v>406</v>
+      </c>
+      <c r="D931" s="5">
+        <v>25</v>
+      </c>
+      <c r="E931" s="5">
+        <v>50</v>
+      </c>
+      <c r="F931" s="5">
+        <v>25</v>
+      </c>
+      <c r="G931" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>

</xml_diff>

<commit_message>
📊 체감온도 기록: 2026-09-14 19:58 KST
</commit_message>
<xml_diff>
--- a/data/체감온도기록_2026.xlsx
+++ b/data/체감온도기록_2026.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3742" uniqueCount="407">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3758" uniqueCount="408">
   <si>
     <t>성동자이리버뷰 체감온도 기록</t>
   </si>
@@ -1235,6 +1235,9 @@
   </si>
   <si>
     <t>14:26</t>
+  </si>
+  <si>
+    <t>19:58</t>
   </si>
 </sst>
 </file>
@@ -1655,7 +1658,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G931"/>
+  <dimension ref="A1:G935"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
@@ -23065,6 +23068,98 @@
         <v>11</v>
       </c>
     </row>
+    <row r="932" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A932" s="5" t="s">
+        <v>404</v>
+      </c>
+      <c r="B932" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="C932" s="5" t="s">
+        <v>407</v>
+      </c>
+      <c r="D932" s="5">
+        <v>25.5</v>
+      </c>
+      <c r="E932" s="5">
+        <v>48</v>
+      </c>
+      <c r="F932" s="5">
+        <v>25</v>
+      </c>
+      <c r="G932" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="933" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A933" s="5" t="s">
+        <v>404</v>
+      </c>
+      <c r="B933" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="C933" s="5" t="s">
+        <v>407</v>
+      </c>
+      <c r="D933" s="5">
+        <v>26.8</v>
+      </c>
+      <c r="E933" s="5">
+        <v>35</v>
+      </c>
+      <c r="F933" s="5">
+        <v>25</v>
+      </c>
+      <c r="G933" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="934" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A934" s="5" t="s">
+        <v>404</v>
+      </c>
+      <c r="B934" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="C934" s="5" t="s">
+        <v>407</v>
+      </c>
+      <c r="D934" s="5">
+        <v>27.2</v>
+      </c>
+      <c r="E934" s="5">
+        <v>37</v>
+      </c>
+      <c r="F934" s="5">
+        <v>26</v>
+      </c>
+      <c r="G934" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="935" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A935" s="5" t="s">
+        <v>404</v>
+      </c>
+      <c r="B935" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="C935" s="5" t="s">
+        <v>407</v>
+      </c>
+      <c r="D935" s="5">
+        <v>26.9</v>
+      </c>
+      <c r="E935" s="5">
+        <v>33</v>
+      </c>
+      <c r="F935" s="5">
+        <v>25</v>
+      </c>
+      <c r="G935" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>

</xml_diff>

<commit_message>
📊 체감온도 기록: 2026-09-15 15:42 KST
</commit_message>
<xml_diff>
--- a/data/체감온도기록_2026.xlsx
+++ b/data/체감온도기록_2026.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3758" uniqueCount="408">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3794" uniqueCount="410">
   <si>
     <t>성동자이리버뷰 체감온도 기록</t>
   </si>
@@ -1238,6 +1238,12 @@
   </si>
   <si>
     <t>19:58</t>
+  </si>
+  <si>
+    <t>2026-09-15</t>
+  </si>
+  <si>
+    <t>15:42</t>
   </si>
 </sst>
 </file>
@@ -1658,7 +1664,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G935"/>
+  <dimension ref="A1:G944"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
@@ -23160,6 +23166,213 @@
         <v>11</v>
       </c>
     </row>
+    <row r="936" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A936" s="5" t="s">
+        <v>408</v>
+      </c>
+      <c r="B936" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="C936" s="5" t="s">
+        <v>409</v>
+      </c>
+      <c r="D936" s="5">
+        <v>16.5</v>
+      </c>
+      <c r="E936" s="5">
+        <v>67</v>
+      </c>
+      <c r="F936" s="5">
+        <v>18</v>
+      </c>
+      <c r="G936" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="937" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A937" s="5" t="s">
+        <v>408</v>
+      </c>
+      <c r="B937" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="C937" s="5" t="s">
+        <v>409</v>
+      </c>
+      <c r="D937" s="5">
+        <v>17.8</v>
+      </c>
+      <c r="E937" s="5">
+        <v>61</v>
+      </c>
+      <c r="F937" s="5">
+        <v>18</v>
+      </c>
+      <c r="G937" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="938" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A938" s="5" t="s">
+        <v>408</v>
+      </c>
+      <c r="B938" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="C938" s="5" t="s">
+        <v>409</v>
+      </c>
+      <c r="D938" s="5">
+        <v>20.4</v>
+      </c>
+      <c r="E938" s="5">
+        <v>54</v>
+      </c>
+      <c r="F938" s="5">
+        <v>21</v>
+      </c>
+      <c r="G938" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="939" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A939" s="5" t="s">
+        <v>408</v>
+      </c>
+      <c r="B939" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C939" s="5" t="s">
+        <v>409</v>
+      </c>
+      <c r="D939" s="5">
+        <v>22.4</v>
+      </c>
+      <c r="E939" s="5">
+        <v>45</v>
+      </c>
+      <c r="F939" s="5">
+        <v>22</v>
+      </c>
+      <c r="G939" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="940" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A940" s="5" t="s">
+        <v>408</v>
+      </c>
+      <c r="B940" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="C940" s="5" t="s">
+        <v>409</v>
+      </c>
+      <c r="D940" s="5">
+        <v>24.3</v>
+      </c>
+      <c r="E940" s="5">
+        <v>37</v>
+      </c>
+      <c r="F940" s="5">
+        <v>23</v>
+      </c>
+      <c r="G940" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="941" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A941" s="5" t="s">
+        <v>408</v>
+      </c>
+      <c r="B941" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="C941" s="5" t="s">
+        <v>409</v>
+      </c>
+      <c r="D941" s="5">
+        <v>25.5</v>
+      </c>
+      <c r="E941" s="5">
+        <v>31</v>
+      </c>
+      <c r="F941" s="5">
+        <v>23</v>
+      </c>
+      <c r="G941" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="942" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A942" s="5" t="s">
+        <v>408</v>
+      </c>
+      <c r="B942" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="C942" s="5" t="s">
+        <v>409</v>
+      </c>
+      <c r="D942" s="5">
+        <v>25.9</v>
+      </c>
+      <c r="E942" s="5">
+        <v>30</v>
+      </c>
+      <c r="F942" s="5">
+        <v>24</v>
+      </c>
+      <c r="G942" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="943" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A943" s="5" t="s">
+        <v>408</v>
+      </c>
+      <c r="B943" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="C943" s="5" t="s">
+        <v>409</v>
+      </c>
+      <c r="D943" s="5">
+        <v>26.7</v>
+      </c>
+      <c r="E943" s="5">
+        <v>27</v>
+      </c>
+      <c r="F943" s="5">
+        <v>24</v>
+      </c>
+      <c r="G943" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="944" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A944" s="5" t="s">
+        <v>408</v>
+      </c>
+      <c r="B944" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="C944" s="5" t="s">
+        <v>409</v>
+      </c>
+      <c r="D944" s="5">
+        <v>27</v>
+      </c>
+      <c r="E944" s="5">
+        <v>23</v>
+      </c>
+      <c r="F944" s="5">
+        <v>24</v>
+      </c>
+      <c r="G944" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>

</xml_diff>

<commit_message>
📊 체감온도 기록: 2026-09-15 21:09 KST
</commit_message>
<xml_diff>
--- a/data/체감온도기록_2026.xlsx
+++ b/data/체감온도기록_2026.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3794" uniqueCount="410">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3802" uniqueCount="411">
   <si>
     <t>성동자이리버뷰 체감온도 기록</t>
   </si>
@@ -1244,6 +1244,9 @@
   </si>
   <si>
     <t>15:42</t>
+  </si>
+  <si>
+    <t>21:09</t>
   </si>
 </sst>
 </file>
@@ -1664,7 +1667,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G944"/>
+  <dimension ref="A1:G946"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
@@ -23373,6 +23376,52 @@
         <v>11</v>
       </c>
     </row>
+    <row r="945" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A945" s="5" t="s">
+        <v>408</v>
+      </c>
+      <c r="B945" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="C945" s="5" t="s">
+        <v>410</v>
+      </c>
+      <c r="D945" s="5">
+        <v>26.5</v>
+      </c>
+      <c r="E945" s="5">
+        <v>23</v>
+      </c>
+      <c r="F945" s="5">
+        <v>23</v>
+      </c>
+      <c r="G945" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="946" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A946" s="5" t="s">
+        <v>408</v>
+      </c>
+      <c r="B946" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="C946" s="5" t="s">
+        <v>410</v>
+      </c>
+      <c r="D946" s="5">
+        <v>26.2</v>
+      </c>
+      <c r="E946" s="5">
+        <v>27</v>
+      </c>
+      <c r="F946" s="5">
+        <v>24</v>
+      </c>
+      <c r="G946" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>

</xml_diff>

<commit_message>
📊 체감온도 기록: 2026-09-16 09:48 KST
</commit_message>
<xml_diff>
--- a/data/체감온도기록_2026.xlsx
+++ b/data/체감온도기록_2026.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3802" uniqueCount="411">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3814" uniqueCount="413">
   <si>
     <t>성동자이리버뷰 체감온도 기록</t>
   </si>
@@ -1247,6 +1247,12 @@
   </si>
   <si>
     <t>21:09</t>
+  </si>
+  <si>
+    <t>2026-09-16</t>
+  </si>
+  <si>
+    <t>09:48</t>
   </si>
 </sst>
 </file>
@@ -1667,7 +1673,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G946"/>
+  <dimension ref="A1:G949"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
@@ -23422,6 +23428,75 @@
         <v>11</v>
       </c>
     </row>
+    <row r="947" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A947" s="5" t="s">
+        <v>411</v>
+      </c>
+      <c r="B947" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="C947" s="5" t="s">
+        <v>412</v>
+      </c>
+      <c r="D947" s="5">
+        <v>15.5</v>
+      </c>
+      <c r="E947" s="5">
+        <v>72</v>
+      </c>
+      <c r="F947" s="5">
+        <v>17</v>
+      </c>
+      <c r="G947" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="948" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A948" s="5" t="s">
+        <v>411</v>
+      </c>
+      <c r="B948" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="C948" s="5" t="s">
+        <v>412</v>
+      </c>
+      <c r="D948" s="5">
+        <v>17.6</v>
+      </c>
+      <c r="E948" s="5">
+        <v>61</v>
+      </c>
+      <c r="F948" s="5">
+        <v>18</v>
+      </c>
+      <c r="G948" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="949" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A949" s="5" t="s">
+        <v>411</v>
+      </c>
+      <c r="B949" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="C949" s="5" t="s">
+        <v>412</v>
+      </c>
+      <c r="D949" s="5">
+        <v>19.3</v>
+      </c>
+      <c r="E949" s="5">
+        <v>53</v>
+      </c>
+      <c r="F949" s="5">
+        <v>19</v>
+      </c>
+      <c r="G949" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>

</xml_diff>

<commit_message>
📊 체감온도 기록: 2026-09-16 21:50 KST
</commit_message>
<xml_diff>
--- a/data/체감온도기록_2026.xlsx
+++ b/data/체감온도기록_2026.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3814" uniqueCount="413">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3846" uniqueCount="414">
   <si>
     <t>성동자이리버뷰 체감온도 기록</t>
   </si>
@@ -1253,6 +1253,9 @@
   </si>
   <si>
     <t>09:48</t>
+  </si>
+  <si>
+    <t>21:49</t>
   </si>
 </sst>
 </file>
@@ -1673,7 +1676,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G949"/>
+  <dimension ref="A1:G957"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
@@ -23497,6 +23500,190 @@
         <v>11</v>
       </c>
     </row>
+    <row r="950" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A950" s="5" t="s">
+        <v>411</v>
+      </c>
+      <c r="B950" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C950" s="5" t="s">
+        <v>413</v>
+      </c>
+      <c r="D950" s="5">
+        <v>21.8</v>
+      </c>
+      <c r="E950" s="5">
+        <v>46</v>
+      </c>
+      <c r="F950" s="5">
+        <v>21</v>
+      </c>
+      <c r="G950" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="951" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A951" s="5" t="s">
+        <v>411</v>
+      </c>
+      <c r="B951" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="C951" s="5" t="s">
+        <v>413</v>
+      </c>
+      <c r="D951" s="5">
+        <v>23.8</v>
+      </c>
+      <c r="E951" s="5">
+        <v>41</v>
+      </c>
+      <c r="F951" s="5">
+        <v>23</v>
+      </c>
+      <c r="G951" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="952" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A952" s="5" t="s">
+        <v>411</v>
+      </c>
+      <c r="B952" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="C952" s="5" t="s">
+        <v>413</v>
+      </c>
+      <c r="D952" s="5">
+        <v>25.9</v>
+      </c>
+      <c r="E952" s="5">
+        <v>38</v>
+      </c>
+      <c r="F952" s="5">
+        <v>24</v>
+      </c>
+      <c r="G952" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="953" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A953" s="5" t="s">
+        <v>411</v>
+      </c>
+      <c r="B953" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="C953" s="5" t="s">
+        <v>413</v>
+      </c>
+      <c r="D953" s="5">
+        <v>26.7</v>
+      </c>
+      <c r="E953" s="5">
+        <v>22</v>
+      </c>
+      <c r="F953" s="5">
+        <v>23</v>
+      </c>
+      <c r="G953" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="954" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A954" s="5" t="s">
+        <v>411</v>
+      </c>
+      <c r="B954" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="C954" s="5" t="s">
+        <v>413</v>
+      </c>
+      <c r="D954" s="5">
+        <v>28.1</v>
+      </c>
+      <c r="E954" s="5">
+        <v>18</v>
+      </c>
+      <c r="F954" s="5">
+        <v>24</v>
+      </c>
+      <c r="G954" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="955" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A955" s="5" t="s">
+        <v>411</v>
+      </c>
+      <c r="B955" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="C955" s="5" t="s">
+        <v>413</v>
+      </c>
+      <c r="D955" s="5">
+        <v>28</v>
+      </c>
+      <c r="E955" s="5">
+        <v>22</v>
+      </c>
+      <c r="F955" s="5">
+        <v>25</v>
+      </c>
+      <c r="G955" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="956" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A956" s="5" t="s">
+        <v>411</v>
+      </c>
+      <c r="B956" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="C956" s="5" t="s">
+        <v>413</v>
+      </c>
+      <c r="D956" s="5">
+        <v>28</v>
+      </c>
+      <c r="E956" s="5">
+        <v>16</v>
+      </c>
+      <c r="F956" s="5">
+        <v>24</v>
+      </c>
+      <c r="G956" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="957" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A957" s="5" t="s">
+        <v>411</v>
+      </c>
+      <c r="B957" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="C957" s="5" t="s">
+        <v>413</v>
+      </c>
+      <c r="D957" s="5">
+        <v>27.8</v>
+      </c>
+      <c r="E957" s="5">
+        <v>27</v>
+      </c>
+      <c r="F957" s="5">
+        <v>25</v>
+      </c>
+      <c r="G957" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>

</xml_diff>

<commit_message>
📊 체감온도 기록: 2026-09-17 09:53 KST
</commit_message>
<xml_diff>
--- a/data/체감온도기록_2026.xlsx
+++ b/data/체감온도기록_2026.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3846" uniqueCount="414">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3858" uniqueCount="416">
   <si>
     <t>성동자이리버뷰 체감온도 기록</t>
   </si>
@@ -1256,6 +1256,12 @@
   </si>
   <si>
     <t>21:49</t>
+  </si>
+  <si>
+    <t>2026-09-17</t>
+  </si>
+  <si>
+    <t>09:52</t>
   </si>
 </sst>
 </file>
@@ -1676,7 +1682,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G957"/>
+  <dimension ref="A1:G960"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
@@ -23684,6 +23690,75 @@
         <v>11</v>
       </c>
     </row>
+    <row r="958" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A958" s="5" t="s">
+        <v>414</v>
+      </c>
+      <c r="B958" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="C958" s="5" t="s">
+        <v>415</v>
+      </c>
+      <c r="D958" s="5">
+        <v>18.8</v>
+      </c>
+      <c r="E958" s="5">
+        <v>64</v>
+      </c>
+      <c r="F958" s="5">
+        <v>20</v>
+      </c>
+      <c r="G958" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="959" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A959" s="5" t="s">
+        <v>414</v>
+      </c>
+      <c r="B959" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="C959" s="5" t="s">
+        <v>415</v>
+      </c>
+      <c r="D959" s="5">
+        <v>21</v>
+      </c>
+      <c r="E959" s="5">
+        <v>53</v>
+      </c>
+      <c r="F959" s="5">
+        <v>21</v>
+      </c>
+      <c r="G959" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="960" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A960" s="5" t="s">
+        <v>414</v>
+      </c>
+      <c r="B960" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="C960" s="5" t="s">
+        <v>415</v>
+      </c>
+      <c r="D960" s="5">
+        <v>21.8</v>
+      </c>
+      <c r="E960" s="5">
+        <v>50</v>
+      </c>
+      <c r="F960" s="5">
+        <v>22</v>
+      </c>
+      <c r="G960" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>

</xml_diff>

<commit_message>
📊 체감온도 기록: 2026-09-17 15:39 KST
</commit_message>
<xml_diff>
--- a/data/체감온도기록_2026.xlsx
+++ b/data/체감온도기록_2026.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3858" uniqueCount="416">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3878" uniqueCount="417">
   <si>
     <t>성동자이리버뷰 체감온도 기록</t>
   </si>
@@ -1262,6 +1262,9 @@
   </si>
   <si>
     <t>09:52</t>
+  </si>
+  <si>
+    <t>15:38</t>
   </si>
 </sst>
 </file>
@@ -1682,7 +1685,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G960"/>
+  <dimension ref="A1:G965"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
@@ -23759,6 +23762,121 @@
         <v>11</v>
       </c>
     </row>
+    <row r="961" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A961" s="5" t="s">
+        <v>414</v>
+      </c>
+      <c r="B961" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C961" s="5" t="s">
+        <v>416</v>
+      </c>
+      <c r="D961" s="5">
+        <v>23.7</v>
+      </c>
+      <c r="E961" s="5">
+        <v>47</v>
+      </c>
+      <c r="F961" s="5">
+        <v>23</v>
+      </c>
+      <c r="G961" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="962" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A962" s="5" t="s">
+        <v>414</v>
+      </c>
+      <c r="B962" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="C962" s="5" t="s">
+        <v>416</v>
+      </c>
+      <c r="D962" s="5">
+        <v>24.4</v>
+      </c>
+      <c r="E962" s="5">
+        <v>45</v>
+      </c>
+      <c r="F962" s="5">
+        <v>24</v>
+      </c>
+      <c r="G962" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="963" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A963" s="5" t="s">
+        <v>414</v>
+      </c>
+      <c r="B963" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="C963" s="5" t="s">
+        <v>416</v>
+      </c>
+      <c r="D963" s="5">
+        <v>26</v>
+      </c>
+      <c r="E963" s="5">
+        <v>43</v>
+      </c>
+      <c r="F963" s="5">
+        <v>25</v>
+      </c>
+      <c r="G963" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="964" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A964" s="5" t="s">
+        <v>414</v>
+      </c>
+      <c r="B964" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="C964" s="5" t="s">
+        <v>416</v>
+      </c>
+      <c r="D964" s="5">
+        <v>26.5</v>
+      </c>
+      <c r="E964" s="5">
+        <v>43</v>
+      </c>
+      <c r="F964" s="5">
+        <v>26</v>
+      </c>
+      <c r="G964" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="965" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A965" s="5" t="s">
+        <v>414</v>
+      </c>
+      <c r="B965" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="C965" s="5" t="s">
+        <v>416</v>
+      </c>
+      <c r="D965" s="5">
+        <v>27.1</v>
+      </c>
+      <c r="E965" s="5">
+        <v>42</v>
+      </c>
+      <c r="F965" s="5">
+        <v>26</v>
+      </c>
+      <c r="G965" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>

</xml_diff>

<commit_message>
📊 체감온도 기록: 2026-09-17 21:05 KST
</commit_message>
<xml_diff>
--- a/data/체감온도기록_2026.xlsx
+++ b/data/체감온도기록_2026.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3878" uniqueCount="417">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3890" uniqueCount="418">
   <si>
     <t>성동자이리버뷰 체감온도 기록</t>
   </si>
@@ -1265,6 +1265,9 @@
   </si>
   <si>
     <t>15:38</t>
+  </si>
+  <si>
+    <t>21:05</t>
   </si>
 </sst>
 </file>
@@ -1685,7 +1688,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G965"/>
+  <dimension ref="A1:G968"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
@@ -23877,6 +23880,75 @@
         <v>11</v>
       </c>
     </row>
+    <row r="966" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A966" s="5" t="s">
+        <v>414</v>
+      </c>
+      <c r="B966" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="C966" s="5" t="s">
+        <v>417</v>
+      </c>
+      <c r="D966" s="5">
+        <v>26.8</v>
+      </c>
+      <c r="E966" s="5">
+        <v>44</v>
+      </c>
+      <c r="F966" s="5">
+        <v>26</v>
+      </c>
+      <c r="G966" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="967" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A967" s="5" t="s">
+        <v>414</v>
+      </c>
+      <c r="B967" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="C967" s="5" t="s">
+        <v>417</v>
+      </c>
+      <c r="D967" s="5">
+        <v>26.6</v>
+      </c>
+      <c r="E967" s="5">
+        <v>46</v>
+      </c>
+      <c r="F967" s="5">
+        <v>26</v>
+      </c>
+      <c r="G967" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="968" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A968" s="5" t="s">
+        <v>414</v>
+      </c>
+      <c r="B968" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="C968" s="5" t="s">
+        <v>417</v>
+      </c>
+      <c r="D968" s="5">
+        <v>26.3</v>
+      </c>
+      <c r="E968" s="5">
+        <v>47</v>
+      </c>
+      <c r="F968" s="5">
+        <v>26</v>
+      </c>
+      <c r="G968" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>

</xml_diff>

<commit_message>
📊 체감온도 기록: 2026-09-18 15:39 KST
</commit_message>
<xml_diff>
--- a/data/체감온도기록_2026.xlsx
+++ b/data/체감온도기록_2026.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3890" uniqueCount="418">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3922" uniqueCount="420">
   <si>
     <t>성동자이리버뷰 체감온도 기록</t>
   </si>
@@ -1268,6 +1268,12 @@
   </si>
   <si>
     <t>21:05</t>
+  </si>
+  <si>
+    <t>2026-09-18</t>
+  </si>
+  <si>
+    <t>15:39</t>
   </si>
 </sst>
 </file>
@@ -1688,7 +1694,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G968"/>
+  <dimension ref="A1:G976"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
@@ -23949,6 +23955,190 @@
         <v>11</v>
       </c>
     </row>
+    <row r="969" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A969" s="5" t="s">
+        <v>418</v>
+      </c>
+      <c r="B969" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="C969" s="5" t="s">
+        <v>419</v>
+      </c>
+      <c r="D969" s="5">
+        <v>20.2</v>
+      </c>
+      <c r="E969" s="5">
+        <v>61</v>
+      </c>
+      <c r="F969" s="5">
+        <v>21</v>
+      </c>
+      <c r="G969" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="970" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A970" s="5" t="s">
+        <v>418</v>
+      </c>
+      <c r="B970" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="C970" s="5" t="s">
+        <v>419</v>
+      </c>
+      <c r="D970" s="5">
+        <v>22.2</v>
+      </c>
+      <c r="E970" s="5">
+        <v>55</v>
+      </c>
+      <c r="F970" s="5">
+        <v>22</v>
+      </c>
+      <c r="G970" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="971" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A971" s="5" t="s">
+        <v>418</v>
+      </c>
+      <c r="B971" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="C971" s="5" t="s">
+        <v>419</v>
+      </c>
+      <c r="D971" s="5">
+        <v>23.8</v>
+      </c>
+      <c r="E971" s="5">
+        <v>51</v>
+      </c>
+      <c r="F971" s="5">
+        <v>24</v>
+      </c>
+      <c r="G971" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="972" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A972" s="5" t="s">
+        <v>418</v>
+      </c>
+      <c r="B972" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C972" s="5" t="s">
+        <v>419</v>
+      </c>
+      <c r="D972" s="5">
+        <v>25</v>
+      </c>
+      <c r="E972" s="5">
+        <v>47</v>
+      </c>
+      <c r="F972" s="5">
+        <v>24</v>
+      </c>
+      <c r="G972" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="973" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A973" s="5" t="s">
+        <v>418</v>
+      </c>
+      <c r="B973" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="C973" s="5" t="s">
+        <v>419</v>
+      </c>
+      <c r="D973" s="5">
+        <v>25.6</v>
+      </c>
+      <c r="E973" s="5">
+        <v>46</v>
+      </c>
+      <c r="F973" s="5">
+        <v>25</v>
+      </c>
+      <c r="G973" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="974" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A974" s="5" t="s">
+        <v>418</v>
+      </c>
+      <c r="B974" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="C974" s="5" t="s">
+        <v>419</v>
+      </c>
+      <c r="D974" s="5">
+        <v>26.6</v>
+      </c>
+      <c r="E974" s="5">
+        <v>44</v>
+      </c>
+      <c r="F974" s="5">
+        <v>26</v>
+      </c>
+      <c r="G974" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="975" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A975" s="5" t="s">
+        <v>418</v>
+      </c>
+      <c r="B975" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="C975" s="5" t="s">
+        <v>419</v>
+      </c>
+      <c r="D975" s="5">
+        <v>27.2</v>
+      </c>
+      <c r="E975" s="5">
+        <v>43</v>
+      </c>
+      <c r="F975" s="5">
+        <v>26</v>
+      </c>
+      <c r="G975" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="976" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A976" s="5" t="s">
+        <v>418</v>
+      </c>
+      <c r="B976" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="C976" s="5" t="s">
+        <v>419</v>
+      </c>
+      <c r="D976" s="5">
+        <v>28.4</v>
+      </c>
+      <c r="E976" s="5">
+        <v>41</v>
+      </c>
+      <c r="F976" s="5">
+        <v>27</v>
+      </c>
+      <c r="G976" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>

</xml_diff>

<commit_message>
📊 체감온도 기록: 2026-09-18 20:49 KST
</commit_message>
<xml_diff>
--- a/data/체감온도기록_2026.xlsx
+++ b/data/체감온도기록_2026.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3922" uniqueCount="420">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3934" uniqueCount="421">
   <si>
     <t>성동자이리버뷰 체감온도 기록</t>
   </si>
@@ -1274,6 +1274,9 @@
   </si>
   <si>
     <t>15:39</t>
+  </si>
+  <si>
+    <t>20:49</t>
   </si>
 </sst>
 </file>
@@ -1694,7 +1697,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G976"/>
+  <dimension ref="A1:G979"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
@@ -24139,6 +24142,75 @@
         <v>11</v>
       </c>
     </row>
+    <row r="977" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A977" s="5" t="s">
+        <v>418</v>
+      </c>
+      <c r="B977" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="C977" s="5" t="s">
+        <v>420</v>
+      </c>
+      <c r="D977" s="5">
+        <v>28.4</v>
+      </c>
+      <c r="E977" s="5">
+        <v>39</v>
+      </c>
+      <c r="F977" s="5">
+        <v>27</v>
+      </c>
+      <c r="G977" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="978" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A978" s="5" t="s">
+        <v>418</v>
+      </c>
+      <c r="B978" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="C978" s="5" t="s">
+        <v>420</v>
+      </c>
+      <c r="D978" s="5">
+        <v>27.9</v>
+      </c>
+      <c r="E978" s="5">
+        <v>40</v>
+      </c>
+      <c r="F978" s="5">
+        <v>27</v>
+      </c>
+      <c r="G978" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="979" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A979" s="5" t="s">
+        <v>418</v>
+      </c>
+      <c r="B979" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="C979" s="5" t="s">
+        <v>420</v>
+      </c>
+      <c r="D979" s="5">
+        <v>27.5</v>
+      </c>
+      <c r="E979" s="5">
+        <v>41</v>
+      </c>
+      <c r="F979" s="5">
+        <v>26</v>
+      </c>
+      <c r="G979" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>

</xml_diff>

<commit_message>
📊 체감온도 기록: 2026-09-19 09:38 KST
</commit_message>
<xml_diff>
--- a/data/체감온도기록_2026.xlsx
+++ b/data/체감온도기록_2026.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3934" uniqueCount="421">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3942" uniqueCount="422">
   <si>
     <t>성동자이리버뷰 체감온도 기록</t>
   </si>
@@ -1277,6 +1277,9 @@
   </si>
   <si>
     <t>20:49</t>
+  </si>
+  <si>
+    <t>2026-09-19</t>
   </si>
 </sst>
 </file>
@@ -1697,7 +1700,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G979"/>
+  <dimension ref="A1:G981"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
@@ -24211,6 +24214,52 @@
         <v>11</v>
       </c>
     </row>
+    <row r="980" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A980" s="5" t="s">
+        <v>421</v>
+      </c>
+      <c r="B980" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="C980" s="5" t="s">
+        <v>398</v>
+      </c>
+      <c r="D980" s="5">
+        <v>21.2</v>
+      </c>
+      <c r="E980" s="5">
+        <v>60</v>
+      </c>
+      <c r="F980" s="5">
+        <v>22</v>
+      </c>
+      <c r="G980" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="981" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A981" s="5" t="s">
+        <v>421</v>
+      </c>
+      <c r="B981" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="C981" s="5" t="s">
+        <v>398</v>
+      </c>
+      <c r="D981" s="5">
+        <v>22.2</v>
+      </c>
+      <c r="E981" s="5">
+        <v>59</v>
+      </c>
+      <c r="F981" s="5">
+        <v>23</v>
+      </c>
+      <c r="G981" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>

</xml_diff>

<commit_message>
📊 체감온도 기록: 2026-09-20 09:23 KST
</commit_message>
<xml_diff>
--- a/data/체감온도기록_2026.xlsx
+++ b/data/체감온도기록_2026.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3942" uniqueCount="422">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3950" uniqueCount="423">
   <si>
     <t>성동자이리버뷰 체감온도 기록</t>
   </si>
@@ -1280,6 +1280,9 @@
   </si>
   <si>
     <t>2026-09-19</t>
+  </si>
+  <si>
+    <t>2026-09-20</t>
   </si>
 </sst>
 </file>
@@ -1700,7 +1703,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G981"/>
+  <dimension ref="A1:G983"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
@@ -24260,6 +24263,52 @@
         <v>11</v>
       </c>
     </row>
+    <row r="982" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A982" s="5" t="s">
+        <v>422</v>
+      </c>
+      <c r="B982" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="C982" s="5" t="s">
+        <v>380</v>
+      </c>
+      <c r="D982" s="5">
+        <v>19.5</v>
+      </c>
+      <c r="E982" s="5">
+        <v>69</v>
+      </c>
+      <c r="F982" s="5">
+        <v>21</v>
+      </c>
+      <c r="G982" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="983" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A983" s="5" t="s">
+        <v>422</v>
+      </c>
+      <c r="B983" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="C983" s="5" t="s">
+        <v>380</v>
+      </c>
+      <c r="D983" s="5">
+        <v>21.3</v>
+      </c>
+      <c r="E983" s="5">
+        <v>62</v>
+      </c>
+      <c r="F983" s="5">
+        <v>22</v>
+      </c>
+      <c r="G983" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>

</xml_diff>

<commit_message>
📊 체감온도 기록: 2026-09-20 14:24 KST
</commit_message>
<xml_diff>
--- a/data/체감온도기록_2026.xlsx
+++ b/data/체감온도기록_2026.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3950" uniqueCount="423">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3970" uniqueCount="424">
   <si>
     <t>성동자이리버뷰 체감온도 기록</t>
   </si>
@@ -1283,6 +1283,9 @@
   </si>
   <si>
     <t>2026-09-20</t>
+  </si>
+  <si>
+    <t>14:24</t>
   </si>
 </sst>
 </file>
@@ -1703,7 +1706,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G983"/>
+  <dimension ref="A1:G988"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
@@ -24309,6 +24312,121 @@
         <v>11</v>
       </c>
     </row>
+    <row r="984" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A984" s="5" t="s">
+        <v>422</v>
+      </c>
+      <c r="B984" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="C984" s="5" t="s">
+        <v>423</v>
+      </c>
+      <c r="D984" s="5">
+        <v>22.5</v>
+      </c>
+      <c r="E984" s="5">
+        <v>58</v>
+      </c>
+      <c r="F984" s="5">
+        <v>23</v>
+      </c>
+      <c r="G984" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="985" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A985" s="5" t="s">
+        <v>422</v>
+      </c>
+      <c r="B985" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C985" s="5" t="s">
+        <v>423</v>
+      </c>
+      <c r="D985" s="5">
+        <v>24.3</v>
+      </c>
+      <c r="E985" s="5">
+        <v>51</v>
+      </c>
+      <c r="F985" s="5">
+        <v>24</v>
+      </c>
+      <c r="G985" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="986" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A986" s="5" t="s">
+        <v>422</v>
+      </c>
+      <c r="B986" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="C986" s="5" t="s">
+        <v>423</v>
+      </c>
+      <c r="D986" s="5">
+        <v>25.3</v>
+      </c>
+      <c r="E986" s="5">
+        <v>45</v>
+      </c>
+      <c r="F986" s="5">
+        <v>25</v>
+      </c>
+      <c r="G986" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="987" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A987" s="5" t="s">
+        <v>422</v>
+      </c>
+      <c r="B987" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="C987" s="5" t="s">
+        <v>423</v>
+      </c>
+      <c r="D987" s="5">
+        <v>27.5</v>
+      </c>
+      <c r="E987" s="5">
+        <v>43</v>
+      </c>
+      <c r="F987" s="5">
+        <v>26</v>
+      </c>
+      <c r="G987" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="988" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A988" s="5" t="s">
+        <v>422</v>
+      </c>
+      <c r="B988" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="C988" s="5" t="s">
+        <v>423</v>
+      </c>
+      <c r="D988" s="5">
+        <v>27.6</v>
+      </c>
+      <c r="E988" s="5">
+        <v>40</v>
+      </c>
+      <c r="F988" s="5">
+        <v>26</v>
+      </c>
+      <c r="G988" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>

</xml_diff>

<commit_message>
📊 체감온도 기록: 2026-09-21 09:29 KST
</commit_message>
<xml_diff>
--- a/data/체감온도기록_2026.xlsx
+++ b/data/체감온도기록_2026.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3970" uniqueCount="424">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3978" uniqueCount="426">
   <si>
     <t>성동자이리버뷰 체감온도 기록</t>
   </si>
@@ -1286,6 +1286,12 @@
   </si>
   <si>
     <t>14:24</t>
+  </si>
+  <si>
+    <t>2026-09-21</t>
+  </si>
+  <si>
+    <t>09:29</t>
   </si>
 </sst>
 </file>
@@ -1706,7 +1712,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G988"/>
+  <dimension ref="A1:G990"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
@@ -24427,6 +24433,52 @@
         <v>11</v>
       </c>
     </row>
+    <row r="989" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A989" s="5" t="s">
+        <v>424</v>
+      </c>
+      <c r="B989" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="C989" s="5" t="s">
+        <v>425</v>
+      </c>
+      <c r="D989" s="5">
+        <v>19.1</v>
+      </c>
+      <c r="E989" s="5">
+        <v>73</v>
+      </c>
+      <c r="F989" s="5">
+        <v>21</v>
+      </c>
+      <c r="G989" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="990" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A990" s="5" t="s">
+        <v>424</v>
+      </c>
+      <c r="B990" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="C990" s="5" t="s">
+        <v>425</v>
+      </c>
+      <c r="D990" s="5">
+        <v>21</v>
+      </c>
+      <c r="E990" s="5">
+        <v>65</v>
+      </c>
+      <c r="F990" s="5">
+        <v>22</v>
+      </c>
+      <c r="G990" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>

</xml_diff>

<commit_message>
📊 체감온도 기록: 2026-09-21 14:29 KST
</commit_message>
<xml_diff>
--- a/data/체감온도기록_2026.xlsx
+++ b/data/체감온도기록_2026.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3978" uniqueCount="426">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3998" uniqueCount="426">
   <si>
     <t>성동자이리버뷰 체감온도 기록</t>
   </si>
@@ -1712,7 +1712,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G990"/>
+  <dimension ref="A1:G995"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
@@ -24479,6 +24479,121 @@
         <v>11</v>
       </c>
     </row>
+    <row r="991" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A991" s="5" t="s">
+        <v>424</v>
+      </c>
+      <c r="B991" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="C991" s="5" t="s">
+        <v>93</v>
+      </c>
+      <c r="D991" s="5">
+        <v>22.7</v>
+      </c>
+      <c r="E991" s="5">
+        <v>55</v>
+      </c>
+      <c r="F991" s="5">
+        <v>23</v>
+      </c>
+      <c r="G991" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="992" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A992" s="5" t="s">
+        <v>424</v>
+      </c>
+      <c r="B992" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C992" s="5" t="s">
+        <v>93</v>
+      </c>
+      <c r="D992" s="5">
+        <v>24.6</v>
+      </c>
+      <c r="E992" s="5">
+        <v>43</v>
+      </c>
+      <c r="F992" s="5">
+        <v>24</v>
+      </c>
+      <c r="G992" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="993" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A993" s="5" t="s">
+        <v>424</v>
+      </c>
+      <c r="B993" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="C993" s="5" t="s">
+        <v>93</v>
+      </c>
+      <c r="D993" s="5">
+        <v>26.1</v>
+      </c>
+      <c r="E993" s="5">
+        <v>36</v>
+      </c>
+      <c r="F993" s="5">
+        <v>24</v>
+      </c>
+      <c r="G993" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="994" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A994" s="5" t="s">
+        <v>424</v>
+      </c>
+      <c r="B994" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="C994" s="5" t="s">
+        <v>93</v>
+      </c>
+      <c r="D994" s="5">
+        <v>26.2</v>
+      </c>
+      <c r="E994" s="5">
+        <v>30</v>
+      </c>
+      <c r="F994" s="5">
+        <v>24</v>
+      </c>
+      <c r="G994" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="995" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A995" s="5" t="s">
+        <v>424</v>
+      </c>
+      <c r="B995" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="C995" s="5" t="s">
+        <v>93</v>
+      </c>
+      <c r="D995" s="5">
+        <v>28.9</v>
+      </c>
+      <c r="E995" s="5">
+        <v>24</v>
+      </c>
+      <c r="F995" s="5">
+        <v>26</v>
+      </c>
+      <c r="G995" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>

</xml_diff>

<commit_message>
📊 체감온도 기록: 2026-09-21 20:06 KST
</commit_message>
<xml_diff>
--- a/data/체감온도기록_2026.xlsx
+++ b/data/체감온도기록_2026.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3998" uniqueCount="426">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4014" uniqueCount="426">
   <si>
     <t>성동자이리버뷰 체감온도 기록</t>
   </si>
@@ -1712,7 +1712,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G995"/>
+  <dimension ref="A1:G999"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
@@ -24594,6 +24594,98 @@
         <v>11</v>
       </c>
     </row>
+    <row r="996" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A996" s="5" t="s">
+        <v>424</v>
+      </c>
+      <c r="B996" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="C996" s="5" t="s">
+        <v>273</v>
+      </c>
+      <c r="D996" s="5">
+        <v>29.1</v>
+      </c>
+      <c r="E996" s="5">
+        <v>25</v>
+      </c>
+      <c r="F996" s="5">
+        <v>26</v>
+      </c>
+      <c r="G996" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="997" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A997" s="5" t="s">
+        <v>424</v>
+      </c>
+      <c r="B997" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="C997" s="5" t="s">
+        <v>273</v>
+      </c>
+      <c r="D997" s="5">
+        <v>29.7</v>
+      </c>
+      <c r="E997" s="5">
+        <v>20</v>
+      </c>
+      <c r="F997" s="5">
+        <v>26</v>
+      </c>
+      <c r="G997" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="998" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A998" s="5" t="s">
+        <v>424</v>
+      </c>
+      <c r="B998" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="C998" s="5" t="s">
+        <v>273</v>
+      </c>
+      <c r="D998" s="5">
+        <v>29.4</v>
+      </c>
+      <c r="E998" s="5">
+        <v>21</v>
+      </c>
+      <c r="F998" s="5">
+        <v>26</v>
+      </c>
+      <c r="G998" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="999" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A999" s="5" t="s">
+        <v>424</v>
+      </c>
+      <c r="B999" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="C999" s="5" t="s">
+        <v>273</v>
+      </c>
+      <c r="D999" s="5">
+        <v>29.5</v>
+      </c>
+      <c r="E999" s="5">
+        <v>21</v>
+      </c>
+      <c r="F999" s="5">
+        <v>26</v>
+      </c>
+      <c r="G999" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>

</xml_diff>

<commit_message>
📊 체감온도 기록: 2026-09-22 10:10 KST
</commit_message>
<xml_diff>
--- a/data/체감온도기록_2026.xlsx
+++ b/data/체감온도기록_2026.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4014" uniqueCount="426">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4026" uniqueCount="427">
   <si>
     <t>성동자이리버뷰 체감온도 기록</t>
   </si>
@@ -1292,6 +1292,9 @@
   </si>
   <si>
     <t>09:29</t>
+  </si>
+  <si>
+    <t>2026-09-22</t>
   </si>
 </sst>
 </file>
@@ -1712,7 +1715,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G999"/>
+  <dimension ref="A1:G1002"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
@@ -24686,6 +24689,75 @@
         <v>11</v>
       </c>
     </row>
+    <row r="1000" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1000" s="5" t="s">
+        <v>426</v>
+      </c>
+      <c r="B1000" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1000" s="5" t="s">
+        <v>160</v>
+      </c>
+      <c r="D1000" s="5">
+        <v>19.9</v>
+      </c>
+      <c r="E1000" s="5">
+        <v>58</v>
+      </c>
+      <c r="F1000" s="5">
+        <v>20</v>
+      </c>
+      <c r="G1000" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1001" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1001" s="5" t="s">
+        <v>426</v>
+      </c>
+      <c r="B1001" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="C1001" s="5" t="s">
+        <v>160</v>
+      </c>
+      <c r="D1001" s="5">
+        <v>21.1</v>
+      </c>
+      <c r="E1001" s="5">
+        <v>57</v>
+      </c>
+      <c r="F1001" s="5">
+        <v>21</v>
+      </c>
+      <c r="G1001" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1002" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1002" s="5" t="s">
+        <v>426</v>
+      </c>
+      <c r="B1002" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="C1002" s="5" t="s">
+        <v>160</v>
+      </c>
+      <c r="D1002" s="5">
+        <v>22.9</v>
+      </c>
+      <c r="E1002" s="5">
+        <v>54</v>
+      </c>
+      <c r="F1002" s="5">
+        <v>23</v>
+      </c>
+      <c r="G1002" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>

</xml_diff>

<commit_message>
📊 체감온도 기록: 2026-09-22 15:47 KST
</commit_message>
<xml_diff>
--- a/data/체감온도기록_2026.xlsx
+++ b/data/체감온도기록_2026.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4026" uniqueCount="427">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4050" uniqueCount="428">
   <si>
     <t>성동자이리버뷰 체감온도 기록</t>
   </si>
@@ -1295,6 +1295,9 @@
   </si>
   <si>
     <t>2026-09-22</t>
+  </si>
+  <si>
+    <t>15:47</t>
   </si>
 </sst>
 </file>
@@ -1715,7 +1718,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G1002"/>
+  <dimension ref="A1:G1008"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
@@ -24758,6 +24761,144 @@
         <v>11</v>
       </c>
     </row>
+    <row r="1003" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1003" s="5" t="s">
+        <v>426</v>
+      </c>
+      <c r="B1003" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1003" s="5" t="s">
+        <v>427</v>
+      </c>
+      <c r="D1003" s="5">
+        <v>24.1</v>
+      </c>
+      <c r="E1003" s="5">
+        <v>49</v>
+      </c>
+      <c r="F1003" s="5">
+        <v>24</v>
+      </c>
+      <c r="G1003" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1004" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1004" s="5" t="s">
+        <v>426</v>
+      </c>
+      <c r="B1004" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="C1004" s="5" t="s">
+        <v>427</v>
+      </c>
+      <c r="D1004" s="5">
+        <v>25.6</v>
+      </c>
+      <c r="E1004" s="5">
+        <v>46</v>
+      </c>
+      <c r="F1004" s="5">
+        <v>25</v>
+      </c>
+      <c r="G1004" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1005" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1005" s="5" t="s">
+        <v>426</v>
+      </c>
+      <c r="B1005" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="C1005" s="5" t="s">
+        <v>427</v>
+      </c>
+      <c r="D1005" s="5">
+        <v>26.9</v>
+      </c>
+      <c r="E1005" s="5">
+        <v>44</v>
+      </c>
+      <c r="F1005" s="5">
+        <v>26</v>
+      </c>
+      <c r="G1005" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1006" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1006" s="5" t="s">
+        <v>426</v>
+      </c>
+      <c r="B1006" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1006" s="5" t="s">
+        <v>427</v>
+      </c>
+      <c r="D1006" s="5">
+        <v>27.6</v>
+      </c>
+      <c r="E1006" s="5">
+        <v>41</v>
+      </c>
+      <c r="F1006" s="5">
+        <v>26</v>
+      </c>
+      <c r="G1006" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1007" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1007" s="5" t="s">
+        <v>426</v>
+      </c>
+      <c r="B1007" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="C1007" s="5" t="s">
+        <v>427</v>
+      </c>
+      <c r="D1007" s="5">
+        <v>28.9</v>
+      </c>
+      <c r="E1007" s="5">
+        <v>35</v>
+      </c>
+      <c r="F1007" s="5">
+        <v>27</v>
+      </c>
+      <c r="G1007" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1008" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1008" s="5" t="s">
+        <v>426</v>
+      </c>
+      <c r="B1008" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="C1008" s="5" t="s">
+        <v>427</v>
+      </c>
+      <c r="D1008" s="5">
+        <v>29.8</v>
+      </c>
+      <c r="E1008" s="5">
+        <v>33</v>
+      </c>
+      <c r="F1008" s="5">
+        <v>28</v>
+      </c>
+      <c r="G1008" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>

</xml_diff>

<commit_message>
📊 체감온도 기록: 2026-09-22 21:49 KST
</commit_message>
<xml_diff>
--- a/data/체감온도기록_2026.xlsx
+++ b/data/체감온도기록_2026.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4050" uniqueCount="428">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4058" uniqueCount="428">
   <si>
     <t>성동자이리버뷰 체감온도 기록</t>
   </si>
@@ -1718,7 +1718,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G1008"/>
+  <dimension ref="A1:G1010"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
@@ -24899,6 +24899,52 @@
         <v>11</v>
       </c>
     </row>
+    <row r="1009" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1009" s="5" t="s">
+        <v>426</v>
+      </c>
+      <c r="B1009" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1009" s="5" t="s">
+        <v>413</v>
+      </c>
+      <c r="D1009" s="5">
+        <v>29.1</v>
+      </c>
+      <c r="E1009" s="5">
+        <v>34</v>
+      </c>
+      <c r="F1009" s="5">
+        <v>27</v>
+      </c>
+      <c r="G1009" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1010" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1010" s="5" t="s">
+        <v>426</v>
+      </c>
+      <c r="B1010" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="C1010" s="5" t="s">
+        <v>413</v>
+      </c>
+      <c r="D1010" s="5">
+        <v>28.5</v>
+      </c>
+      <c r="E1010" s="5">
+        <v>36</v>
+      </c>
+      <c r="F1010" s="5">
+        <v>27</v>
+      </c>
+      <c r="G1010" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>

</xml_diff>

<commit_message>
📊 체감온도 기록: 2026-09-23 09:56 KST
</commit_message>
<xml_diff>
--- a/data/체감온도기록_2026.xlsx
+++ b/data/체감온도기록_2026.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4058" uniqueCount="428">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4070" uniqueCount="430">
   <si>
     <t>성동자이리버뷰 체감온도 기록</t>
   </si>
@@ -1298,6 +1298,12 @@
   </si>
   <si>
     <t>15:47</t>
+  </si>
+  <si>
+    <t>2026-09-23</t>
+  </si>
+  <si>
+    <t>09:56</t>
   </si>
 </sst>
 </file>
@@ -1718,7 +1724,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G1010"/>
+  <dimension ref="A1:G1013"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
@@ -24945,6 +24951,75 @@
         <v>11</v>
       </c>
     </row>
+    <row r="1011" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1011" s="5" t="s">
+        <v>428</v>
+      </c>
+      <c r="B1011" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1011" s="5" t="s">
+        <v>429</v>
+      </c>
+      <c r="D1011" s="5">
+        <v>20.1</v>
+      </c>
+      <c r="E1011" s="5">
+        <v>74</v>
+      </c>
+      <c r="F1011" s="5">
+        <v>22</v>
+      </c>
+      <c r="G1011" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1012" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1012" s="5" t="s">
+        <v>428</v>
+      </c>
+      <c r="B1012" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="C1012" s="5" t="s">
+        <v>429</v>
+      </c>
+      <c r="D1012" s="5">
+        <v>22.3</v>
+      </c>
+      <c r="E1012" s="5">
+        <v>65</v>
+      </c>
+      <c r="F1012" s="5">
+        <v>23</v>
+      </c>
+      <c r="G1012" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1013" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1013" s="5" t="s">
+        <v>428</v>
+      </c>
+      <c r="B1013" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="C1013" s="5" t="s">
+        <v>429</v>
+      </c>
+      <c r="D1013" s="5">
+        <v>23.8</v>
+      </c>
+      <c r="E1013" s="5">
+        <v>61</v>
+      </c>
+      <c r="F1013" s="5">
+        <v>24</v>
+      </c>
+      <c r="G1013" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>

</xml_diff>

<commit_message>
📊 체감온도 기록: 2026-09-23 15:39 KST
</commit_message>
<xml_diff>
--- a/data/체감온도기록_2026.xlsx
+++ b/data/체감온도기록_2026.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4070" uniqueCount="430">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4090" uniqueCount="430">
   <si>
     <t>성동자이리버뷰 체감온도 기록</t>
   </si>
@@ -1724,7 +1724,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G1013"/>
+  <dimension ref="A1:G1018"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
@@ -25020,6 +25020,121 @@
         <v>11</v>
       </c>
     </row>
+    <row r="1014" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1014" s="5" t="s">
+        <v>428</v>
+      </c>
+      <c r="B1014" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1014" s="5" t="s">
+        <v>419</v>
+      </c>
+      <c r="D1014" s="5">
+        <v>24.6</v>
+      </c>
+      <c r="E1014" s="5">
+        <v>57</v>
+      </c>
+      <c r="F1014" s="5">
+        <v>25</v>
+      </c>
+      <c r="G1014" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1015" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1015" s="5" t="s">
+        <v>428</v>
+      </c>
+      <c r="B1015" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="C1015" s="5" t="s">
+        <v>419</v>
+      </c>
+      <c r="D1015" s="5">
+        <v>25.7</v>
+      </c>
+      <c r="E1015" s="5">
+        <v>53</v>
+      </c>
+      <c r="F1015" s="5">
+        <v>26</v>
+      </c>
+      <c r="G1015" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1016" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1016" s="5" t="s">
+        <v>428</v>
+      </c>
+      <c r="B1016" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="C1016" s="5" t="s">
+        <v>419</v>
+      </c>
+      <c r="D1016" s="5">
+        <v>26.6</v>
+      </c>
+      <c r="E1016" s="5">
+        <v>49</v>
+      </c>
+      <c r="F1016" s="5">
+        <v>26</v>
+      </c>
+      <c r="G1016" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1017" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1017" s="5" t="s">
+        <v>428</v>
+      </c>
+      <c r="B1017" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1017" s="5" t="s">
+        <v>419</v>
+      </c>
+      <c r="D1017" s="5">
+        <v>27</v>
+      </c>
+      <c r="E1017" s="5">
+        <v>48</v>
+      </c>
+      <c r="F1017" s="5">
+        <v>26</v>
+      </c>
+      <c r="G1017" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1018" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1018" s="5" t="s">
+        <v>428</v>
+      </c>
+      <c r="B1018" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="C1018" s="5" t="s">
+        <v>419</v>
+      </c>
+      <c r="D1018" s="5">
+        <v>28.2</v>
+      </c>
+      <c r="E1018" s="5">
+        <v>42</v>
+      </c>
+      <c r="F1018" s="5">
+        <v>27</v>
+      </c>
+      <c r="G1018" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>

</xml_diff>

<commit_message>
📊 체감온도 기록: 2026-09-23 21:10 KST
</commit_message>
<xml_diff>
--- a/data/체감온도기록_2026.xlsx
+++ b/data/체감온도기록_2026.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4090" uniqueCount="430">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4102" uniqueCount="431">
   <si>
     <t>성동자이리버뷰 체감온도 기록</t>
   </si>
@@ -1304,6 +1304,9 @@
   </si>
   <si>
     <t>09:56</t>
+  </si>
+  <si>
+    <t>21:10</t>
   </si>
 </sst>
 </file>
@@ -1724,7 +1727,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G1018"/>
+  <dimension ref="A1:G1021"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
@@ -25135,6 +25138,75 @@
         <v>11</v>
       </c>
     </row>
+    <row r="1019" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1019" s="5" t="s">
+        <v>428</v>
+      </c>
+      <c r="B1019" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="C1019" s="5" t="s">
+        <v>430</v>
+      </c>
+      <c r="D1019" s="5">
+        <v>28.5</v>
+      </c>
+      <c r="E1019" s="5">
+        <v>43</v>
+      </c>
+      <c r="F1019" s="5">
+        <v>27</v>
+      </c>
+      <c r="G1019" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1020" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1020" s="5" t="s">
+        <v>428</v>
+      </c>
+      <c r="B1020" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1020" s="5" t="s">
+        <v>430</v>
+      </c>
+      <c r="D1020" s="5">
+        <v>28.9</v>
+      </c>
+      <c r="E1020" s="5">
+        <v>40</v>
+      </c>
+      <c r="F1020" s="5">
+        <v>28</v>
+      </c>
+      <c r="G1020" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1021" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1021" s="5" t="s">
+        <v>428</v>
+      </c>
+      <c r="B1021" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="C1021" s="5" t="s">
+        <v>430</v>
+      </c>
+      <c r="D1021" s="5">
+        <v>27.8</v>
+      </c>
+      <c r="E1021" s="5">
+        <v>44</v>
+      </c>
+      <c r="F1021" s="5">
+        <v>27</v>
+      </c>
+      <c r="G1021" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>

</xml_diff>

<commit_message>
📊 체감온도 기록: 2026-09-24 21:18 KST
</commit_message>
<xml_diff>
--- a/data/체감온도기록_2026.xlsx
+++ b/data/체감온도기록_2026.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4102" uniqueCount="431">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4146" uniqueCount="433">
   <si>
     <t>성동자이리버뷰 체감온도 기록</t>
   </si>
@@ -1307,6 +1307,12 @@
   </si>
   <si>
     <t>21:10</t>
+  </si>
+  <si>
+    <t>2026-09-24</t>
+  </si>
+  <si>
+    <t>21:17</t>
   </si>
 </sst>
 </file>
@@ -1727,7 +1733,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G1021"/>
+  <dimension ref="A1:G1032"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
@@ -25207,6 +25213,259 @@
         <v>11</v>
       </c>
     </row>
+    <row r="1022" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1022" s="5" t="s">
+        <v>431</v>
+      </c>
+      <c r="B1022" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1022" s="5" t="s">
+        <v>432</v>
+      </c>
+      <c r="D1022" s="5">
+        <v>20.2</v>
+      </c>
+      <c r="E1022" s="5">
+        <v>84</v>
+      </c>
+      <c r="F1022" s="5">
+        <v>22</v>
+      </c>
+      <c r="G1022" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1023" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1023" s="5" t="s">
+        <v>431</v>
+      </c>
+      <c r="B1023" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="C1023" s="5" t="s">
+        <v>432</v>
+      </c>
+      <c r="D1023" s="5">
+        <v>21.7</v>
+      </c>
+      <c r="E1023" s="5">
+        <v>77</v>
+      </c>
+      <c r="F1023" s="5">
+        <v>23</v>
+      </c>
+      <c r="G1023" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1024" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1024" s="5" t="s">
+        <v>431</v>
+      </c>
+      <c r="B1024" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="C1024" s="5" t="s">
+        <v>432</v>
+      </c>
+      <c r="D1024" s="5">
+        <v>22.4</v>
+      </c>
+      <c r="E1024" s="5">
+        <v>75</v>
+      </c>
+      <c r="F1024" s="5">
+        <v>24</v>
+      </c>
+      <c r="G1024" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1025" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1025" s="5" t="s">
+        <v>431</v>
+      </c>
+      <c r="B1025" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1025" s="5" t="s">
+        <v>432</v>
+      </c>
+      <c r="D1025" s="5">
+        <v>24</v>
+      </c>
+      <c r="E1025" s="5">
+        <v>67</v>
+      </c>
+      <c r="F1025" s="5">
+        <v>25</v>
+      </c>
+      <c r="G1025" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1026" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1026" s="5" t="s">
+        <v>431</v>
+      </c>
+      <c r="B1026" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="C1026" s="5" t="s">
+        <v>432</v>
+      </c>
+      <c r="D1026" s="5">
+        <v>24.4</v>
+      </c>
+      <c r="E1026" s="5">
+        <v>62</v>
+      </c>
+      <c r="F1026" s="5">
+        <v>25</v>
+      </c>
+      <c r="G1026" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1027" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1027" s="5" t="s">
+        <v>431</v>
+      </c>
+      <c r="B1027" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="C1027" s="5" t="s">
+        <v>432</v>
+      </c>
+      <c r="D1027" s="5">
+        <v>25.6</v>
+      </c>
+      <c r="E1027" s="5">
+        <v>54</v>
+      </c>
+      <c r="F1027" s="5">
+        <v>26</v>
+      </c>
+      <c r="G1027" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1028" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1028" s="5" t="s">
+        <v>431</v>
+      </c>
+      <c r="B1028" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1028" s="5" t="s">
+        <v>432</v>
+      </c>
+      <c r="D1028" s="5">
+        <v>26.1</v>
+      </c>
+      <c r="E1028" s="5">
+        <v>51</v>
+      </c>
+      <c r="F1028" s="5">
+        <v>26</v>
+      </c>
+      <c r="G1028" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1029" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1029" s="5" t="s">
+        <v>431</v>
+      </c>
+      <c r="B1029" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="C1029" s="5" t="s">
+        <v>432</v>
+      </c>
+      <c r="D1029" s="5">
+        <v>26.5</v>
+      </c>
+      <c r="E1029" s="5">
+        <v>50</v>
+      </c>
+      <c r="F1029" s="5">
+        <v>26</v>
+      </c>
+      <c r="G1029" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1030" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1030" s="5" t="s">
+        <v>431</v>
+      </c>
+      <c r="B1030" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="C1030" s="5" t="s">
+        <v>432</v>
+      </c>
+      <c r="D1030" s="5">
+        <v>27.2</v>
+      </c>
+      <c r="E1030" s="5">
+        <v>48</v>
+      </c>
+      <c r="F1030" s="5">
+        <v>27</v>
+      </c>
+      <c r="G1030" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1031" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1031" s="5" t="s">
+        <v>431</v>
+      </c>
+      <c r="B1031" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1031" s="5" t="s">
+        <v>432</v>
+      </c>
+      <c r="D1031" s="5">
+        <v>26.7</v>
+      </c>
+      <c r="E1031" s="5">
+        <v>50</v>
+      </c>
+      <c r="F1031" s="5">
+        <v>26</v>
+      </c>
+      <c r="G1031" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1032" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1032" s="5" t="s">
+        <v>431</v>
+      </c>
+      <c r="B1032" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="C1032" s="5" t="s">
+        <v>432</v>
+      </c>
+      <c r="D1032" s="5">
+        <v>25.9</v>
+      </c>
+      <c r="E1032" s="5">
+        <v>54</v>
+      </c>
+      <c r="F1032" s="5">
+        <v>26</v>
+      </c>
+      <c r="G1032" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>

</xml_diff>

<commit_message>
📊 체감온도 기록: 2026-09-25 15:36 KST
</commit_message>
<xml_diff>
--- a/data/체감온도기록_2026.xlsx
+++ b/data/체감온도기록_2026.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4146" uniqueCount="433">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4180" uniqueCount="435">
   <si>
     <t>성동자이리버뷰 체감온도 기록</t>
   </si>
@@ -1313,6 +1313,12 @@
   </si>
   <si>
     <t>21:17</t>
+  </si>
+  <si>
+    <t>2026-09-25</t>
+  </si>
+  <si>
+    <t>15:36</t>
   </si>
 </sst>
 </file>
@@ -1733,7 +1739,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G1032"/>
+  <dimension ref="A1:G1040"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
@@ -25466,6 +25472,190 @@
         <v>11</v>
       </c>
     </row>
+    <row r="1033" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1033" s="5" t="s">
+        <v>433</v>
+      </c>
+      <c r="B1033" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1033" s="5" t="s">
+        <v>434</v>
+      </c>
+      <c r="D1033" s="5" t="s">
+        <v>106</v>
+      </c>
+      <c r="E1033" s="5" t="s">
+        <v>106</v>
+      </c>
+      <c r="F1033" s="5">
+        <v>22</v>
+      </c>
+      <c r="G1033" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1034" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1034" s="5" t="s">
+        <v>433</v>
+      </c>
+      <c r="B1034" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="C1034" s="5" t="s">
+        <v>434</v>
+      </c>
+      <c r="D1034" s="5">
+        <v>21.1</v>
+      </c>
+      <c r="E1034" s="5">
+        <v>71</v>
+      </c>
+      <c r="F1034" s="5">
+        <v>22</v>
+      </c>
+      <c r="G1034" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1035" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1035" s="5" t="s">
+        <v>433</v>
+      </c>
+      <c r="B1035" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="C1035" s="5" t="s">
+        <v>434</v>
+      </c>
+      <c r="D1035" s="5">
+        <v>22</v>
+      </c>
+      <c r="E1035" s="5">
+        <v>68</v>
+      </c>
+      <c r="F1035" s="5">
+        <v>23</v>
+      </c>
+      <c r="G1035" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1036" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1036" s="5" t="s">
+        <v>433</v>
+      </c>
+      <c r="B1036" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1036" s="5" t="s">
+        <v>434</v>
+      </c>
+      <c r="D1036" s="5">
+        <v>23</v>
+      </c>
+      <c r="E1036" s="5">
+        <v>65</v>
+      </c>
+      <c r="F1036" s="5">
+        <v>24</v>
+      </c>
+      <c r="G1036" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1037" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1037" s="5" t="s">
+        <v>433</v>
+      </c>
+      <c r="B1037" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="C1037" s="5" t="s">
+        <v>434</v>
+      </c>
+      <c r="D1037" s="5">
+        <v>23.6</v>
+      </c>
+      <c r="E1037" s="5">
+        <v>62</v>
+      </c>
+      <c r="F1037" s="5">
+        <v>24</v>
+      </c>
+      <c r="G1037" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1038" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1038" s="5" t="s">
+        <v>433</v>
+      </c>
+      <c r="B1038" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="C1038" s="5" t="s">
+        <v>434</v>
+      </c>
+      <c r="D1038" s="5">
+        <v>23.7</v>
+      </c>
+      <c r="E1038" s="5">
+        <v>62</v>
+      </c>
+      <c r="F1038" s="5">
+        <v>24</v>
+      </c>
+      <c r="G1038" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1039" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1039" s="5" t="s">
+        <v>433</v>
+      </c>
+      <c r="B1039" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1039" s="5" t="s">
+        <v>434</v>
+      </c>
+      <c r="D1039" s="5">
+        <v>23.6</v>
+      </c>
+      <c r="E1039" s="5">
+        <v>64</v>
+      </c>
+      <c r="F1039" s="5">
+        <v>24</v>
+      </c>
+      <c r="G1039" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1040" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1040" s="5" t="s">
+        <v>433</v>
+      </c>
+      <c r="B1040" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="C1040" s="5" t="s">
+        <v>434</v>
+      </c>
+      <c r="D1040" s="5">
+        <v>22.4</v>
+      </c>
+      <c r="E1040" s="5">
+        <v>74</v>
+      </c>
+      <c r="F1040" s="5">
+        <v>24</v>
+      </c>
+      <c r="G1040" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>

</xml_diff>

<commit_message>
📊 체감온도 기록: 2026-09-25 21:14 KST
</commit_message>
<xml_diff>
--- a/data/체감온도기록_2026.xlsx
+++ b/data/체감온도기록_2026.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4180" uniqueCount="435">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4192" uniqueCount="436">
   <si>
     <t>성동자이리버뷰 체감온도 기록</t>
   </si>
@@ -1319,6 +1319,9 @@
   </si>
   <si>
     <t>15:36</t>
+  </si>
+  <si>
+    <t>21:14</t>
   </si>
 </sst>
 </file>
@@ -1739,7 +1742,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G1040"/>
+  <dimension ref="A1:G1043"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
@@ -25656,6 +25659,75 @@
         <v>11</v>
       </c>
     </row>
+    <row r="1041" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1041" s="5" t="s">
+        <v>433</v>
+      </c>
+      <c r="B1041" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="C1041" s="5" t="s">
+        <v>435</v>
+      </c>
+      <c r="D1041" s="5">
+        <v>20.2</v>
+      </c>
+      <c r="E1041" s="5">
+        <v>87</v>
+      </c>
+      <c r="F1041" s="5">
+        <v>23</v>
+      </c>
+      <c r="G1041" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1042" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1042" s="5" t="s">
+        <v>433</v>
+      </c>
+      <c r="B1042" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1042" s="5" t="s">
+        <v>435</v>
+      </c>
+      <c r="D1042" s="5">
+        <v>20.4</v>
+      </c>
+      <c r="E1042" s="5">
+        <v>89</v>
+      </c>
+      <c r="F1042" s="5">
+        <v>23</v>
+      </c>
+      <c r="G1042" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1043" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1043" s="5" t="s">
+        <v>433</v>
+      </c>
+      <c r="B1043" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="C1043" s="5" t="s">
+        <v>435</v>
+      </c>
+      <c r="D1043" s="5">
+        <v>19.6</v>
+      </c>
+      <c r="E1043" s="5">
+        <v>88</v>
+      </c>
+      <c r="F1043" s="5">
+        <v>22</v>
+      </c>
+      <c r="G1043" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>

</xml_diff>

<commit_message>
📊 체감온도 기록: 2026-09-26 09:52 KST
</commit_message>
<xml_diff>
--- a/data/체감온도기록_2026.xlsx
+++ b/data/체감온도기록_2026.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4192" uniqueCount="436">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4204" uniqueCount="437">
   <si>
     <t>성동자이리버뷰 체감온도 기록</t>
   </si>
@@ -1322,6 +1322,9 @@
   </si>
   <si>
     <t>21:14</t>
+  </si>
+  <si>
+    <t>2026-09-26</t>
   </si>
 </sst>
 </file>
@@ -1742,7 +1745,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G1043"/>
+  <dimension ref="A1:G1046"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
@@ -25728,6 +25731,75 @@
         <v>11</v>
       </c>
     </row>
+    <row r="1044" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1044" s="5" t="s">
+        <v>436</v>
+      </c>
+      <c r="B1044" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1044" s="5" t="s">
+        <v>415</v>
+      </c>
+      <c r="D1044" s="5">
+        <v>18.8</v>
+      </c>
+      <c r="E1044" s="5">
+        <v>81</v>
+      </c>
+      <c r="F1044" s="5">
+        <v>21</v>
+      </c>
+      <c r="G1044" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1045" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1045" s="5" t="s">
+        <v>436</v>
+      </c>
+      <c r="B1045" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="C1045" s="5" t="s">
+        <v>415</v>
+      </c>
+      <c r="D1045" s="5">
+        <v>19.1</v>
+      </c>
+      <c r="E1045" s="5">
+        <v>80</v>
+      </c>
+      <c r="F1045" s="5">
+        <v>21</v>
+      </c>
+      <c r="G1045" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1046" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1046" s="5" t="s">
+        <v>436</v>
+      </c>
+      <c r="B1046" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="C1046" s="5" t="s">
+        <v>415</v>
+      </c>
+      <c r="D1046" s="5">
+        <v>21</v>
+      </c>
+      <c r="E1046" s="5">
+        <v>69</v>
+      </c>
+      <c r="F1046" s="5">
+        <v>22</v>
+      </c>
+      <c r="G1046" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>

</xml_diff>

<commit_message>
📊 체감온도 기록: 2026-09-26 15:36 KST
</commit_message>
<xml_diff>
--- a/data/체감온도기록_2026.xlsx
+++ b/data/체감온도기록_2026.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4204" uniqueCount="437">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4224" uniqueCount="437">
   <si>
     <t>성동자이리버뷰 체감온도 기록</t>
   </si>
@@ -1745,7 +1745,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G1046"/>
+  <dimension ref="A1:G1051"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
@@ -25800,6 +25800,121 @@
         <v>11</v>
       </c>
     </row>
+    <row r="1047" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1047" s="5" t="s">
+        <v>436</v>
+      </c>
+      <c r="B1047" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1047" s="5" t="s">
+        <v>434</v>
+      </c>
+      <c r="D1047" s="5">
+        <v>22.1</v>
+      </c>
+      <c r="E1047" s="5">
+        <v>64</v>
+      </c>
+      <c r="F1047" s="5">
+        <v>23</v>
+      </c>
+      <c r="G1047" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1048" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1048" s="5" t="s">
+        <v>436</v>
+      </c>
+      <c r="B1048" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="C1048" s="5" t="s">
+        <v>434</v>
+      </c>
+      <c r="D1048" s="5">
+        <v>23.9</v>
+      </c>
+      <c r="E1048" s="5">
+        <v>60</v>
+      </c>
+      <c r="F1048" s="5">
+        <v>24</v>
+      </c>
+      <c r="G1048" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1049" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1049" s="5" t="s">
+        <v>436</v>
+      </c>
+      <c r="B1049" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="C1049" s="5" t="s">
+        <v>434</v>
+      </c>
+      <c r="D1049" s="5">
+        <v>25</v>
+      </c>
+      <c r="E1049" s="5">
+        <v>52</v>
+      </c>
+      <c r="F1049" s="5">
+        <v>25</v>
+      </c>
+      <c r="G1049" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1050" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1050" s="5" t="s">
+        <v>436</v>
+      </c>
+      <c r="B1050" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1050" s="5" t="s">
+        <v>434</v>
+      </c>
+      <c r="D1050" s="5">
+        <v>25.3</v>
+      </c>
+      <c r="E1050" s="5">
+        <v>47</v>
+      </c>
+      <c r="F1050" s="5">
+        <v>25</v>
+      </c>
+      <c r="G1050" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1051" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1051" s="5" t="s">
+        <v>436</v>
+      </c>
+      <c r="B1051" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="C1051" s="5" t="s">
+        <v>434</v>
+      </c>
+      <c r="D1051" s="5">
+        <v>26.6</v>
+      </c>
+      <c r="E1051" s="5">
+        <v>46</v>
+      </c>
+      <c r="F1051" s="5">
+        <v>26</v>
+      </c>
+      <c r="G1051" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>

</xml_diff>

<commit_message>
📊 체감온도 기록: 2026-09-26 20:47 KST
</commit_message>
<xml_diff>
--- a/data/체감온도기록_2026.xlsx
+++ b/data/체감온도기록_2026.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4224" uniqueCount="437">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4236" uniqueCount="438">
   <si>
     <t>성동자이리버뷰 체감온도 기록</t>
   </si>
@@ -1325,6 +1325,9 @@
   </si>
   <si>
     <t>2026-09-26</t>
+  </si>
+  <si>
+    <t>20:46</t>
   </si>
 </sst>
 </file>
@@ -1745,7 +1748,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G1051"/>
+  <dimension ref="A1:G1054"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
@@ -25915,6 +25918,75 @@
         <v>11</v>
       </c>
     </row>
+    <row r="1052" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1052" s="5" t="s">
+        <v>436</v>
+      </c>
+      <c r="B1052" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="C1052" s="5" t="s">
+        <v>437</v>
+      </c>
+      <c r="D1052" s="5">
+        <v>26.6</v>
+      </c>
+      <c r="E1052" s="5">
+        <v>45</v>
+      </c>
+      <c r="F1052" s="5">
+        <v>26</v>
+      </c>
+      <c r="G1052" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1053" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1053" s="5" t="s">
+        <v>436</v>
+      </c>
+      <c r="B1053" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1053" s="5" t="s">
+        <v>437</v>
+      </c>
+      <c r="D1053" s="5">
+        <v>26</v>
+      </c>
+      <c r="E1053" s="5">
+        <v>47</v>
+      </c>
+      <c r="F1053" s="5">
+        <v>25</v>
+      </c>
+      <c r="G1053" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1054" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1054" s="5" t="s">
+        <v>436</v>
+      </c>
+      <c r="B1054" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="C1054" s="5" t="s">
+        <v>437</v>
+      </c>
+      <c r="D1054" s="5">
+        <v>25.9</v>
+      </c>
+      <c r="E1054" s="5">
+        <v>48</v>
+      </c>
+      <c r="F1054" s="5">
+        <v>25</v>
+      </c>
+      <c r="G1054" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>

</xml_diff>

<commit_message>
📊 체감온도 기록: 2026-09-27 09:52 KST
</commit_message>
<xml_diff>
--- a/data/체감온도기록_2026.xlsx
+++ b/data/체감온도기록_2026.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4236" uniqueCount="438">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4248" uniqueCount="439">
   <si>
     <t>성동자이리버뷰 체감온도 기록</t>
   </si>
@@ -1328,6 +1328,9 @@
   </si>
   <si>
     <t>20:46</t>
+  </si>
+  <si>
+    <t>2026-09-27</t>
   </si>
 </sst>
 </file>
@@ -1748,7 +1751,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G1054"/>
+  <dimension ref="A1:G1057"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
@@ -25987,6 +25990,75 @@
         <v>11</v>
       </c>
     </row>
+    <row r="1055" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1055" s="5" t="s">
+        <v>438</v>
+      </c>
+      <c r="B1055" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1055" s="5" t="s">
+        <v>415</v>
+      </c>
+      <c r="D1055" s="5">
+        <v>18.1</v>
+      </c>
+      <c r="E1055" s="5">
+        <v>84</v>
+      </c>
+      <c r="F1055" s="5">
+        <v>20</v>
+      </c>
+      <c r="G1055" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1056" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1056" s="5" t="s">
+        <v>438</v>
+      </c>
+      <c r="B1056" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="C1056" s="5" t="s">
+        <v>415</v>
+      </c>
+      <c r="D1056" s="5">
+        <v>19.3</v>
+      </c>
+      <c r="E1056" s="5">
+        <v>79</v>
+      </c>
+      <c r="F1056" s="5">
+        <v>21</v>
+      </c>
+      <c r="G1056" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1057" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1057" s="5" t="s">
+        <v>438</v>
+      </c>
+      <c r="B1057" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="C1057" s="5" t="s">
+        <v>415</v>
+      </c>
+      <c r="D1057" s="5">
+        <v>21</v>
+      </c>
+      <c r="E1057" s="5">
+        <v>73</v>
+      </c>
+      <c r="F1057" s="5">
+        <v>22</v>
+      </c>
+      <c r="G1057" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>

</xml_diff>

<commit_message>
📊 체감온도 기록: 2026-09-27 22:17 KST
</commit_message>
<xml_diff>
--- a/data/체감온도기록_2026.xlsx
+++ b/data/체감온도기록_2026.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4248" uniqueCount="439">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4280" uniqueCount="440">
   <si>
     <t>성동자이리버뷰 체감온도 기록</t>
   </si>
@@ -1331,6 +1331,9 @@
   </si>
   <si>
     <t>2026-09-27</t>
+  </si>
+  <si>
+    <t>22:17</t>
   </si>
 </sst>
 </file>
@@ -1751,7 +1754,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G1057"/>
+  <dimension ref="A1:G1065"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
@@ -26059,6 +26062,190 @@
         <v>11</v>
       </c>
     </row>
+    <row r="1058" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1058" s="5" t="s">
+        <v>438</v>
+      </c>
+      <c r="B1058" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1058" s="5" t="s">
+        <v>439</v>
+      </c>
+      <c r="D1058" s="5">
+        <v>23.4</v>
+      </c>
+      <c r="E1058" s="5">
+        <v>64</v>
+      </c>
+      <c r="F1058" s="5">
+        <v>24</v>
+      </c>
+      <c r="G1058" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1059" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1059" s="5" t="s">
+        <v>438</v>
+      </c>
+      <c r="B1059" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="C1059" s="5" t="s">
+        <v>439</v>
+      </c>
+      <c r="D1059" s="5">
+        <v>25.9</v>
+      </c>
+      <c r="E1059" s="5">
+        <v>55</v>
+      </c>
+      <c r="F1059" s="5">
+        <v>26</v>
+      </c>
+      <c r="G1059" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1060" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1060" s="5" t="s">
+        <v>438</v>
+      </c>
+      <c r="B1060" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="C1060" s="5" t="s">
+        <v>439</v>
+      </c>
+      <c r="D1060" s="5">
+        <v>26</v>
+      </c>
+      <c r="E1060" s="5">
+        <v>47</v>
+      </c>
+      <c r="F1060" s="5">
+        <v>25</v>
+      </c>
+      <c r="G1060" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1061" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1061" s="5" t="s">
+        <v>438</v>
+      </c>
+      <c r="B1061" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1061" s="5" t="s">
+        <v>439</v>
+      </c>
+      <c r="D1061" s="5">
+        <v>28.5</v>
+      </c>
+      <c r="E1061" s="5">
+        <v>39</v>
+      </c>
+      <c r="F1061" s="5">
+        <v>27</v>
+      </c>
+      <c r="G1061" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1062" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1062" s="5" t="s">
+        <v>438</v>
+      </c>
+      <c r="B1062" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="C1062" s="5" t="s">
+        <v>439</v>
+      </c>
+      <c r="D1062" s="5">
+        <v>27.6</v>
+      </c>
+      <c r="E1062" s="5">
+        <v>43</v>
+      </c>
+      <c r="F1062" s="5">
+        <v>27</v>
+      </c>
+      <c r="G1062" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1063" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1063" s="5" t="s">
+        <v>438</v>
+      </c>
+      <c r="B1063" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="C1063" s="5" t="s">
+        <v>439</v>
+      </c>
+      <c r="D1063" s="5">
+        <v>27.5</v>
+      </c>
+      <c r="E1063" s="5">
+        <v>46</v>
+      </c>
+      <c r="F1063" s="5">
+        <v>27</v>
+      </c>
+      <c r="G1063" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1064" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1064" s="5" t="s">
+        <v>438</v>
+      </c>
+      <c r="B1064" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1064" s="5" t="s">
+        <v>439</v>
+      </c>
+      <c r="D1064" s="5">
+        <v>28</v>
+      </c>
+      <c r="E1064" s="5">
+        <v>44</v>
+      </c>
+      <c r="F1064" s="5">
+        <v>27</v>
+      </c>
+      <c r="G1064" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1065" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1065" s="5" t="s">
+        <v>438</v>
+      </c>
+      <c r="B1065" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="C1065" s="5" t="s">
+        <v>439</v>
+      </c>
+      <c r="D1065" s="5">
+        <v>27</v>
+      </c>
+      <c r="E1065" s="5">
+        <v>51</v>
+      </c>
+      <c r="F1065" s="5">
+        <v>27</v>
+      </c>
+      <c r="G1065" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>

</xml_diff>

<commit_message>
📊 체감온도 기록: 2026-09-28 16:38 KST
</commit_message>
<xml_diff>
--- a/data/체감온도기록_2026.xlsx
+++ b/data/체감온도기록_2026.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4280" uniqueCount="440">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4316" uniqueCount="441">
   <si>
     <t>성동자이리버뷰 체감온도 기록</t>
   </si>
@@ -1334,6 +1334,9 @@
   </si>
   <si>
     <t>22:17</t>
+  </si>
+  <si>
+    <t>2026-09-28</t>
   </si>
 </sst>
 </file>
@@ -1754,7 +1757,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G1065"/>
+  <dimension ref="A1:G1074"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
@@ -26246,6 +26249,213 @@
         <v>11</v>
       </c>
     </row>
+    <row r="1066" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1066" s="5" t="s">
+        <v>440</v>
+      </c>
+      <c r="B1066" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1066" s="5" t="s">
+        <v>316</v>
+      </c>
+      <c r="D1066" s="5">
+        <v>20</v>
+      </c>
+      <c r="E1066" s="5">
+        <v>80</v>
+      </c>
+      <c r="F1066" s="5">
+        <v>22</v>
+      </c>
+      <c r="G1066" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1067" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1067" s="5" t="s">
+        <v>440</v>
+      </c>
+      <c r="B1067" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="C1067" s="5" t="s">
+        <v>316</v>
+      </c>
+      <c r="D1067" s="5">
+        <v>20.7</v>
+      </c>
+      <c r="E1067" s="5">
+        <v>73</v>
+      </c>
+      <c r="F1067" s="5">
+        <v>22</v>
+      </c>
+      <c r="G1067" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1068" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1068" s="5" t="s">
+        <v>440</v>
+      </c>
+      <c r="B1068" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="C1068" s="5" t="s">
+        <v>316</v>
+      </c>
+      <c r="D1068" s="5">
+        <v>21.5</v>
+      </c>
+      <c r="E1068" s="5">
+        <v>68</v>
+      </c>
+      <c r="F1068" s="5">
+        <v>23</v>
+      </c>
+      <c r="G1068" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1069" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1069" s="5" t="s">
+        <v>440</v>
+      </c>
+      <c r="B1069" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1069" s="5" t="s">
+        <v>316</v>
+      </c>
+      <c r="D1069" s="5">
+        <v>22.6</v>
+      </c>
+      <c r="E1069" s="5">
+        <v>61</v>
+      </c>
+      <c r="F1069" s="5">
+        <v>23</v>
+      </c>
+      <c r="G1069" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1070" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1070" s="5" t="s">
+        <v>440</v>
+      </c>
+      <c r="B1070" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="C1070" s="5" t="s">
+        <v>316</v>
+      </c>
+      <c r="D1070" s="5">
+        <v>23.2</v>
+      </c>
+      <c r="E1070" s="5">
+        <v>54</v>
+      </c>
+      <c r="F1070" s="5">
+        <v>23</v>
+      </c>
+      <c r="G1070" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1071" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1071" s="5" t="s">
+        <v>440</v>
+      </c>
+      <c r="B1071" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="C1071" s="5" t="s">
+        <v>316</v>
+      </c>
+      <c r="D1071" s="5">
+        <v>25.1</v>
+      </c>
+      <c r="E1071" s="5">
+        <v>40</v>
+      </c>
+      <c r="F1071" s="5">
+        <v>24</v>
+      </c>
+      <c r="G1071" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1072" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1072" s="5" t="s">
+        <v>440</v>
+      </c>
+      <c r="B1072" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1072" s="5" t="s">
+        <v>316</v>
+      </c>
+      <c r="D1072" s="5">
+        <v>24.7</v>
+      </c>
+      <c r="E1072" s="5">
+        <v>42</v>
+      </c>
+      <c r="F1072" s="5">
+        <v>24</v>
+      </c>
+      <c r="G1072" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1073" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1073" s="5" t="s">
+        <v>440</v>
+      </c>
+      <c r="B1073" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="C1073" s="5" t="s">
+        <v>316</v>
+      </c>
+      <c r="D1073" s="5">
+        <v>25.8</v>
+      </c>
+      <c r="E1073" s="5">
+        <v>26</v>
+      </c>
+      <c r="F1073" s="5">
+        <v>23</v>
+      </c>
+      <c r="G1073" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1074" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1074" s="5" t="s">
+        <v>440</v>
+      </c>
+      <c r="B1074" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="C1074" s="5" t="s">
+        <v>316</v>
+      </c>
+      <c r="D1074" s="5">
+        <v>25.2</v>
+      </c>
+      <c r="E1074" s="5">
+        <v>37</v>
+      </c>
+      <c r="F1074" s="5">
+        <v>24</v>
+      </c>
+      <c r="G1074" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>

</xml_diff>

<commit_message>
📊 체감온도 기록: 2026-09-29 11:18 KST
</commit_message>
<xml_diff>
--- a/data/체감온도기록_2026.xlsx
+++ b/data/체감온도기록_2026.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4316" uniqueCount="441">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4332" uniqueCount="443">
   <si>
     <t>성동자이리버뷰 체감온도 기록</t>
   </si>
@@ -1337,6 +1337,12 @@
   </si>
   <si>
     <t>2026-09-28</t>
+  </si>
+  <si>
+    <t>2026-09-29</t>
+  </si>
+  <si>
+    <t>11:18</t>
   </si>
 </sst>
 </file>
@@ -1757,7 +1763,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G1074"/>
+  <dimension ref="A1:G1078"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
@@ -26456,6 +26462,98 @@
         <v>11</v>
       </c>
     </row>
+    <row r="1075" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1075" s="5" t="s">
+        <v>441</v>
+      </c>
+      <c r="B1075" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1075" s="5" t="s">
+        <v>442</v>
+      </c>
+      <c r="D1075" s="5">
+        <v>16.2</v>
+      </c>
+      <c r="E1075" s="5">
+        <v>74</v>
+      </c>
+      <c r="F1075" s="5">
+        <v>18</v>
+      </c>
+      <c r="G1075" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1076" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1076" s="5" t="s">
+        <v>441</v>
+      </c>
+      <c r="B1076" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="C1076" s="5" t="s">
+        <v>442</v>
+      </c>
+      <c r="D1076" s="5">
+        <v>18.1</v>
+      </c>
+      <c r="E1076" s="5">
+        <v>68</v>
+      </c>
+      <c r="F1076" s="5">
+        <v>19</v>
+      </c>
+      <c r="G1076" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1077" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1077" s="5" t="s">
+        <v>441</v>
+      </c>
+      <c r="B1077" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="C1077" s="5" t="s">
+        <v>442</v>
+      </c>
+      <c r="D1077" s="5">
+        <v>19.9</v>
+      </c>
+      <c r="E1077" s="5">
+        <v>61</v>
+      </c>
+      <c r="F1077" s="5">
+        <v>21</v>
+      </c>
+      <c r="G1077" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1078" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1078" s="5" t="s">
+        <v>441</v>
+      </c>
+      <c r="B1078" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1078" s="5" t="s">
+        <v>442</v>
+      </c>
+      <c r="D1078" s="5">
+        <v>22</v>
+      </c>
+      <c r="E1078" s="5">
+        <v>54</v>
+      </c>
+      <c r="F1078" s="5">
+        <v>22</v>
+      </c>
+      <c r="G1078" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>

</xml_diff>

<commit_message>
📊 체감온도 기록: 2026-09-29 18:03 KST
</commit_message>
<xml_diff>
--- a/data/체감온도기록_2026.xlsx
+++ b/data/체감온도기록_2026.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4332" uniqueCount="443">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4360" uniqueCount="444">
   <si>
     <t>성동자이리버뷰 체감온도 기록</t>
   </si>
@@ -1343,6 +1343,9 @@
   </si>
   <si>
     <t>11:18</t>
+  </si>
+  <si>
+    <t>18:03</t>
   </si>
 </sst>
 </file>
@@ -1763,7 +1766,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G1078"/>
+  <dimension ref="A1:G1085"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
@@ -26554,6 +26557,167 @@
         <v>11</v>
       </c>
     </row>
+    <row r="1079" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1079" s="5" t="s">
+        <v>441</v>
+      </c>
+      <c r="B1079" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="C1079" s="5" t="s">
+        <v>443</v>
+      </c>
+      <c r="D1079" s="5">
+        <v>23.7</v>
+      </c>
+      <c r="E1079" s="5">
+        <v>48</v>
+      </c>
+      <c r="F1079" s="5">
+        <v>23</v>
+      </c>
+      <c r="G1079" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1080" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1080" s="5" t="s">
+        <v>441</v>
+      </c>
+      <c r="B1080" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="C1080" s="5" t="s">
+        <v>443</v>
+      </c>
+      <c r="D1080" s="5">
+        <v>24.8</v>
+      </c>
+      <c r="E1080" s="5">
+        <v>45</v>
+      </c>
+      <c r="F1080" s="5">
+        <v>24</v>
+      </c>
+      <c r="G1080" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1081" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1081" s="5" t="s">
+        <v>441</v>
+      </c>
+      <c r="B1081" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1081" s="5" t="s">
+        <v>443</v>
+      </c>
+      <c r="D1081" s="5">
+        <v>26.2</v>
+      </c>
+      <c r="E1081" s="5">
+        <v>41</v>
+      </c>
+      <c r="F1081" s="5">
+        <v>25</v>
+      </c>
+      <c r="G1081" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1082" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1082" s="5" t="s">
+        <v>441</v>
+      </c>
+      <c r="B1082" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="C1082" s="5" t="s">
+        <v>443</v>
+      </c>
+      <c r="D1082" s="5">
+        <v>26.8</v>
+      </c>
+      <c r="E1082" s="5">
+        <v>40</v>
+      </c>
+      <c r="F1082" s="5">
+        <v>26</v>
+      </c>
+      <c r="G1082" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1083" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1083" s="5" t="s">
+        <v>441</v>
+      </c>
+      <c r="B1083" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="C1083" s="5" t="s">
+        <v>443</v>
+      </c>
+      <c r="D1083" s="5">
+        <v>27</v>
+      </c>
+      <c r="E1083" s="5">
+        <v>41</v>
+      </c>
+      <c r="F1083" s="5">
+        <v>26</v>
+      </c>
+      <c r="G1083" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1084" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1084" s="5" t="s">
+        <v>441</v>
+      </c>
+      <c r="B1084" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1084" s="5" t="s">
+        <v>443</v>
+      </c>
+      <c r="D1084" s="5">
+        <v>26.5</v>
+      </c>
+      <c r="E1084" s="5">
+        <v>40</v>
+      </c>
+      <c r="F1084" s="5">
+        <v>25</v>
+      </c>
+      <c r="G1084" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1085" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1085" s="5" t="s">
+        <v>441</v>
+      </c>
+      <c r="B1085" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="C1085" s="5" t="s">
+        <v>443</v>
+      </c>
+      <c r="D1085" s="5">
+        <v>26.4</v>
+      </c>
+      <c r="E1085" s="5">
+        <v>39</v>
+      </c>
+      <c r="F1085" s="5">
+        <v>25</v>
+      </c>
+      <c r="G1085" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>

</xml_diff>

<commit_message>
📊 체감온도 기록: 2026-09-30 16:27 KST
</commit_message>
<xml_diff>
--- a/data/체감온도기록_2026.xlsx
+++ b/data/체감온도기록_2026.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4360" uniqueCount="444">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4396" uniqueCount="446">
   <si>
     <t>성동자이리버뷰 체감온도 기록</t>
   </si>
@@ -1346,6 +1346,12 @@
   </si>
   <si>
     <t>18:03</t>
+  </si>
+  <si>
+    <t>2026-09-30</t>
+  </si>
+  <si>
+    <t>16:27</t>
   </si>
 </sst>
 </file>
@@ -1766,7 +1772,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G1085"/>
+  <dimension ref="A1:G1094"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
@@ -26718,6 +26724,213 @@
         <v>11</v>
       </c>
     </row>
+    <row r="1086" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1086" s="5" t="s">
+        <v>444</v>
+      </c>
+      <c r="B1086" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1086" s="5" t="s">
+        <v>445</v>
+      </c>
+      <c r="D1086" s="5">
+        <v>18.1</v>
+      </c>
+      <c r="E1086" s="5">
+        <v>74</v>
+      </c>
+      <c r="F1086" s="5">
+        <v>20</v>
+      </c>
+      <c r="G1086" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1087" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1087" s="5" t="s">
+        <v>444</v>
+      </c>
+      <c r="B1087" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="C1087" s="5" t="s">
+        <v>445</v>
+      </c>
+      <c r="D1087" s="5">
+        <v>20</v>
+      </c>
+      <c r="E1087" s="5">
+        <v>69</v>
+      </c>
+      <c r="F1087" s="5">
+        <v>21</v>
+      </c>
+      <c r="G1087" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1088" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1088" s="5" t="s">
+        <v>444</v>
+      </c>
+      <c r="B1088" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="C1088" s="5" t="s">
+        <v>445</v>
+      </c>
+      <c r="D1088" s="5">
+        <v>22.1</v>
+      </c>
+      <c r="E1088" s="5">
+        <v>63</v>
+      </c>
+      <c r="F1088" s="5">
+        <v>23</v>
+      </c>
+      <c r="G1088" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1089" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1089" s="5" t="s">
+        <v>444</v>
+      </c>
+      <c r="B1089" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1089" s="5" t="s">
+        <v>445</v>
+      </c>
+      <c r="D1089" s="5">
+        <v>23.3</v>
+      </c>
+      <c r="E1089" s="5">
+        <v>58</v>
+      </c>
+      <c r="F1089" s="5">
+        <v>24</v>
+      </c>
+      <c r="G1089" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1090" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1090" s="5" t="s">
+        <v>444</v>
+      </c>
+      <c r="B1090" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="C1090" s="5" t="s">
+        <v>445</v>
+      </c>
+      <c r="D1090" s="5">
+        <v>24</v>
+      </c>
+      <c r="E1090" s="5">
+        <v>53</v>
+      </c>
+      <c r="F1090" s="5">
+        <v>24</v>
+      </c>
+      <c r="G1090" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1091" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1091" s="5" t="s">
+        <v>444</v>
+      </c>
+      <c r="B1091" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="C1091" s="5" t="s">
+        <v>445</v>
+      </c>
+      <c r="D1091" s="5">
+        <v>26.7</v>
+      </c>
+      <c r="E1091" s="5">
+        <v>41</v>
+      </c>
+      <c r="F1091" s="5">
+        <v>26</v>
+      </c>
+      <c r="G1091" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1092" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1092" s="5" t="s">
+        <v>444</v>
+      </c>
+      <c r="B1092" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1092" s="5" t="s">
+        <v>445</v>
+      </c>
+      <c r="D1092" s="5">
+        <v>26.9</v>
+      </c>
+      <c r="E1092" s="5">
+        <v>38</v>
+      </c>
+      <c r="F1092" s="5">
+        <v>25</v>
+      </c>
+      <c r="G1092" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1093" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1093" s="5" t="s">
+        <v>444</v>
+      </c>
+      <c r="B1093" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="C1093" s="5" t="s">
+        <v>445</v>
+      </c>
+      <c r="D1093" s="5">
+        <v>27.4</v>
+      </c>
+      <c r="E1093" s="5">
+        <v>39</v>
+      </c>
+      <c r="F1093" s="5">
+        <v>26</v>
+      </c>
+      <c r="G1093" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1094" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1094" s="5" t="s">
+        <v>444</v>
+      </c>
+      <c r="B1094" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="C1094" s="5" t="s">
+        <v>445</v>
+      </c>
+      <c r="D1094" s="5">
+        <v>27.2</v>
+      </c>
+      <c r="E1094" s="5">
+        <v>34</v>
+      </c>
+      <c r="F1094" s="5">
+        <v>25</v>
+      </c>
+      <c r="G1094" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>

</xml_diff>

<commit_message>
📊 체감온도 기록: 2026-09-30 23:14 KST
</commit_message>
<xml_diff>
--- a/data/체감온도기록_2026.xlsx
+++ b/data/체감온도기록_2026.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4396" uniqueCount="446">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4404" uniqueCount="447">
   <si>
     <t>성동자이리버뷰 체감온도 기록</t>
   </si>
@@ -1352,6 +1352,9 @@
   </si>
   <si>
     <t>16:27</t>
+  </si>
+  <si>
+    <t>23:14</t>
   </si>
 </sst>
 </file>
@@ -1772,7 +1775,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G1094"/>
+  <dimension ref="A1:G1096"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
@@ -26931,6 +26934,52 @@
         <v>11</v>
       </c>
     </row>
+    <row r="1095" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1095" s="5" t="s">
+        <v>444</v>
+      </c>
+      <c r="B1095" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1095" s="5" t="s">
+        <v>446</v>
+      </c>
+      <c r="D1095" s="5">
+        <v>26.7</v>
+      </c>
+      <c r="E1095" s="5">
+        <v>36</v>
+      </c>
+      <c r="F1095" s="5">
+        <v>25</v>
+      </c>
+      <c r="G1095" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1096" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1096" s="5" t="s">
+        <v>444</v>
+      </c>
+      <c r="B1096" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="C1096" s="5" t="s">
+        <v>446</v>
+      </c>
+      <c r="D1096" s="5">
+        <v>25.1</v>
+      </c>
+      <c r="E1096" s="5">
+        <v>41</v>
+      </c>
+      <c r="F1096" s="5">
+        <v>24</v>
+      </c>
+      <c r="G1096" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>

</xml_diff>

<commit_message>
📊 체감온도 기록: 2026-10-01 10:34 KST
</commit_message>
<xml_diff>
--- a/data/체감온도기록_2026.xlsx
+++ b/data/체감온도기록_2026.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4404" uniqueCount="447">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4416" uniqueCount="449">
   <si>
     <t>성동자이리버뷰 체감온도 기록</t>
   </si>
@@ -1355,6 +1355,12 @@
   </si>
   <si>
     <t>23:14</t>
+  </si>
+  <si>
+    <t>2026-10-01</t>
+  </si>
+  <si>
+    <t>10:34</t>
   </si>
 </sst>
 </file>
@@ -1775,7 +1781,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G1096"/>
+  <dimension ref="A1:G1099"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
@@ -26980,6 +26986,75 @@
         <v>11</v>
       </c>
     </row>
+    <row r="1097" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1097" s="5" t="s">
+        <v>447</v>
+      </c>
+      <c r="B1097" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1097" s="5" t="s">
+        <v>448</v>
+      </c>
+      <c r="D1097" s="5">
+        <v>15.8</v>
+      </c>
+      <c r="E1097" s="5">
+        <v>39</v>
+      </c>
+      <c r="F1097" s="5">
+        <v>15</v>
+      </c>
+      <c r="G1097" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1098" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1098" s="5" t="s">
+        <v>447</v>
+      </c>
+      <c r="B1098" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="C1098" s="5" t="s">
+        <v>448</v>
+      </c>
+      <c r="D1098" s="5">
+        <v>16.4</v>
+      </c>
+      <c r="E1098" s="5">
+        <v>39</v>
+      </c>
+      <c r="F1098" s="5">
+        <v>16</v>
+      </c>
+      <c r="G1098" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1099" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1099" s="5" t="s">
+        <v>447</v>
+      </c>
+      <c r="B1099" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="C1099" s="5" t="s">
+        <v>448</v>
+      </c>
+      <c r="D1099" s="5">
+        <v>17</v>
+      </c>
+      <c r="E1099" s="5">
+        <v>32</v>
+      </c>
+      <c r="F1099" s="5">
+        <v>16</v>
+      </c>
+      <c r="G1099" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>

</xml_diff>

<commit_message>
📊 체감온도 기록: 2026-10-01 16:48 KST
</commit_message>
<xml_diff>
--- a/data/체감온도기록_2026.xlsx
+++ b/data/체감온도기록_2026.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4416" uniqueCount="449">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4444" uniqueCount="449">
   <si>
     <t>성동자이리버뷰 체감온도 기록</t>
   </si>
@@ -1781,7 +1781,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G1099"/>
+  <dimension ref="A1:G1106"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
@@ -27055,6 +27055,167 @@
         <v>11</v>
       </c>
     </row>
+    <row r="1100" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1100" s="5" t="s">
+        <v>447</v>
+      </c>
+      <c r="B1100" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1100" s="5" t="s">
+        <v>179</v>
+      </c>
+      <c r="D1100" s="5">
+        <v>18.5</v>
+      </c>
+      <c r="E1100" s="5">
+        <v>23</v>
+      </c>
+      <c r="F1100" s="5">
+        <v>16</v>
+      </c>
+      <c r="G1100" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1101" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1101" s="5" t="s">
+        <v>447</v>
+      </c>
+      <c r="B1101" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="C1101" s="5" t="s">
+        <v>179</v>
+      </c>
+      <c r="D1101" s="5">
+        <v>20</v>
+      </c>
+      <c r="E1101" s="5">
+        <v>18</v>
+      </c>
+      <c r="F1101" s="5">
+        <v>17</v>
+      </c>
+      <c r="G1101" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1102" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1102" s="5" t="s">
+        <v>447</v>
+      </c>
+      <c r="B1102" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="C1102" s="5" t="s">
+        <v>179</v>
+      </c>
+      <c r="D1102" s="5">
+        <v>20.5</v>
+      </c>
+      <c r="E1102" s="5">
+        <v>16</v>
+      </c>
+      <c r="F1102" s="5">
+        <v>17</v>
+      </c>
+      <c r="G1102" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1103" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1103" s="5" t="s">
+        <v>447</v>
+      </c>
+      <c r="B1103" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1103" s="5" t="s">
+        <v>179</v>
+      </c>
+      <c r="D1103" s="5">
+        <v>20.8</v>
+      </c>
+      <c r="E1103" s="5">
+        <v>18</v>
+      </c>
+      <c r="F1103" s="5">
+        <v>18</v>
+      </c>
+      <c r="G1103" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1104" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1104" s="5" t="s">
+        <v>447</v>
+      </c>
+      <c r="B1104" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="C1104" s="5" t="s">
+        <v>179</v>
+      </c>
+      <c r="D1104" s="5">
+        <v>21.6</v>
+      </c>
+      <c r="E1104" s="5">
+        <v>20</v>
+      </c>
+      <c r="F1104" s="5">
+        <v>19</v>
+      </c>
+      <c r="G1104" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1105" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1105" s="5" t="s">
+        <v>447</v>
+      </c>
+      <c r="B1105" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="C1105" s="5" t="s">
+        <v>179</v>
+      </c>
+      <c r="D1105" s="5">
+        <v>22.1</v>
+      </c>
+      <c r="E1105" s="5">
+        <v>22</v>
+      </c>
+      <c r="F1105" s="5">
+        <v>19</v>
+      </c>
+      <c r="G1105" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1106" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1106" s="5" t="s">
+        <v>447</v>
+      </c>
+      <c r="B1106" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1106" s="5" t="s">
+        <v>179</v>
+      </c>
+      <c r="D1106" s="5">
+        <v>21.6</v>
+      </c>
+      <c r="E1106" s="5">
+        <v>26</v>
+      </c>
+      <c r="F1106" s="5">
+        <v>19</v>
+      </c>
+      <c r="G1106" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>

</xml_diff>

<commit_message>
📊 체감온도 기록: 2026-10-02 10:48 KST
</commit_message>
<xml_diff>
--- a/data/체감온도기록_2026.xlsx
+++ b/data/체감온도기록_2026.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4444" uniqueCount="449">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4460" uniqueCount="451">
   <si>
     <t>성동자이리버뷰 체감온도 기록</t>
   </si>
@@ -1361,6 +1361,12 @@
   </si>
   <si>
     <t>10:34</t>
+  </si>
+  <si>
+    <t>2026-10-02</t>
+  </si>
+  <si>
+    <t>10:48</t>
   </si>
 </sst>
 </file>
@@ -1781,7 +1787,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G1106"/>
+  <dimension ref="A1:G1110"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
@@ -27216,6 +27222,98 @@
         <v>11</v>
       </c>
     </row>
+    <row r="1107" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1107" s="5" t="s">
+        <v>449</v>
+      </c>
+      <c r="B1107" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1107" s="5" t="s">
+        <v>450</v>
+      </c>
+      <c r="D1107" s="5">
+        <v>12.6</v>
+      </c>
+      <c r="E1107" s="5">
+        <v>52</v>
+      </c>
+      <c r="F1107" s="5">
+        <v>13</v>
+      </c>
+      <c r="G1107" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1108" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1108" s="5" t="s">
+        <v>449</v>
+      </c>
+      <c r="B1108" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="C1108" s="5" t="s">
+        <v>450</v>
+      </c>
+      <c r="D1108" s="5">
+        <v>13.7</v>
+      </c>
+      <c r="E1108" s="5">
+        <v>51</v>
+      </c>
+      <c r="F1108" s="5">
+        <v>14</v>
+      </c>
+      <c r="G1108" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1109" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1109" s="5" t="s">
+        <v>449</v>
+      </c>
+      <c r="B1109" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="C1109" s="5" t="s">
+        <v>450</v>
+      </c>
+      <c r="D1109" s="5">
+        <v>16.4</v>
+      </c>
+      <c r="E1109" s="5">
+        <v>41</v>
+      </c>
+      <c r="F1109" s="5">
+        <v>16</v>
+      </c>
+      <c r="G1109" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1110" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1110" s="5" t="s">
+        <v>449</v>
+      </c>
+      <c r="B1110" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1110" s="5" t="s">
+        <v>450</v>
+      </c>
+      <c r="D1110" s="5">
+        <v>18.3</v>
+      </c>
+      <c r="E1110" s="5">
+        <v>34</v>
+      </c>
+      <c r="F1110" s="5">
+        <v>17</v>
+      </c>
+      <c r="G1110" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>

</xml_diff>

<commit_message>
📊 체감온도 기록: 2026-10-02 18:00 KST
</commit_message>
<xml_diff>
--- a/data/체감온도기록_2026.xlsx
+++ b/data/체감온도기록_2026.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4460" uniqueCount="451">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4488" uniqueCount="451">
   <si>
     <t>성동자이리버뷰 체감온도 기록</t>
   </si>
@@ -1787,7 +1787,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G1110"/>
+  <dimension ref="A1:G1117"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
@@ -27314,6 +27314,167 @@
         <v>11</v>
       </c>
     </row>
+    <row r="1111" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1111" s="5" t="s">
+        <v>449</v>
+      </c>
+      <c r="B1111" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="C1111" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1111" s="5">
+        <v>18.8</v>
+      </c>
+      <c r="E1111" s="5">
+        <v>26</v>
+      </c>
+      <c r="F1111" s="5">
+        <v>17</v>
+      </c>
+      <c r="G1111" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1112" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1112" s="5" t="s">
+        <v>449</v>
+      </c>
+      <c r="B1112" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="C1112" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1112" s="5">
+        <v>19.9</v>
+      </c>
+      <c r="E1112" s="5">
+        <v>23</v>
+      </c>
+      <c r="F1112" s="5">
+        <v>17</v>
+      </c>
+      <c r="G1112" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1113" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1113" s="5" t="s">
+        <v>449</v>
+      </c>
+      <c r="B1113" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1113" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1113" s="5">
+        <v>20.7</v>
+      </c>
+      <c r="E1113" s="5">
+        <v>22</v>
+      </c>
+      <c r="F1113" s="5">
+        <v>18</v>
+      </c>
+      <c r="G1113" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1114" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1114" s="5" t="s">
+        <v>449</v>
+      </c>
+      <c r="B1114" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="C1114" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1114" s="5">
+        <v>21</v>
+      </c>
+      <c r="E1114" s="5">
+        <v>24</v>
+      </c>
+      <c r="F1114" s="5">
+        <v>19</v>
+      </c>
+      <c r="G1114" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1115" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1115" s="5" t="s">
+        <v>449</v>
+      </c>
+      <c r="B1115" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="C1115" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1115" s="5">
+        <v>21.5</v>
+      </c>
+      <c r="E1115" s="5">
+        <v>24</v>
+      </c>
+      <c r="F1115" s="5">
+        <v>19</v>
+      </c>
+      <c r="G1115" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1116" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1116" s="5" t="s">
+        <v>449</v>
+      </c>
+      <c r="B1116" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1116" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1116" s="5">
+        <v>21.7</v>
+      </c>
+      <c r="E1116" s="5">
+        <v>24</v>
+      </c>
+      <c r="F1116" s="5">
+        <v>19</v>
+      </c>
+      <c r="G1116" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1117" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1117" s="5" t="s">
+        <v>449</v>
+      </c>
+      <c r="B1117" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="C1117" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1117" s="5">
+        <v>21.4</v>
+      </c>
+      <c r="E1117" s="5">
+        <v>25</v>
+      </c>
+      <c r="F1117" s="5">
+        <v>19</v>
+      </c>
+      <c r="G1117" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>

</xml_diff>

<commit_message>
📊 체감온도 기록: 2026-10-03 10:26 KST
</commit_message>
<xml_diff>
--- a/data/체감온도기록_2026.xlsx
+++ b/data/체감온도기록_2026.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4488" uniqueCount="451">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4500" uniqueCount="453">
   <si>
     <t>성동자이리버뷰 체감온도 기록</t>
   </si>
@@ -1367,6 +1367,12 @@
   </si>
   <si>
     <t>10:48</t>
+  </si>
+  <si>
+    <t>2026-10-03</t>
+  </si>
+  <si>
+    <t>10:26</t>
   </si>
 </sst>
 </file>
@@ -1787,7 +1793,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G1117"/>
+  <dimension ref="A1:G1120"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
@@ -27475,6 +27481,75 @@
         <v>11</v>
       </c>
     </row>
+    <row r="1118" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1118" s="5" t="s">
+        <v>451</v>
+      </c>
+      <c r="B1118" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1118" s="5" t="s">
+        <v>452</v>
+      </c>
+      <c r="D1118" s="5">
+        <v>12.5</v>
+      </c>
+      <c r="E1118" s="5">
+        <v>57</v>
+      </c>
+      <c r="F1118" s="5">
+        <v>13</v>
+      </c>
+      <c r="G1118" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1119" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1119" s="5" t="s">
+        <v>451</v>
+      </c>
+      <c r="B1119" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="C1119" s="5" t="s">
+        <v>452</v>
+      </c>
+      <c r="D1119" s="5">
+        <v>13.5</v>
+      </c>
+      <c r="E1119" s="5">
+        <v>53</v>
+      </c>
+      <c r="F1119" s="5">
+        <v>14</v>
+      </c>
+      <c r="G1119" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1120" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1120" s="5" t="s">
+        <v>451</v>
+      </c>
+      <c r="B1120" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="C1120" s="5" t="s">
+        <v>452</v>
+      </c>
+      <c r="D1120" s="5">
+        <v>15.9</v>
+      </c>
+      <c r="E1120" s="5">
+        <v>47</v>
+      </c>
+      <c r="F1120" s="5">
+        <v>16</v>
+      </c>
+      <c r="G1120" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>

</xml_diff>

<commit_message>
📊 체감온도 기록: 2026-10-03 16:05 KST
</commit_message>
<xml_diff>
--- a/data/체감온도기록_2026.xlsx
+++ b/data/체감온도기록_2026.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4500" uniqueCount="453">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4524" uniqueCount="454">
   <si>
     <t>성동자이리버뷰 체감온도 기록</t>
   </si>
@@ -1373,6 +1373,9 @@
   </si>
   <si>
     <t>10:26</t>
+  </si>
+  <si>
+    <t>16:05</t>
   </si>
 </sst>
 </file>
@@ -1793,7 +1796,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G1120"/>
+  <dimension ref="A1:G1126"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
@@ -27550,6 +27553,144 @@
         <v>11</v>
       </c>
     </row>
+    <row r="1121" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1121" s="5" t="s">
+        <v>451</v>
+      </c>
+      <c r="B1121" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1121" s="5" t="s">
+        <v>453</v>
+      </c>
+      <c r="D1121" s="5">
+        <v>17.4</v>
+      </c>
+      <c r="E1121" s="5">
+        <v>44</v>
+      </c>
+      <c r="F1121" s="5">
+        <v>17</v>
+      </c>
+      <c r="G1121" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1122" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1122" s="5" t="s">
+        <v>451</v>
+      </c>
+      <c r="B1122" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="C1122" s="5" t="s">
+        <v>453</v>
+      </c>
+      <c r="D1122" s="5">
+        <v>19.2</v>
+      </c>
+      <c r="E1122" s="5">
+        <v>43</v>
+      </c>
+      <c r="F1122" s="5">
+        <v>19</v>
+      </c>
+      <c r="G1122" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1123" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1123" s="5" t="s">
+        <v>451</v>
+      </c>
+      <c r="B1123" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="C1123" s="5" t="s">
+        <v>453</v>
+      </c>
+      <c r="D1123" s="5">
+        <v>20.9</v>
+      </c>
+      <c r="E1123" s="5">
+        <v>40</v>
+      </c>
+      <c r="F1123" s="5">
+        <v>20</v>
+      </c>
+      <c r="G1123" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1124" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1124" s="5" t="s">
+        <v>451</v>
+      </c>
+      <c r="B1124" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1124" s="5" t="s">
+        <v>453</v>
+      </c>
+      <c r="D1124" s="5">
+        <v>22.4</v>
+      </c>
+      <c r="E1124" s="5">
+        <v>36</v>
+      </c>
+      <c r="F1124" s="5">
+        <v>21</v>
+      </c>
+      <c r="G1124" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1125" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1125" s="5" t="s">
+        <v>451</v>
+      </c>
+      <c r="B1125" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="C1125" s="5" t="s">
+        <v>453</v>
+      </c>
+      <c r="D1125" s="5">
+        <v>22</v>
+      </c>
+      <c r="E1125" s="5">
+        <v>40</v>
+      </c>
+      <c r="F1125" s="5">
+        <v>21</v>
+      </c>
+      <c r="G1125" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1126" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1126" s="5" t="s">
+        <v>451</v>
+      </c>
+      <c r="B1126" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="C1126" s="5" t="s">
+        <v>453</v>
+      </c>
+      <c r="D1126" s="5">
+        <v>22.1</v>
+      </c>
+      <c r="E1126" s="5">
+        <v>39</v>
+      </c>
+      <c r="F1126" s="5">
+        <v>21</v>
+      </c>
+      <c r="G1126" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>

</xml_diff>

<commit_message>
📊 체감온도 기록: 2026-10-03 21:43 KST
</commit_message>
<xml_diff>
--- a/data/체감온도기록_2026.xlsx
+++ b/data/체감온도기록_2026.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4524" uniqueCount="454">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4532" uniqueCount="455">
   <si>
     <t>성동자이리버뷰 체감온도 기록</t>
   </si>
@@ -1376,6 +1376,9 @@
   </si>
   <si>
     <t>16:05</t>
+  </si>
+  <si>
+    <t>21:43</t>
   </si>
 </sst>
 </file>
@@ -1796,7 +1799,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G1126"/>
+  <dimension ref="A1:G1128"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
@@ -27691,6 +27694,52 @@
         <v>11</v>
       </c>
     </row>
+    <row r="1127" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1127" s="5" t="s">
+        <v>451</v>
+      </c>
+      <c r="B1127" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1127" s="5" t="s">
+        <v>454</v>
+      </c>
+      <c r="D1127" s="5">
+        <v>21.7</v>
+      </c>
+      <c r="E1127" s="5">
+        <v>41</v>
+      </c>
+      <c r="F1127" s="5">
+        <v>21</v>
+      </c>
+      <c r="G1127" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1128" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1128" s="5" t="s">
+        <v>451</v>
+      </c>
+      <c r="B1128" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="C1128" s="5" t="s">
+        <v>454</v>
+      </c>
+      <c r="D1128" s="5">
+        <v>21.3</v>
+      </c>
+      <c r="E1128" s="5">
+        <v>43</v>
+      </c>
+      <c r="F1128" s="5">
+        <v>21</v>
+      </c>
+      <c r="G1128" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>

</xml_diff>

<commit_message>
📊 체감온도 기록: 2026-10-04 10:59 KST
</commit_message>
<xml_diff>
--- a/data/체감온도기록_2026.xlsx
+++ b/data/체감온도기록_2026.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4532" uniqueCount="455">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4548" uniqueCount="456">
   <si>
     <t>성동자이리버뷰 체감온도 기록</t>
   </si>
@@ -1379,6 +1379,9 @@
   </si>
   <si>
     <t>21:43</t>
+  </si>
+  <si>
+    <t>2026-10-04</t>
   </si>
 </sst>
 </file>
@@ -1799,7 +1802,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G1128"/>
+  <dimension ref="A1:G1132"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
@@ -27740,6 +27743,98 @@
         <v>11</v>
       </c>
     </row>
+    <row r="1129" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1129" s="5" t="s">
+        <v>455</v>
+      </c>
+      <c r="B1129" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1129" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="D1129" s="5">
+        <v>15.5</v>
+      </c>
+      <c r="E1129" s="5">
+        <v>68</v>
+      </c>
+      <c r="F1129" s="5">
+        <v>17</v>
+      </c>
+      <c r="G1129" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1130" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1130" s="5" t="s">
+        <v>455</v>
+      </c>
+      <c r="B1130" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="C1130" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="D1130" s="5">
+        <v>17.3</v>
+      </c>
+      <c r="E1130" s="5">
+        <v>61</v>
+      </c>
+      <c r="F1130" s="5">
+        <v>18</v>
+      </c>
+      <c r="G1130" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1131" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1131" s="5" t="s">
+        <v>455</v>
+      </c>
+      <c r="B1131" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="C1131" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="D1131" s="5">
+        <v>18.9</v>
+      </c>
+      <c r="E1131" s="5">
+        <v>57</v>
+      </c>
+      <c r="F1131" s="5">
+        <v>19</v>
+      </c>
+      <c r="G1131" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1132" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1132" s="5" t="s">
+        <v>455</v>
+      </c>
+      <c r="B1132" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1132" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="D1132" s="5">
+        <v>21.2</v>
+      </c>
+      <c r="E1132" s="5">
+        <v>52</v>
+      </c>
+      <c r="F1132" s="5">
+        <v>21</v>
+      </c>
+      <c r="G1132" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>

</xml_diff>

<commit_message>
📊 체감온도 기록: 2026-10-04 17:47 KST
</commit_message>
<xml_diff>
--- a/data/체감온도기록_2026.xlsx
+++ b/data/체감온도기록_2026.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4548" uniqueCount="456">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4576" uniqueCount="456">
   <si>
     <t>성동자이리버뷰 체감온도 기록</t>
   </si>
@@ -1802,7 +1802,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G1132"/>
+  <dimension ref="A1:G1139"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
@@ -27835,6 +27835,167 @@
         <v>11</v>
       </c>
     </row>
+    <row r="1133" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1133" s="5" t="s">
+        <v>455</v>
+      </c>
+      <c r="B1133" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="C1133" s="5" t="s">
+        <v>300</v>
+      </c>
+      <c r="D1133" s="5">
+        <v>22.7</v>
+      </c>
+      <c r="E1133" s="5">
+        <v>47</v>
+      </c>
+      <c r="F1133" s="5">
+        <v>22</v>
+      </c>
+      <c r="G1133" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1134" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1134" s="5" t="s">
+        <v>455</v>
+      </c>
+      <c r="B1134" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="C1134" s="5" t="s">
+        <v>300</v>
+      </c>
+      <c r="D1134" s="5">
+        <v>24</v>
+      </c>
+      <c r="E1134" s="5">
+        <v>43</v>
+      </c>
+      <c r="F1134" s="5">
+        <v>23</v>
+      </c>
+      <c r="G1134" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1135" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1135" s="5" t="s">
+        <v>455</v>
+      </c>
+      <c r="B1135" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1135" s="5" t="s">
+        <v>300</v>
+      </c>
+      <c r="D1135" s="5">
+        <v>24</v>
+      </c>
+      <c r="E1135" s="5">
+        <v>42</v>
+      </c>
+      <c r="F1135" s="5">
+        <v>23</v>
+      </c>
+      <c r="G1135" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1136" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1136" s="5" t="s">
+        <v>455</v>
+      </c>
+      <c r="B1136" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="C1136" s="5" t="s">
+        <v>300</v>
+      </c>
+      <c r="D1136" s="5">
+        <v>24.4</v>
+      </c>
+      <c r="E1136" s="5">
+        <v>38</v>
+      </c>
+      <c r="F1136" s="5">
+        <v>23</v>
+      </c>
+      <c r="G1136" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1137" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1137" s="5" t="s">
+        <v>455</v>
+      </c>
+      <c r="B1137" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="C1137" s="5" t="s">
+        <v>300</v>
+      </c>
+      <c r="D1137" s="5">
+        <v>25.9</v>
+      </c>
+      <c r="E1137" s="5">
+        <v>37</v>
+      </c>
+      <c r="F1137" s="5">
+        <v>24</v>
+      </c>
+      <c r="G1137" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1138" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1138" s="5" t="s">
+        <v>455</v>
+      </c>
+      <c r="B1138" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1138" s="5" t="s">
+        <v>300</v>
+      </c>
+      <c r="D1138" s="5">
+        <v>25.2</v>
+      </c>
+      <c r="E1138" s="5">
+        <v>38</v>
+      </c>
+      <c r="F1138" s="5">
+        <v>24</v>
+      </c>
+      <c r="G1138" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1139" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1139" s="5" t="s">
+        <v>455</v>
+      </c>
+      <c r="B1139" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="C1139" s="5" t="s">
+        <v>300</v>
+      </c>
+      <c r="D1139" s="5">
+        <v>23.8</v>
+      </c>
+      <c r="E1139" s="5">
+        <v>42</v>
+      </c>
+      <c r="F1139" s="5">
+        <v>23</v>
+      </c>
+      <c r="G1139" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>

</xml_diff>

<commit_message>
📊 체감온도 기록: 2026-10-05 10:16 KST
</commit_message>
<xml_diff>
--- a/data/체감온도기록_2026.xlsx
+++ b/data/체감온도기록_2026.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4576" uniqueCount="456">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4588" uniqueCount="458">
   <si>
     <t>성동자이리버뷰 체감온도 기록</t>
   </si>
@@ -1382,6 +1382,12 @@
   </si>
   <si>
     <t>2026-10-04</t>
+  </si>
+  <si>
+    <t>2026-10-05</t>
+  </si>
+  <si>
+    <t>10:16</t>
   </si>
 </sst>
 </file>
@@ -1802,7 +1808,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G1139"/>
+  <dimension ref="A1:G1142"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
@@ -27996,6 +28002,75 @@
         <v>11</v>
       </c>
     </row>
+    <row r="1140" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1140" s="5" t="s">
+        <v>456</v>
+      </c>
+      <c r="B1140" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1140" s="5" t="s">
+        <v>457</v>
+      </c>
+      <c r="D1140" s="5">
+        <v>15.9</v>
+      </c>
+      <c r="E1140" s="5">
+        <v>65</v>
+      </c>
+      <c r="F1140" s="5">
+        <v>17</v>
+      </c>
+      <c r="G1140" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1141" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1141" s="5" t="s">
+        <v>456</v>
+      </c>
+      <c r="B1141" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="C1141" s="5" t="s">
+        <v>457</v>
+      </c>
+      <c r="D1141" s="5">
+        <v>16.5</v>
+      </c>
+      <c r="E1141" s="5">
+        <v>61</v>
+      </c>
+      <c r="F1141" s="5">
+        <v>17</v>
+      </c>
+      <c r="G1141" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1142" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1142" s="5" t="s">
+        <v>456</v>
+      </c>
+      <c r="B1142" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="C1142" s="5" t="s">
+        <v>457</v>
+      </c>
+      <c r="D1142" s="5">
+        <v>17.4</v>
+      </c>
+      <c r="E1142" s="5">
+        <v>55</v>
+      </c>
+      <c r="F1142" s="5">
+        <v>18</v>
+      </c>
+      <c r="G1142" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>

</xml_diff>

<commit_message>
📊 체감온도 기록: 2026-10-05 16:41 KST
</commit_message>
<xml_diff>
--- a/data/체감온도기록_2026.xlsx
+++ b/data/체감온도기록_2026.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4588" uniqueCount="458">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4616" uniqueCount="459">
   <si>
     <t>성동자이리버뷰 체감온도 기록</t>
   </si>
@@ -1388,6 +1388,9 @@
   </si>
   <si>
     <t>10:16</t>
+  </si>
+  <si>
+    <t>16:41</t>
   </si>
 </sst>
 </file>
@@ -1808,7 +1811,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G1142"/>
+  <dimension ref="A1:G1149"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
@@ -28071,6 +28074,167 @@
         <v>11</v>
       </c>
     </row>
+    <row r="1143" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1143" s="5" t="s">
+        <v>456</v>
+      </c>
+      <c r="B1143" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1143" s="5" t="s">
+        <v>458</v>
+      </c>
+      <c r="D1143" s="5">
+        <v>18</v>
+      </c>
+      <c r="E1143" s="5">
+        <v>55</v>
+      </c>
+      <c r="F1143" s="5">
+        <v>18</v>
+      </c>
+      <c r="G1143" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1144" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1144" s="5" t="s">
+        <v>456</v>
+      </c>
+      <c r="B1144" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="C1144" s="5" t="s">
+        <v>458</v>
+      </c>
+      <c r="D1144" s="5">
+        <v>18.1</v>
+      </c>
+      <c r="E1144" s="5">
+        <v>54</v>
+      </c>
+      <c r="F1144" s="5">
+        <v>18</v>
+      </c>
+      <c r="G1144" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1145" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1145" s="5" t="s">
+        <v>456</v>
+      </c>
+      <c r="B1145" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="C1145" s="5" t="s">
+        <v>458</v>
+      </c>
+      <c r="D1145" s="5">
+        <v>19.6</v>
+      </c>
+      <c r="E1145" s="5">
+        <v>49</v>
+      </c>
+      <c r="F1145" s="5">
+        <v>19</v>
+      </c>
+      <c r="G1145" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1146" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1146" s="5" t="s">
+        <v>456</v>
+      </c>
+      <c r="B1146" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1146" s="5" t="s">
+        <v>458</v>
+      </c>
+      <c r="D1146" s="5">
+        <v>19.2</v>
+      </c>
+      <c r="E1146" s="5">
+        <v>52</v>
+      </c>
+      <c r="F1146" s="5">
+        <v>19</v>
+      </c>
+      <c r="G1146" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1147" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1147" s="5" t="s">
+        <v>456</v>
+      </c>
+      <c r="B1147" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="C1147" s="5" t="s">
+        <v>458</v>
+      </c>
+      <c r="D1147" s="5">
+        <v>20.5</v>
+      </c>
+      <c r="E1147" s="5">
+        <v>45</v>
+      </c>
+      <c r="F1147" s="5">
+        <v>20</v>
+      </c>
+      <c r="G1147" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1148" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1148" s="5" t="s">
+        <v>456</v>
+      </c>
+      <c r="B1148" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="C1148" s="5" t="s">
+        <v>458</v>
+      </c>
+      <c r="D1148" s="5">
+        <v>19.8</v>
+      </c>
+      <c r="E1148" s="5">
+        <v>44</v>
+      </c>
+      <c r="F1148" s="5">
+        <v>19</v>
+      </c>
+      <c r="G1148" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1149" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1149" s="5" t="s">
+        <v>456</v>
+      </c>
+      <c r="B1149" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1149" s="5" t="s">
+        <v>458</v>
+      </c>
+      <c r="D1149" s="5">
+        <v>19.6</v>
+      </c>
+      <c r="E1149" s="5">
+        <v>47</v>
+      </c>
+      <c r="F1149" s="5">
+        <v>19</v>
+      </c>
+      <c r="G1149" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>

</xml_diff>

<commit_message>
📊 체감온도 기록: 2026-10-06 11:30 KST
</commit_message>
<xml_diff>
--- a/data/체감온도기록_2026.xlsx
+++ b/data/체감온도기록_2026.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4616" uniqueCount="459">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4632" uniqueCount="461">
   <si>
     <t>성동자이리버뷰 체감온도 기록</t>
   </si>
@@ -1391,6 +1391,12 @@
   </si>
   <si>
     <t>16:41</t>
+  </si>
+  <si>
+    <t>2026-10-06</t>
+  </si>
+  <si>
+    <t>11:30</t>
   </si>
 </sst>
 </file>
@@ -1811,7 +1817,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G1149"/>
+  <dimension ref="A1:G1153"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
@@ -28235,6 +28241,98 @@
         <v>11</v>
       </c>
     </row>
+    <row r="1150" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1150" s="5" t="s">
+        <v>459</v>
+      </c>
+      <c r="B1150" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1150" s="5" t="s">
+        <v>460</v>
+      </c>
+      <c r="D1150" s="5">
+        <v>11.1</v>
+      </c>
+      <c r="E1150" s="5">
+        <v>70</v>
+      </c>
+      <c r="F1150" s="5">
+        <v>12</v>
+      </c>
+      <c r="G1150" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1151" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1151" s="5" t="s">
+        <v>459</v>
+      </c>
+      <c r="B1151" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="C1151" s="5" t="s">
+        <v>460</v>
+      </c>
+      <c r="D1151" s="5">
+        <v>13.6</v>
+      </c>
+      <c r="E1151" s="5">
+        <v>61</v>
+      </c>
+      <c r="F1151" s="5">
+        <v>14</v>
+      </c>
+      <c r="G1151" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1152" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1152" s="5" t="s">
+        <v>459</v>
+      </c>
+      <c r="B1152" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="C1152" s="5" t="s">
+        <v>460</v>
+      </c>
+      <c r="D1152" s="5">
+        <v>15.8</v>
+      </c>
+      <c r="E1152" s="5">
+        <v>56</v>
+      </c>
+      <c r="F1152" s="5">
+        <v>16</v>
+      </c>
+      <c r="G1152" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1153" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1153" s="5" t="s">
+        <v>459</v>
+      </c>
+      <c r="B1153" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1153" s="5" t="s">
+        <v>460</v>
+      </c>
+      <c r="D1153" s="5">
+        <v>18.5</v>
+      </c>
+      <c r="E1153" s="5">
+        <v>45</v>
+      </c>
+      <c r="F1153" s="5">
+        <v>18</v>
+      </c>
+      <c r="G1153" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>

</xml_diff>

<commit_message>
📊 체감온도 기록: 2026-10-06 18:25 KST
</commit_message>
<xml_diff>
--- a/data/체감온도기록_2026.xlsx
+++ b/data/체감온도기록_2026.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4632" uniqueCount="461">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4660" uniqueCount="462">
   <si>
     <t>성동자이리버뷰 체감온도 기록</t>
   </si>
@@ -1397,6 +1397,9 @@
   </si>
   <si>
     <t>11:30</t>
+  </si>
+  <si>
+    <t>18:25</t>
   </si>
 </sst>
 </file>
@@ -1817,7 +1820,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G1153"/>
+  <dimension ref="A1:G1160"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
@@ -28333,6 +28336,167 @@
         <v>11</v>
       </c>
     </row>
+    <row r="1154" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1154" s="5" t="s">
+        <v>459</v>
+      </c>
+      <c r="B1154" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="C1154" s="5" t="s">
+        <v>461</v>
+      </c>
+      <c r="D1154" s="5">
+        <v>18.8</v>
+      </c>
+      <c r="E1154" s="5">
+        <v>32</v>
+      </c>
+      <c r="F1154" s="5">
+        <v>17</v>
+      </c>
+      <c r="G1154" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1155" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1155" s="5" t="s">
+        <v>459</v>
+      </c>
+      <c r="B1155" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="C1155" s="5" t="s">
+        <v>461</v>
+      </c>
+      <c r="D1155" s="5">
+        <v>20.3</v>
+      </c>
+      <c r="E1155" s="5">
+        <v>26</v>
+      </c>
+      <c r="F1155" s="5">
+        <v>18</v>
+      </c>
+      <c r="G1155" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1156" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1156" s="5" t="s">
+        <v>459</v>
+      </c>
+      <c r="B1156" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1156" s="5" t="s">
+        <v>461</v>
+      </c>
+      <c r="D1156" s="5">
+        <v>21.1</v>
+      </c>
+      <c r="E1156" s="5">
+        <v>26</v>
+      </c>
+      <c r="F1156" s="5">
+        <v>19</v>
+      </c>
+      <c r="G1156" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1157" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1157" s="5" t="s">
+        <v>459</v>
+      </c>
+      <c r="B1157" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="C1157" s="5" t="s">
+        <v>461</v>
+      </c>
+      <c r="D1157" s="5">
+        <v>21.4</v>
+      </c>
+      <c r="E1157" s="5">
+        <v>26</v>
+      </c>
+      <c r="F1157" s="5">
+        <v>19</v>
+      </c>
+      <c r="G1157" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1158" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1158" s="5" t="s">
+        <v>459</v>
+      </c>
+      <c r="B1158" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="C1158" s="5" t="s">
+        <v>461</v>
+      </c>
+      <c r="D1158" s="5">
+        <v>21.6</v>
+      </c>
+      <c r="E1158" s="5">
+        <v>27</v>
+      </c>
+      <c r="F1158" s="5">
+        <v>19</v>
+      </c>
+      <c r="G1158" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1159" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1159" s="5" t="s">
+        <v>459</v>
+      </c>
+      <c r="B1159" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1159" s="5" t="s">
+        <v>461</v>
+      </c>
+      <c r="D1159" s="5">
+        <v>21.7</v>
+      </c>
+      <c r="E1159" s="5">
+        <v>30</v>
+      </c>
+      <c r="F1159" s="5">
+        <v>20</v>
+      </c>
+      <c r="G1159" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1160" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1160" s="5" t="s">
+        <v>459</v>
+      </c>
+      <c r="B1160" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="C1160" s="5" t="s">
+        <v>461</v>
+      </c>
+      <c r="D1160" s="5">
+        <v>21.9</v>
+      </c>
+      <c r="E1160" s="5">
+        <v>32</v>
+      </c>
+      <c r="F1160" s="5">
+        <v>20</v>
+      </c>
+      <c r="G1160" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>

</xml_diff>

<commit_message>
📊 체감온도 기록: 2026-10-07 10:48 KST
</commit_message>
<xml_diff>
--- a/data/체감온도기록_2026.xlsx
+++ b/data/체감온도기록_2026.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4660" uniqueCount="462">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4676" uniqueCount="463">
   <si>
     <t>성동자이리버뷰 체감온도 기록</t>
   </si>
@@ -1400,6 +1400,9 @@
   </si>
   <si>
     <t>18:25</t>
+  </si>
+  <si>
+    <t>2026-10-07</t>
   </si>
 </sst>
 </file>
@@ -1820,7 +1823,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G1160"/>
+  <dimension ref="A1:G1164"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
@@ -28497,6 +28500,98 @@
         <v>11</v>
       </c>
     </row>
+    <row r="1161" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1161" s="5" t="s">
+        <v>462</v>
+      </c>
+      <c r="B1161" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1161" s="5" t="s">
+        <v>450</v>
+      </c>
+      <c r="D1161" s="5">
+        <v>12.6</v>
+      </c>
+      <c r="E1161" s="5">
+        <v>79</v>
+      </c>
+      <c r="F1161" s="5">
+        <v>14</v>
+      </c>
+      <c r="G1161" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1162" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1162" s="5" t="s">
+        <v>462</v>
+      </c>
+      <c r="B1162" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="C1162" s="5" t="s">
+        <v>450</v>
+      </c>
+      <c r="D1162" s="5">
+        <v>14.9</v>
+      </c>
+      <c r="E1162" s="5">
+        <v>70</v>
+      </c>
+      <c r="F1162" s="5">
+        <v>16</v>
+      </c>
+      <c r="G1162" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1163" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1163" s="5" t="s">
+        <v>462</v>
+      </c>
+      <c r="B1163" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="C1163" s="5" t="s">
+        <v>450</v>
+      </c>
+      <c r="D1163" s="5">
+        <v>16.5</v>
+      </c>
+      <c r="E1163" s="5">
+        <v>63</v>
+      </c>
+      <c r="F1163" s="5">
+        <v>17</v>
+      </c>
+      <c r="G1163" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1164" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1164" s="5" t="s">
+        <v>462</v>
+      </c>
+      <c r="B1164" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1164" s="5" t="s">
+        <v>450</v>
+      </c>
+      <c r="D1164" s="5">
+        <v>18.9</v>
+      </c>
+      <c r="E1164" s="5">
+        <v>55</v>
+      </c>
+      <c r="F1164" s="5">
+        <v>19</v>
+      </c>
+      <c r="G1164" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>

</xml_diff>

<commit_message>
📊 체감온도 기록: 2026-10-07 18:15 KST
</commit_message>
<xml_diff>
--- a/data/체감온도기록_2026.xlsx
+++ b/data/체감온도기록_2026.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4676" uniqueCount="463">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4704" uniqueCount="463">
   <si>
     <t>성동자이리버뷰 체감온도 기록</t>
   </si>
@@ -1823,7 +1823,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G1164"/>
+  <dimension ref="A1:G1171"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
@@ -28592,6 +28592,167 @@
         <v>11</v>
       </c>
     </row>
+    <row r="1165" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1165" s="5" t="s">
+        <v>462</v>
+      </c>
+      <c r="B1165" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="C1165" s="5" t="s">
+        <v>328</v>
+      </c>
+      <c r="D1165" s="5">
+        <v>20</v>
+      </c>
+      <c r="E1165" s="5">
+        <v>48</v>
+      </c>
+      <c r="F1165" s="5">
+        <v>20</v>
+      </c>
+      <c r="G1165" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1166" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1166" s="5" t="s">
+        <v>462</v>
+      </c>
+      <c r="B1166" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="C1166" s="5" t="s">
+        <v>328</v>
+      </c>
+      <c r="D1166" s="5">
+        <v>22.7</v>
+      </c>
+      <c r="E1166" s="5">
+        <v>38</v>
+      </c>
+      <c r="F1166" s="5">
+        <v>21</v>
+      </c>
+      <c r="G1166" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1167" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1167" s="5" t="s">
+        <v>462</v>
+      </c>
+      <c r="B1167" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1167" s="5" t="s">
+        <v>328</v>
+      </c>
+      <c r="D1167" s="5">
+        <v>23.3</v>
+      </c>
+      <c r="E1167" s="5">
+        <v>35</v>
+      </c>
+      <c r="F1167" s="5">
+        <v>22</v>
+      </c>
+      <c r="G1167" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1168" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1168" s="5" t="s">
+        <v>462</v>
+      </c>
+      <c r="B1168" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="C1168" s="5" t="s">
+        <v>328</v>
+      </c>
+      <c r="D1168" s="5">
+        <v>23.6</v>
+      </c>
+      <c r="E1168" s="5">
+        <v>27</v>
+      </c>
+      <c r="F1168" s="5">
+        <v>21</v>
+      </c>
+      <c r="G1168" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1169" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1169" s="5" t="s">
+        <v>462</v>
+      </c>
+      <c r="B1169" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="C1169" s="5" t="s">
+        <v>328</v>
+      </c>
+      <c r="D1169" s="5">
+        <v>24.2</v>
+      </c>
+      <c r="E1169" s="5">
+        <v>27</v>
+      </c>
+      <c r="F1169" s="5">
+        <v>22</v>
+      </c>
+      <c r="G1169" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1170" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1170" s="5" t="s">
+        <v>462</v>
+      </c>
+      <c r="B1170" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1170" s="5" t="s">
+        <v>328</v>
+      </c>
+      <c r="D1170" s="5">
+        <v>23.3</v>
+      </c>
+      <c r="E1170" s="5">
+        <v>31</v>
+      </c>
+      <c r="F1170" s="5">
+        <v>21</v>
+      </c>
+      <c r="G1170" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1171" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1171" s="5" t="s">
+        <v>462</v>
+      </c>
+      <c r="B1171" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="C1171" s="5" t="s">
+        <v>328</v>
+      </c>
+      <c r="D1171" s="5">
+        <v>22.4</v>
+      </c>
+      <c r="E1171" s="5">
+        <v>33</v>
+      </c>
+      <c r="F1171" s="5">
+        <v>21</v>
+      </c>
+      <c r="G1171" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>

</xml_diff>

<commit_message>
📊 체감온도 기록: 2026-10-08 11:16 KST
</commit_message>
<xml_diff>
--- a/data/체감온도기록_2026.xlsx
+++ b/data/체감온도기록_2026.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4704" uniqueCount="463">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4720" uniqueCount="465">
   <si>
     <t>성동자이리버뷰 체감온도 기록</t>
   </si>
@@ -1403,6 +1403,12 @@
   </si>
   <si>
     <t>2026-10-07</t>
+  </si>
+  <si>
+    <t>2026-10-08</t>
+  </si>
+  <si>
+    <t>11:16</t>
   </si>
 </sst>
 </file>
@@ -1823,7 +1829,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G1171"/>
+  <dimension ref="A1:G1175"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
@@ -28753,6 +28759,98 @@
         <v>11</v>
       </c>
     </row>
+    <row r="1172" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1172" s="5" t="s">
+        <v>463</v>
+      </c>
+      <c r="B1172" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1172" s="5" t="s">
+        <v>464</v>
+      </c>
+      <c r="D1172" s="5">
+        <v>12.3</v>
+      </c>
+      <c r="E1172" s="5">
+        <v>71</v>
+      </c>
+      <c r="F1172" s="5">
+        <v>14</v>
+      </c>
+      <c r="G1172" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1173" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1173" s="5" t="s">
+        <v>463</v>
+      </c>
+      <c r="B1173" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="C1173" s="5" t="s">
+        <v>464</v>
+      </c>
+      <c r="D1173" s="5">
+        <v>14.8</v>
+      </c>
+      <c r="E1173" s="5">
+        <v>63</v>
+      </c>
+      <c r="F1173" s="5">
+        <v>16</v>
+      </c>
+      <c r="G1173" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1174" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1174" s="5" t="s">
+        <v>463</v>
+      </c>
+      <c r="B1174" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="C1174" s="5" t="s">
+        <v>464</v>
+      </c>
+      <c r="D1174" s="5">
+        <v>16.9</v>
+      </c>
+      <c r="E1174" s="5">
+        <v>55</v>
+      </c>
+      <c r="F1174" s="5">
+        <v>17</v>
+      </c>
+      <c r="G1174" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1175" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1175" s="5" t="s">
+        <v>463</v>
+      </c>
+      <c r="B1175" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1175" s="5" t="s">
+        <v>464</v>
+      </c>
+      <c r="D1175" s="5">
+        <v>18.6</v>
+      </c>
+      <c r="E1175" s="5">
+        <v>50</v>
+      </c>
+      <c r="F1175" s="5">
+        <v>19</v>
+      </c>
+      <c r="G1175" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>

</xml_diff>

<commit_message>
📊 체감온도 기록: 2026-10-08 18:27 KST
</commit_message>
<xml_diff>
--- a/data/체감온도기록_2026.xlsx
+++ b/data/체감온도기록_2026.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4720" uniqueCount="465">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4748" uniqueCount="466">
   <si>
     <t>성동자이리버뷰 체감온도 기록</t>
   </si>
@@ -1409,6 +1409,9 @@
   </si>
   <si>
     <t>11:16</t>
+  </si>
+  <si>
+    <t>18:27</t>
   </si>
 </sst>
 </file>
@@ -1829,7 +1832,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G1175"/>
+  <dimension ref="A1:G1182"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
@@ -28851,6 +28854,167 @@
         <v>11</v>
       </c>
     </row>
+    <row r="1176" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1176" s="5" t="s">
+        <v>463</v>
+      </c>
+      <c r="B1176" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="C1176" s="5" t="s">
+        <v>465</v>
+      </c>
+      <c r="D1176" s="5">
+        <v>21.4</v>
+      </c>
+      <c r="E1176" s="5">
+        <v>45</v>
+      </c>
+      <c r="F1176" s="5">
+        <v>21</v>
+      </c>
+      <c r="G1176" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1177" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1177" s="5" t="s">
+        <v>463</v>
+      </c>
+      <c r="B1177" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="C1177" s="5" t="s">
+        <v>465</v>
+      </c>
+      <c r="D1177" s="5">
+        <v>22.4</v>
+      </c>
+      <c r="E1177" s="5">
+        <v>35</v>
+      </c>
+      <c r="F1177" s="5">
+        <v>21</v>
+      </c>
+      <c r="G1177" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1178" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1178" s="5" t="s">
+        <v>463</v>
+      </c>
+      <c r="B1178" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1178" s="5" t="s">
+        <v>465</v>
+      </c>
+      <c r="D1178" s="5">
+        <v>24.1</v>
+      </c>
+      <c r="E1178" s="5">
+        <v>34</v>
+      </c>
+      <c r="F1178" s="5">
+        <v>22</v>
+      </c>
+      <c r="G1178" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1179" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1179" s="5" t="s">
+        <v>463</v>
+      </c>
+      <c r="B1179" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="C1179" s="5" t="s">
+        <v>465</v>
+      </c>
+      <c r="D1179" s="5">
+        <v>24.6</v>
+      </c>
+      <c r="E1179" s="5">
+        <v>34</v>
+      </c>
+      <c r="F1179" s="5">
+        <v>23</v>
+      </c>
+      <c r="G1179" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1180" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1180" s="5" t="s">
+        <v>463</v>
+      </c>
+      <c r="B1180" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="C1180" s="5" t="s">
+        <v>465</v>
+      </c>
+      <c r="D1180" s="5">
+        <v>25.1</v>
+      </c>
+      <c r="E1180" s="5">
+        <v>31</v>
+      </c>
+      <c r="F1180" s="5">
+        <v>23</v>
+      </c>
+      <c r="G1180" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1181" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1181" s="5" t="s">
+        <v>463</v>
+      </c>
+      <c r="B1181" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1181" s="5" t="s">
+        <v>465</v>
+      </c>
+      <c r="D1181" s="5">
+        <v>24.9</v>
+      </c>
+      <c r="E1181" s="5">
+        <v>31</v>
+      </c>
+      <c r="F1181" s="5">
+        <v>23</v>
+      </c>
+      <c r="G1181" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1182" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1182" s="5" t="s">
+        <v>463</v>
+      </c>
+      <c r="B1182" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="C1182" s="5" t="s">
+        <v>465</v>
+      </c>
+      <c r="D1182" s="5">
+        <v>24.2</v>
+      </c>
+      <c r="E1182" s="5">
+        <v>32</v>
+      </c>
+      <c r="F1182" s="5">
+        <v>22</v>
+      </c>
+      <c r="G1182" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>

</xml_diff>

<commit_message>
📊 체감온도 기록: 2026-10-09 11:33 KST
</commit_message>
<xml_diff>
--- a/data/체감온도기록_2026.xlsx
+++ b/data/체감온도기록_2026.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4748" uniqueCount="466">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4764" uniqueCount="468">
   <si>
     <t>성동자이리버뷰 체감온도 기록</t>
   </si>
@@ -1412,6 +1412,12 @@
   </si>
   <si>
     <t>18:27</t>
+  </si>
+  <si>
+    <t>2026-10-09</t>
+  </si>
+  <si>
+    <t>11:33</t>
   </si>
 </sst>
 </file>
@@ -1832,7 +1838,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G1182"/>
+  <dimension ref="A1:G1186"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
@@ -29015,6 +29021,98 @@
         <v>11</v>
       </c>
     </row>
+    <row r="1183" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1183" s="5" t="s">
+        <v>466</v>
+      </c>
+      <c r="B1183" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1183" s="5" t="s">
+        <v>467</v>
+      </c>
+      <c r="D1183" s="5">
+        <v>13.5</v>
+      </c>
+      <c r="E1183" s="5">
+        <v>74</v>
+      </c>
+      <c r="F1183" s="5">
+        <v>15</v>
+      </c>
+      <c r="G1183" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1184" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1184" s="5" t="s">
+        <v>466</v>
+      </c>
+      <c r="B1184" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="C1184" s="5" t="s">
+        <v>467</v>
+      </c>
+      <c r="D1184" s="5">
+        <v>15.5</v>
+      </c>
+      <c r="E1184" s="5">
+        <v>68</v>
+      </c>
+      <c r="F1184" s="5">
+        <v>17</v>
+      </c>
+      <c r="G1184" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1185" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1185" s="5" t="s">
+        <v>466</v>
+      </c>
+      <c r="B1185" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="C1185" s="5" t="s">
+        <v>467</v>
+      </c>
+      <c r="D1185" s="5">
+        <v>17</v>
+      </c>
+      <c r="E1185" s="5">
+        <v>62</v>
+      </c>
+      <c r="F1185" s="5">
+        <v>18</v>
+      </c>
+      <c r="G1185" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1186" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1186" s="5" t="s">
+        <v>466</v>
+      </c>
+      <c r="B1186" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1186" s="5" t="s">
+        <v>467</v>
+      </c>
+      <c r="D1186" s="5">
+        <v>19.4</v>
+      </c>
+      <c r="E1186" s="5">
+        <v>55</v>
+      </c>
+      <c r="F1186" s="5">
+        <v>20</v>
+      </c>
+      <c r="G1186" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>

</xml_diff>

<commit_message>
📊 체감온도 기록: 2026-10-09 18:38 KST
</commit_message>
<xml_diff>
--- a/data/체감온도기록_2026.xlsx
+++ b/data/체감온도기록_2026.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4764" uniqueCount="468">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4792" uniqueCount="469">
   <si>
     <t>성동자이리버뷰 체감온도 기록</t>
   </si>
@@ -1418,6 +1418,9 @@
   </si>
   <si>
     <t>11:33</t>
+  </si>
+  <si>
+    <t>18:38</t>
   </si>
 </sst>
 </file>
@@ -1838,7 +1841,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G1186"/>
+  <dimension ref="A1:G1193"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
@@ -29113,6 +29116,167 @@
         <v>11</v>
       </c>
     </row>
+    <row r="1187" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1187" s="5" t="s">
+        <v>466</v>
+      </c>
+      <c r="B1187" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="C1187" s="5" t="s">
+        <v>468</v>
+      </c>
+      <c r="D1187" s="5">
+        <v>22</v>
+      </c>
+      <c r="E1187" s="5">
+        <v>47</v>
+      </c>
+      <c r="F1187" s="5">
+        <v>22</v>
+      </c>
+      <c r="G1187" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1188" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1188" s="5" t="s">
+        <v>466</v>
+      </c>
+      <c r="B1188" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="C1188" s="5" t="s">
+        <v>468</v>
+      </c>
+      <c r="D1188" s="5">
+        <v>22.5</v>
+      </c>
+      <c r="E1188" s="5">
+        <v>42</v>
+      </c>
+      <c r="F1188" s="5">
+        <v>22</v>
+      </c>
+      <c r="G1188" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1189" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1189" s="5" t="s">
+        <v>466</v>
+      </c>
+      <c r="B1189" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1189" s="5" t="s">
+        <v>468</v>
+      </c>
+      <c r="D1189" s="5">
+        <v>23.3</v>
+      </c>
+      <c r="E1189" s="5">
+        <v>39</v>
+      </c>
+      <c r="F1189" s="5">
+        <v>22</v>
+      </c>
+      <c r="G1189" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1190" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1190" s="5" t="s">
+        <v>466</v>
+      </c>
+      <c r="B1190" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="C1190" s="5" t="s">
+        <v>468</v>
+      </c>
+      <c r="D1190" s="5">
+        <v>25.4</v>
+      </c>
+      <c r="E1190" s="5">
+        <v>29</v>
+      </c>
+      <c r="F1190" s="5">
+        <v>23</v>
+      </c>
+      <c r="G1190" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1191" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1191" s="5" t="s">
+        <v>466</v>
+      </c>
+      <c r="B1191" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="C1191" s="5" t="s">
+        <v>468</v>
+      </c>
+      <c r="D1191" s="5">
+        <v>25.7</v>
+      </c>
+      <c r="E1191" s="5">
+        <v>27</v>
+      </c>
+      <c r="F1191" s="5">
+        <v>23</v>
+      </c>
+      <c r="G1191" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1192" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1192" s="5" t="s">
+        <v>466</v>
+      </c>
+      <c r="B1192" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1192" s="5" t="s">
+        <v>468</v>
+      </c>
+      <c r="D1192" s="5">
+        <v>25.4</v>
+      </c>
+      <c r="E1192" s="5">
+        <v>29</v>
+      </c>
+      <c r="F1192" s="5">
+        <v>23</v>
+      </c>
+      <c r="G1192" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1193" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1193" s="5" t="s">
+        <v>466</v>
+      </c>
+      <c r="B1193" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="C1193" s="5" t="s">
+        <v>468</v>
+      </c>
+      <c r="D1193" s="5">
+        <v>25</v>
+      </c>
+      <c r="E1193" s="5">
+        <v>30</v>
+      </c>
+      <c r="F1193" s="5">
+        <v>23</v>
+      </c>
+      <c r="G1193" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>

</xml_diff>

<commit_message>
📊 체감온도 기록: 2026-10-10 10:54 KST
</commit_message>
<xml_diff>
--- a/data/체감온도기록_2026.xlsx
+++ b/data/체감온도기록_2026.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4792" uniqueCount="469">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4808" uniqueCount="471">
   <si>
     <t>성동자이리버뷰 체감온도 기록</t>
   </si>
@@ -1421,6 +1421,12 @@
   </si>
   <si>
     <t>18:38</t>
+  </si>
+  <si>
+    <t>2026-10-10</t>
+  </si>
+  <si>
+    <t>10:54</t>
   </si>
 </sst>
 </file>
@@ -1841,7 +1847,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G1193"/>
+  <dimension ref="A1:G1197"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
@@ -29277,6 +29283,98 @@
         <v>11</v>
       </c>
     </row>
+    <row r="1194" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1194" s="5" t="s">
+        <v>469</v>
+      </c>
+      <c r="B1194" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1194" s="5" t="s">
+        <v>470</v>
+      </c>
+      <c r="D1194" s="5">
+        <v>14.1</v>
+      </c>
+      <c r="E1194" s="5">
+        <v>76</v>
+      </c>
+      <c r="F1194" s="5">
+        <v>16</v>
+      </c>
+      <c r="G1194" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1195" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1195" s="5" t="s">
+        <v>469</v>
+      </c>
+      <c r="B1195" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="C1195" s="5" t="s">
+        <v>470</v>
+      </c>
+      <c r="D1195" s="5">
+        <v>15.5</v>
+      </c>
+      <c r="E1195" s="5">
+        <v>70</v>
+      </c>
+      <c r="F1195" s="5">
+        <v>17</v>
+      </c>
+      <c r="G1195" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1196" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1196" s="5" t="s">
+        <v>469</v>
+      </c>
+      <c r="B1196" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="C1196" s="5" t="s">
+        <v>470</v>
+      </c>
+      <c r="D1196" s="5">
+        <v>17.7</v>
+      </c>
+      <c r="E1196" s="5">
+        <v>62</v>
+      </c>
+      <c r="F1196" s="5">
+        <v>18</v>
+      </c>
+      <c r="G1196" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1197" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1197" s="5" t="s">
+        <v>469</v>
+      </c>
+      <c r="B1197" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1197" s="5" t="s">
+        <v>470</v>
+      </c>
+      <c r="D1197" s="5">
+        <v>20.3</v>
+      </c>
+      <c r="E1197" s="5">
+        <v>54</v>
+      </c>
+      <c r="F1197" s="5">
+        <v>20</v>
+      </c>
+      <c r="G1197" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>

</xml_diff>

<commit_message>
📊 체감온도 기록: 2026-10-11 10:14 KST
</commit_message>
<xml_diff>
--- a/data/체감온도기록_2026.xlsx
+++ b/data/체감온도기록_2026.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4808" uniqueCount="471">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4820" uniqueCount="472">
   <si>
     <t>성동자이리버뷰 체감온도 기록</t>
   </si>
@@ -1427,6 +1427,9 @@
   </si>
   <si>
     <t>10:54</t>
+  </si>
+  <si>
+    <t>2026-10-11</t>
   </si>
 </sst>
 </file>
@@ -1847,7 +1850,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G1197"/>
+  <dimension ref="A1:G1200"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
@@ -29375,6 +29378,75 @@
         <v>11</v>
       </c>
     </row>
+    <row r="1198" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1198" s="5" t="s">
+        <v>471</v>
+      </c>
+      <c r="B1198" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1198" s="5" t="s">
+        <v>260</v>
+      </c>
+      <c r="D1198" s="5">
+        <v>16.2</v>
+      </c>
+      <c r="E1198" s="5">
+        <v>66</v>
+      </c>
+      <c r="F1198" s="5">
+        <v>17</v>
+      </c>
+      <c r="G1198" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1199" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1199" s="5" t="s">
+        <v>471</v>
+      </c>
+      <c r="B1199" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="C1199" s="5" t="s">
+        <v>260</v>
+      </c>
+      <c r="D1199" s="5">
+        <v>18</v>
+      </c>
+      <c r="E1199" s="5">
+        <v>61</v>
+      </c>
+      <c r="F1199" s="5">
+        <v>19</v>
+      </c>
+      <c r="G1199" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1200" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1200" s="5" t="s">
+        <v>471</v>
+      </c>
+      <c r="B1200" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="C1200" s="5" t="s">
+        <v>260</v>
+      </c>
+      <c r="D1200" s="5">
+        <v>20</v>
+      </c>
+      <c r="E1200" s="5">
+        <v>56</v>
+      </c>
+      <c r="F1200" s="5">
+        <v>20</v>
+      </c>
+      <c r="G1200" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>

</xml_diff>

<commit_message>
📊 체감온도 기록: 2026-10-11 16:48 KST
</commit_message>
<xml_diff>
--- a/data/체감온도기록_2026.xlsx
+++ b/data/체감온도기록_2026.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4820" uniqueCount="472">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4848" uniqueCount="472">
   <si>
     <t>성동자이리버뷰 체감온도 기록</t>
   </si>
@@ -1850,7 +1850,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G1200"/>
+  <dimension ref="A1:G1207"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
@@ -29447,6 +29447,167 @@
         <v>11</v>
       </c>
     </row>
+    <row r="1201" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1201" s="5" t="s">
+        <v>471</v>
+      </c>
+      <c r="B1201" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1201" s="5" t="s">
+        <v>179</v>
+      </c>
+      <c r="D1201" s="5">
+        <v>22.4</v>
+      </c>
+      <c r="E1201" s="5">
+        <v>49</v>
+      </c>
+      <c r="F1201" s="5">
+        <v>22</v>
+      </c>
+      <c r="G1201" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1202" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1202" s="5" t="s">
+        <v>471</v>
+      </c>
+      <c r="B1202" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="C1202" s="5" t="s">
+        <v>179</v>
+      </c>
+      <c r="D1202" s="5">
+        <v>24.3</v>
+      </c>
+      <c r="E1202" s="5">
+        <v>43</v>
+      </c>
+      <c r="F1202" s="5">
+        <v>23</v>
+      </c>
+      <c r="G1202" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1203" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1203" s="5" t="s">
+        <v>471</v>
+      </c>
+      <c r="B1203" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="C1203" s="5" t="s">
+        <v>179</v>
+      </c>
+      <c r="D1203" s="5">
+        <v>25.9</v>
+      </c>
+      <c r="E1203" s="5">
+        <v>40</v>
+      </c>
+      <c r="F1203" s="5">
+        <v>25</v>
+      </c>
+      <c r="G1203" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1204" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1204" s="5" t="s">
+        <v>471</v>
+      </c>
+      <c r="B1204" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1204" s="5" t="s">
+        <v>179</v>
+      </c>
+      <c r="D1204" s="5">
+        <v>27.8</v>
+      </c>
+      <c r="E1204" s="5">
+        <v>36</v>
+      </c>
+      <c r="F1204" s="5">
+        <v>26</v>
+      </c>
+      <c r="G1204" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1205" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1205" s="5" t="s">
+        <v>471</v>
+      </c>
+      <c r="B1205" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="C1205" s="5" t="s">
+        <v>179</v>
+      </c>
+      <c r="D1205" s="5">
+        <v>27.8</v>
+      </c>
+      <c r="E1205" s="5">
+        <v>37</v>
+      </c>
+      <c r="F1205" s="5">
+        <v>26</v>
+      </c>
+      <c r="G1205" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1206" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1206" s="5" t="s">
+        <v>471</v>
+      </c>
+      <c r="B1206" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="C1206" s="5" t="s">
+        <v>179</v>
+      </c>
+      <c r="D1206" s="5">
+        <v>27.6</v>
+      </c>
+      <c r="E1206" s="5">
+        <v>39</v>
+      </c>
+      <c r="F1206" s="5">
+        <v>26</v>
+      </c>
+      <c r="G1206" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1207" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1207" s="5" t="s">
+        <v>471</v>
+      </c>
+      <c r="B1207" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1207" s="5" t="s">
+        <v>179</v>
+      </c>
+      <c r="D1207" s="5">
+        <v>27.6</v>
+      </c>
+      <c r="E1207" s="5">
+        <v>39</v>
+      </c>
+      <c r="F1207" s="5">
+        <v>26</v>
+      </c>
+      <c r="G1207" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>

</xml_diff>

<commit_message>
📊 체감온도 기록: 2026-10-12 10:47 KST
</commit_message>
<xml_diff>
--- a/data/체감온도기록_2026.xlsx
+++ b/data/체감온도기록_2026.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4848" uniqueCount="472">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4864" uniqueCount="474">
   <si>
     <t>성동자이리버뷰 체감온도 기록</t>
   </si>
@@ -1430,6 +1430,12 @@
   </si>
   <si>
     <t>2026-10-11</t>
+  </si>
+  <si>
+    <t>2026-10-12</t>
+  </si>
+  <si>
+    <t>10:47</t>
   </si>
 </sst>
 </file>
@@ -1850,7 +1856,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G1207"/>
+  <dimension ref="A1:G1211"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
@@ -29608,6 +29614,98 @@
         <v>11</v>
       </c>
     </row>
+    <row r="1208" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1208" s="5" t="s">
+        <v>472</v>
+      </c>
+      <c r="B1208" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1208" s="5" t="s">
+        <v>473</v>
+      </c>
+      <c r="D1208" s="5">
+        <v>20.2</v>
+      </c>
+      <c r="E1208" s="5">
+        <v>68</v>
+      </c>
+      <c r="F1208" s="5">
+        <v>21</v>
+      </c>
+      <c r="G1208" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1209" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1209" s="5" t="s">
+        <v>472</v>
+      </c>
+      <c r="B1209" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="C1209" s="5" t="s">
+        <v>473</v>
+      </c>
+      <c r="D1209" s="5">
+        <v>21.1</v>
+      </c>
+      <c r="E1209" s="5">
+        <v>66</v>
+      </c>
+      <c r="F1209" s="5">
+        <v>22</v>
+      </c>
+      <c r="G1209" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1210" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1210" s="5" t="s">
+        <v>472</v>
+      </c>
+      <c r="B1210" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="C1210" s="5" t="s">
+        <v>473</v>
+      </c>
+      <c r="D1210" s="5">
+        <v>22</v>
+      </c>
+      <c r="E1210" s="5">
+        <v>63</v>
+      </c>
+      <c r="F1210" s="5">
+        <v>23</v>
+      </c>
+      <c r="G1210" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1211" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1211" s="5" t="s">
+        <v>472</v>
+      </c>
+      <c r="B1211" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1211" s="5" t="s">
+        <v>473</v>
+      </c>
+      <c r="D1211" s="5">
+        <v>24.1</v>
+      </c>
+      <c r="E1211" s="5">
+        <v>59</v>
+      </c>
+      <c r="F1211" s="5">
+        <v>25</v>
+      </c>
+      <c r="G1211" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>

</xml_diff>

<commit_message>
📊 체감온도 기록: 2026-10-12 18:45 KST
</commit_message>
<xml_diff>
--- a/data/체감온도기록_2026.xlsx
+++ b/data/체감온도기록_2026.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4864" uniqueCount="474">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4892" uniqueCount="475">
   <si>
     <t>성동자이리버뷰 체감온도 기록</t>
   </si>
@@ -1436,6 +1436,9 @@
   </si>
   <si>
     <t>10:47</t>
+  </si>
+  <si>
+    <t>18:45</t>
   </si>
 </sst>
 </file>
@@ -1856,7 +1859,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G1211"/>
+  <dimension ref="A1:G1218"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
@@ -29706,6 +29709,167 @@
         <v>11</v>
       </c>
     </row>
+    <row r="1212" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1212" s="5" t="s">
+        <v>472</v>
+      </c>
+      <c r="B1212" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="C1212" s="5" t="s">
+        <v>474</v>
+      </c>
+      <c r="D1212" s="5">
+        <v>25.7</v>
+      </c>
+      <c r="E1212" s="5">
+        <v>56</v>
+      </c>
+      <c r="F1212" s="5">
+        <v>26</v>
+      </c>
+      <c r="G1212" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1213" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1213" s="5" t="s">
+        <v>472</v>
+      </c>
+      <c r="B1213" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="C1213" s="5" t="s">
+        <v>474</v>
+      </c>
+      <c r="D1213" s="5">
+        <v>27.3</v>
+      </c>
+      <c r="E1213" s="5">
+        <v>51</v>
+      </c>
+      <c r="F1213" s="5">
+        <v>27</v>
+      </c>
+      <c r="G1213" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1214" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1214" s="5" t="s">
+        <v>472</v>
+      </c>
+      <c r="B1214" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1214" s="5" t="s">
+        <v>474</v>
+      </c>
+      <c r="D1214" s="5">
+        <v>26.7</v>
+      </c>
+      <c r="E1214" s="5">
+        <v>52</v>
+      </c>
+      <c r="F1214" s="5">
+        <v>27</v>
+      </c>
+      <c r="G1214" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1215" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1215" s="5" t="s">
+        <v>472</v>
+      </c>
+      <c r="B1215" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="C1215" s="5" t="s">
+        <v>474</v>
+      </c>
+      <c r="D1215" s="5">
+        <v>27.8</v>
+      </c>
+      <c r="E1215" s="5">
+        <v>49</v>
+      </c>
+      <c r="F1215" s="5">
+        <v>27</v>
+      </c>
+      <c r="G1215" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1216" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1216" s="5" t="s">
+        <v>472</v>
+      </c>
+      <c r="B1216" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="C1216" s="5" t="s">
+        <v>474</v>
+      </c>
+      <c r="D1216" s="5">
+        <v>27.8</v>
+      </c>
+      <c r="E1216" s="5">
+        <v>49</v>
+      </c>
+      <c r="F1216" s="5">
+        <v>27</v>
+      </c>
+      <c r="G1216" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1217" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1217" s="5" t="s">
+        <v>472</v>
+      </c>
+      <c r="B1217" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1217" s="5" t="s">
+        <v>474</v>
+      </c>
+      <c r="D1217" s="5">
+        <v>27.9</v>
+      </c>
+      <c r="E1217" s="5">
+        <v>48</v>
+      </c>
+      <c r="F1217" s="5">
+        <v>27</v>
+      </c>
+      <c r="G1217" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1218" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1218" s="5" t="s">
+        <v>472</v>
+      </c>
+      <c r="B1218" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="C1218" s="5" t="s">
+        <v>474</v>
+      </c>
+      <c r="D1218" s="5">
+        <v>26.9</v>
+      </c>
+      <c r="E1218" s="5">
+        <v>54</v>
+      </c>
+      <c r="F1218" s="5">
+        <v>27</v>
+      </c>
+      <c r="G1218" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>

</xml_diff>

<commit_message>
📊 체감온도 기록: 2026-10-13 12:10 KST
</commit_message>
<xml_diff>
--- a/data/체감온도기록_2026.xlsx
+++ b/data/체감온도기록_2026.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4892" uniqueCount="475">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4912" uniqueCount="477">
   <si>
     <t>성동자이리버뷰 체감온도 기록</t>
   </si>
@@ -1439,6 +1439,12 @@
   </si>
   <si>
     <t>18:45</t>
+  </si>
+  <si>
+    <t>2026-10-13</t>
+  </si>
+  <si>
+    <t>12:10</t>
   </si>
 </sst>
 </file>
@@ -1859,7 +1865,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G1218"/>
+  <dimension ref="A1:G1223"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
@@ -29870,6 +29876,121 @@
         <v>11</v>
       </c>
     </row>
+    <row r="1219" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1219" s="5" t="s">
+        <v>475</v>
+      </c>
+      <c r="B1219" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1219" s="5" t="s">
+        <v>476</v>
+      </c>
+      <c r="D1219" s="5">
+        <v>17.5</v>
+      </c>
+      <c r="E1219" s="5">
+        <v>92</v>
+      </c>
+      <c r="F1219" s="5">
+        <v>20</v>
+      </c>
+      <c r="G1219" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1220" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1220" s="5" t="s">
+        <v>475</v>
+      </c>
+      <c r="B1220" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="C1220" s="5" t="s">
+        <v>476</v>
+      </c>
+      <c r="D1220" s="5">
+        <v>16.2</v>
+      </c>
+      <c r="E1220" s="5">
+        <v>87</v>
+      </c>
+      <c r="F1220" s="5">
+        <v>19</v>
+      </c>
+      <c r="G1220" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1221" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1221" s="5" t="s">
+        <v>475</v>
+      </c>
+      <c r="B1221" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="C1221" s="5" t="s">
+        <v>476</v>
+      </c>
+      <c r="D1221" s="5">
+        <v>16.3</v>
+      </c>
+      <c r="E1221" s="5">
+        <v>90</v>
+      </c>
+      <c r="F1221" s="5">
+        <v>19</v>
+      </c>
+      <c r="G1221" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1222" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1222" s="5" t="s">
+        <v>475</v>
+      </c>
+      <c r="B1222" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1222" s="5" t="s">
+        <v>476</v>
+      </c>
+      <c r="D1222" s="5">
+        <v>17.1</v>
+      </c>
+      <c r="E1222" s="5">
+        <v>82</v>
+      </c>
+      <c r="F1222" s="5">
+        <v>19</v>
+      </c>
+      <c r="G1222" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1223" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1223" s="5" t="s">
+        <v>475</v>
+      </c>
+      <c r="B1223" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="C1223" s="5" t="s">
+        <v>476</v>
+      </c>
+      <c r="D1223" s="5">
+        <v>17.5</v>
+      </c>
+      <c r="E1223" s="5">
+        <v>81</v>
+      </c>
+      <c r="F1223" s="5">
+        <v>19</v>
+      </c>
+      <c r="G1223" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>

</xml_diff>

<commit_message>
📊 체감온도 기록: 2026-10-13 20:06 KST
</commit_message>
<xml_diff>
--- a/data/체감온도기록_2026.xlsx
+++ b/data/체감온도기록_2026.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4912" uniqueCount="477">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4936" uniqueCount="477">
   <si>
     <t>성동자이리버뷰 체감온도 기록</t>
   </si>
@@ -1865,7 +1865,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G1223"/>
+  <dimension ref="A1:G1229"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
@@ -29991,6 +29991,144 @@
         <v>11</v>
       </c>
     </row>
+    <row r="1224" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1224" s="5" t="s">
+        <v>475</v>
+      </c>
+      <c r="B1224" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="C1224" s="5" t="s">
+        <v>273</v>
+      </c>
+      <c r="D1224" s="5">
+        <v>18.8</v>
+      </c>
+      <c r="E1224" s="5">
+        <v>74</v>
+      </c>
+      <c r="F1224" s="5">
+        <v>20</v>
+      </c>
+      <c r="G1224" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1225" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1225" s="5" t="s">
+        <v>475</v>
+      </c>
+      <c r="B1225" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1225" s="5" t="s">
+        <v>273</v>
+      </c>
+      <c r="D1225" s="5">
+        <v>19.6</v>
+      </c>
+      <c r="E1225" s="5">
+        <v>63</v>
+      </c>
+      <c r="F1225" s="5">
+        <v>20</v>
+      </c>
+      <c r="G1225" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1226" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1226" s="5" t="s">
+        <v>475</v>
+      </c>
+      <c r="B1226" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="C1226" s="5" t="s">
+        <v>273</v>
+      </c>
+      <c r="D1226" s="5">
+        <v>21</v>
+      </c>
+      <c r="E1226" s="5">
+        <v>61</v>
+      </c>
+      <c r="F1226" s="5">
+        <v>22</v>
+      </c>
+      <c r="G1226" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1227" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1227" s="5" t="s">
+        <v>475</v>
+      </c>
+      <c r="B1227" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="C1227" s="5" t="s">
+        <v>273</v>
+      </c>
+      <c r="D1227" s="5">
+        <v>21.2</v>
+      </c>
+      <c r="E1227" s="5">
+        <v>56</v>
+      </c>
+      <c r="F1227" s="5">
+        <v>21</v>
+      </c>
+      <c r="G1227" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1228" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1228" s="5" t="s">
+        <v>475</v>
+      </c>
+      <c r="B1228" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1228" s="5" t="s">
+        <v>273</v>
+      </c>
+      <c r="D1228" s="5">
+        <v>20.6</v>
+      </c>
+      <c r="E1228" s="5">
+        <v>58</v>
+      </c>
+      <c r="F1228" s="5">
+        <v>21</v>
+      </c>
+      <c r="G1228" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1229" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1229" s="5" t="s">
+        <v>475</v>
+      </c>
+      <c r="B1229" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="C1229" s="5" t="s">
+        <v>273</v>
+      </c>
+      <c r="D1229" s="5">
+        <v>19.9</v>
+      </c>
+      <c r="E1229" s="5">
+        <v>58</v>
+      </c>
+      <c r="F1229" s="5">
+        <v>20</v>
+      </c>
+      <c r="G1229" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>

</xml_diff>

<commit_message>
📊 체감온도 기록: 2026-10-14 10:23 KST
</commit_message>
<xml_diff>
--- a/data/체감온도기록_2026.xlsx
+++ b/data/체감온도기록_2026.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4936" uniqueCount="477">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4948" uniqueCount="478">
   <si>
     <t>성동자이리버뷰 체감온도 기록</t>
   </si>
@@ -1445,6 +1445,9 @@
   </si>
   <si>
     <t>12:10</t>
+  </si>
+  <si>
+    <t>2026-10-14</t>
   </si>
 </sst>
 </file>
@@ -1865,7 +1868,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G1229"/>
+  <dimension ref="A1:G1232"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
@@ -30129,6 +30132,75 @@
         <v>11</v>
       </c>
     </row>
+    <row r="1230" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1230" s="5" t="s">
+        <v>477</v>
+      </c>
+      <c r="B1230" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1230" s="5" t="s">
+        <v>369</v>
+      </c>
+      <c r="D1230" s="5">
+        <v>12.4</v>
+      </c>
+      <c r="E1230" s="5">
+        <v>32</v>
+      </c>
+      <c r="F1230" s="5">
+        <v>12</v>
+      </c>
+      <c r="G1230" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1231" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1231" s="5" t="s">
+        <v>477</v>
+      </c>
+      <c r="B1231" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="C1231" s="5" t="s">
+        <v>369</v>
+      </c>
+      <c r="D1231" s="5">
+        <v>13.8</v>
+      </c>
+      <c r="E1231" s="5">
+        <v>27</v>
+      </c>
+      <c r="F1231" s="5">
+        <v>12</v>
+      </c>
+      <c r="G1231" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1232" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1232" s="5" t="s">
+        <v>477</v>
+      </c>
+      <c r="B1232" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="C1232" s="5" t="s">
+        <v>369</v>
+      </c>
+      <c r="D1232" s="5">
+        <v>14.7</v>
+      </c>
+      <c r="E1232" s="5">
+        <v>23</v>
+      </c>
+      <c r="F1232" s="5">
+        <v>13</v>
+      </c>
+      <c r="G1232" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>

</xml_diff>

<commit_message>
📊 체감온도 기록: 2026-10-14 15:42 KST
</commit_message>
<xml_diff>
--- a/data/체감온도기록_2026.xlsx
+++ b/data/체감온도기록_2026.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4948" uniqueCount="478">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4972" uniqueCount="478">
   <si>
     <t>성동자이리버뷰 체감온도 기록</t>
   </si>
@@ -1868,7 +1868,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G1232"/>
+  <dimension ref="A1:G1238"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
@@ -30201,6 +30201,144 @@
         <v>11</v>
       </c>
     </row>
+    <row r="1233" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1233" s="5" t="s">
+        <v>477</v>
+      </c>
+      <c r="B1233" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1233" s="5" t="s">
+        <v>409</v>
+      </c>
+      <c r="D1233" s="5">
+        <v>15.5</v>
+      </c>
+      <c r="E1233" s="5">
+        <v>22</v>
+      </c>
+      <c r="F1233" s="5">
+        <v>14</v>
+      </c>
+      <c r="G1233" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1234" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1234" s="5" t="s">
+        <v>477</v>
+      </c>
+      <c r="B1234" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="C1234" s="5" t="s">
+        <v>409</v>
+      </c>
+      <c r="D1234" s="5">
+        <v>16.5</v>
+      </c>
+      <c r="E1234" s="5">
+        <v>21</v>
+      </c>
+      <c r="F1234" s="5">
+        <v>14</v>
+      </c>
+      <c r="G1234" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1235" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1235" s="5" t="s">
+        <v>477</v>
+      </c>
+      <c r="B1235" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="C1235" s="5" t="s">
+        <v>409</v>
+      </c>
+      <c r="D1235" s="5">
+        <v>17.2</v>
+      </c>
+      <c r="E1235" s="5">
+        <v>21</v>
+      </c>
+      <c r="F1235" s="5">
+        <v>15</v>
+      </c>
+      <c r="G1235" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1236" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1236" s="5" t="s">
+        <v>477</v>
+      </c>
+      <c r="B1236" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1236" s="5" t="s">
+        <v>409</v>
+      </c>
+      <c r="D1236" s="5">
+        <v>18.8</v>
+      </c>
+      <c r="E1236" s="5">
+        <v>20</v>
+      </c>
+      <c r="F1236" s="5">
+        <v>16</v>
+      </c>
+      <c r="G1236" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1237" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1237" s="5" t="s">
+        <v>477</v>
+      </c>
+      <c r="B1237" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="C1237" s="5" t="s">
+        <v>409</v>
+      </c>
+      <c r="D1237" s="5">
+        <v>18.5</v>
+      </c>
+      <c r="E1237" s="5">
+        <v>21</v>
+      </c>
+      <c r="F1237" s="5">
+        <v>16</v>
+      </c>
+      <c r="G1237" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1238" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1238" s="5" t="s">
+        <v>477</v>
+      </c>
+      <c r="B1238" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="C1238" s="5" t="s">
+        <v>409</v>
+      </c>
+      <c r="D1238" s="5">
+        <v>18.9</v>
+      </c>
+      <c r="E1238" s="5">
+        <v>24</v>
+      </c>
+      <c r="F1238" s="5">
+        <v>17</v>
+      </c>
+      <c r="G1238" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>

</xml_diff>

<commit_message>
📊 체감온도 기록: 2026-10-14 21:24 KST
</commit_message>
<xml_diff>
--- a/data/체감온도기록_2026.xlsx
+++ b/data/체감온도기록_2026.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4972" uniqueCount="478">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4980" uniqueCount="479">
   <si>
     <t>성동자이리버뷰 체감온도 기록</t>
   </si>
@@ -1448,6 +1448,9 @@
   </si>
   <si>
     <t>2026-10-14</t>
+  </si>
+  <si>
+    <t>21:24</t>
   </si>
 </sst>
 </file>
@@ -1868,7 +1871,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G1238"/>
+  <dimension ref="A1:G1240"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
@@ -30339,6 +30342,52 @@
         <v>11</v>
       </c>
     </row>
+    <row r="1239" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1239" s="5" t="s">
+        <v>477</v>
+      </c>
+      <c r="B1239" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1239" s="5" t="s">
+        <v>478</v>
+      </c>
+      <c r="D1239" s="5">
+        <v>19.1</v>
+      </c>
+      <c r="E1239" s="5">
+        <v>26</v>
+      </c>
+      <c r="F1239" s="5">
+        <v>17</v>
+      </c>
+      <c r="G1239" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1240" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1240" s="5" t="s">
+        <v>477</v>
+      </c>
+      <c r="B1240" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="C1240" s="5" t="s">
+        <v>478</v>
+      </c>
+      <c r="D1240" s="5">
+        <v>18.6</v>
+      </c>
+      <c r="E1240" s="5">
+        <v>30</v>
+      </c>
+      <c r="F1240" s="5">
+        <v>17</v>
+      </c>
+      <c r="G1240" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>

</xml_diff>

<commit_message>
📊 체감온도 기록: 2026-10-15 09:52 KST
</commit_message>
<xml_diff>
--- a/data/체감온도기록_2026.xlsx
+++ b/data/체감온도기록_2026.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4980" uniqueCount="479">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4992" uniqueCount="480">
   <si>
     <t>성동자이리버뷰 체감온도 기록</t>
   </si>
@@ -1451,6 +1451,9 @@
   </si>
   <si>
     <t>21:24</t>
+  </si>
+  <si>
+    <t>2026-10-15</t>
   </si>
 </sst>
 </file>
@@ -1871,7 +1874,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G1240"/>
+  <dimension ref="A1:G1243"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
@@ -30388,6 +30391,75 @@
         <v>11</v>
       </c>
     </row>
+    <row r="1241" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1241" s="5" t="s">
+        <v>479</v>
+      </c>
+      <c r="B1241" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1241" s="5" t="s">
+        <v>415</v>
+      </c>
+      <c r="D1241" s="5">
+        <v>13.2</v>
+      </c>
+      <c r="E1241" s="5">
+        <v>72</v>
+      </c>
+      <c r="F1241" s="5">
+        <v>15</v>
+      </c>
+      <c r="G1241" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1242" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1242" s="5" t="s">
+        <v>479</v>
+      </c>
+      <c r="B1242" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="C1242" s="5" t="s">
+        <v>415</v>
+      </c>
+      <c r="D1242" s="5">
+        <v>14.3</v>
+      </c>
+      <c r="E1242" s="5">
+        <v>64</v>
+      </c>
+      <c r="F1242" s="5">
+        <v>15</v>
+      </c>
+      <c r="G1242" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1243" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1243" s="5" t="s">
+        <v>479</v>
+      </c>
+      <c r="B1243" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="C1243" s="5" t="s">
+        <v>415</v>
+      </c>
+      <c r="D1243" s="5">
+        <v>14.9</v>
+      </c>
+      <c r="E1243" s="5">
+        <v>62</v>
+      </c>
+      <c r="F1243" s="5">
+        <v>16</v>
+      </c>
+      <c r="G1243" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>

</xml_diff>

<commit_message>
📊 체감온도 기록: 2026-10-15 15:27 KST
</commit_message>
<xml_diff>
--- a/data/체감온도기록_2026.xlsx
+++ b/data/체감온도기록_2026.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4992" uniqueCount="480">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5012" uniqueCount="481">
   <si>
     <t>성동자이리버뷰 체감온도 기록</t>
   </si>
@@ -1454,6 +1454,9 @@
   </si>
   <si>
     <t>2026-10-15</t>
+  </si>
+  <si>
+    <t>15:26</t>
   </si>
 </sst>
 </file>
@@ -1874,7 +1877,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G1243"/>
+  <dimension ref="A1:G1248"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
@@ -30460,6 +30463,121 @@
         <v>11</v>
       </c>
     </row>
+    <row r="1244" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1244" s="5" t="s">
+        <v>479</v>
+      </c>
+      <c r="B1244" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1244" s="5" t="s">
+        <v>480</v>
+      </c>
+      <c r="D1244" s="5">
+        <v>17</v>
+      </c>
+      <c r="E1244" s="5">
+        <v>57</v>
+      </c>
+      <c r="F1244" s="5">
+        <v>17</v>
+      </c>
+      <c r="G1244" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1245" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1245" s="5" t="s">
+        <v>479</v>
+      </c>
+      <c r="B1245" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="C1245" s="5" t="s">
+        <v>480</v>
+      </c>
+      <c r="D1245" s="5">
+        <v>18.8</v>
+      </c>
+      <c r="E1245" s="5">
+        <v>51</v>
+      </c>
+      <c r="F1245" s="5">
+        <v>19</v>
+      </c>
+      <c r="G1245" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1246" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1246" s="5" t="s">
+        <v>479</v>
+      </c>
+      <c r="B1246" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="C1246" s="5" t="s">
+        <v>480</v>
+      </c>
+      <c r="D1246" s="5">
+        <v>20.2</v>
+      </c>
+      <c r="E1246" s="5">
+        <v>47</v>
+      </c>
+      <c r="F1246" s="5">
+        <v>20</v>
+      </c>
+      <c r="G1246" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1247" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1247" s="5" t="s">
+        <v>479</v>
+      </c>
+      <c r="B1247" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1247" s="5" t="s">
+        <v>480</v>
+      </c>
+      <c r="D1247" s="5">
+        <v>20.3</v>
+      </c>
+      <c r="E1247" s="5">
+        <v>50</v>
+      </c>
+      <c r="F1247" s="5">
+        <v>20</v>
+      </c>
+      <c r="G1247" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1248" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1248" s="5" t="s">
+        <v>479</v>
+      </c>
+      <c r="B1248" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="C1248" s="5" t="s">
+        <v>480</v>
+      </c>
+      <c r="D1248" s="5">
+        <v>20</v>
+      </c>
+      <c r="E1248" s="5">
+        <v>53</v>
+      </c>
+      <c r="F1248" s="5">
+        <v>20</v>
+      </c>
+      <c r="G1248" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>

</xml_diff>

<commit_message>
📊 체감온도 기록: 2026-10-15 21:07 KST
</commit_message>
<xml_diff>
--- a/data/체감온도기록_2026.xlsx
+++ b/data/체감온도기록_2026.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5012" uniqueCount="481">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5024" uniqueCount="482">
   <si>
     <t>성동자이리버뷰 체감온도 기록</t>
   </si>
@@ -1457,6 +1457,9 @@
   </si>
   <si>
     <t>15:26</t>
+  </si>
+  <si>
+    <t>21:07</t>
   </si>
 </sst>
 </file>
@@ -1877,7 +1880,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G1248"/>
+  <dimension ref="A1:G1251"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
@@ -30578,6 +30581,75 @@
         <v>11</v>
       </c>
     </row>
+    <row r="1249" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1249" s="5" t="s">
+        <v>479</v>
+      </c>
+      <c r="B1249" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="C1249" s="5" t="s">
+        <v>481</v>
+      </c>
+      <c r="D1249" s="5">
+        <v>20.3</v>
+      </c>
+      <c r="E1249" s="5">
+        <v>53</v>
+      </c>
+      <c r="F1249" s="5">
+        <v>20</v>
+      </c>
+      <c r="G1249" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1250" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1250" s="5" t="s">
+        <v>479</v>
+      </c>
+      <c r="B1250" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1250" s="5" t="s">
+        <v>481</v>
+      </c>
+      <c r="D1250" s="5">
+        <v>20.3</v>
+      </c>
+      <c r="E1250" s="5">
+        <v>53</v>
+      </c>
+      <c r="F1250" s="5">
+        <v>20</v>
+      </c>
+      <c r="G1250" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1251" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1251" s="5" t="s">
+        <v>479</v>
+      </c>
+      <c r="B1251" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="C1251" s="5" t="s">
+        <v>481</v>
+      </c>
+      <c r="D1251" s="5">
+        <v>19.9</v>
+      </c>
+      <c r="E1251" s="5">
+        <v>56</v>
+      </c>
+      <c r="F1251" s="5">
+        <v>20</v>
+      </c>
+      <c r="G1251" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>

</xml_diff>

<commit_message>
📊 체감온도 기록: 2026-10-16 09:45 KST
</commit_message>
<xml_diff>
--- a/data/체감온도기록_2026.xlsx
+++ b/data/체감온도기록_2026.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5024" uniqueCount="482">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5036" uniqueCount="484">
   <si>
     <t>성동자이리버뷰 체감온도 기록</t>
   </si>
@@ -1460,6 +1460,12 @@
   </si>
   <si>
     <t>21:07</t>
+  </si>
+  <si>
+    <t>2026-10-16</t>
+  </si>
+  <si>
+    <t>09:45</t>
   </si>
 </sst>
 </file>
@@ -1880,7 +1886,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G1251"/>
+  <dimension ref="A1:G1254"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
@@ -30650,6 +30656,75 @@
         <v>11</v>
       </c>
     </row>
+    <row r="1252" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1252" s="5" t="s">
+        <v>482</v>
+      </c>
+      <c r="B1252" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1252" s="5" t="s">
+        <v>483</v>
+      </c>
+      <c r="D1252" s="5">
+        <v>17.2</v>
+      </c>
+      <c r="E1252" s="5">
+        <v>70</v>
+      </c>
+      <c r="F1252" s="5">
+        <v>18</v>
+      </c>
+      <c r="G1252" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1253" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1253" s="5" t="s">
+        <v>482</v>
+      </c>
+      <c r="B1253" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="C1253" s="5" t="s">
+        <v>483</v>
+      </c>
+      <c r="D1253" s="5">
+        <v>17.6</v>
+      </c>
+      <c r="E1253" s="5">
+        <v>67</v>
+      </c>
+      <c r="F1253" s="5">
+        <v>19</v>
+      </c>
+      <c r="G1253" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1254" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1254" s="5" t="s">
+        <v>482</v>
+      </c>
+      <c r="B1254" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="C1254" s="5" t="s">
+        <v>483</v>
+      </c>
+      <c r="D1254" s="5">
+        <v>18.3</v>
+      </c>
+      <c r="E1254" s="5">
+        <v>66</v>
+      </c>
+      <c r="F1254" s="5">
+        <v>19</v>
+      </c>
+      <c r="G1254" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>

</xml_diff>

<commit_message>
📊 체감온도 기록: 2026-10-16 15:22 KST
</commit_message>
<xml_diff>
--- a/data/체감온도기록_2026.xlsx
+++ b/data/체감온도기록_2026.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5036" uniqueCount="484">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5056" uniqueCount="485">
   <si>
     <t>성동자이리버뷰 체감온도 기록</t>
   </si>
@@ -1466,6 +1466,9 @@
   </si>
   <si>
     <t>09:45</t>
+  </si>
+  <si>
+    <t>15:22</t>
   </si>
 </sst>
 </file>
@@ -1886,7 +1889,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G1254"/>
+  <dimension ref="A1:G1259"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
@@ -30725,6 +30728,121 @@
         <v>11</v>
       </c>
     </row>
+    <row r="1255" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1255" s="5" t="s">
+        <v>482</v>
+      </c>
+      <c r="B1255" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1255" s="5" t="s">
+        <v>484</v>
+      </c>
+      <c r="D1255" s="5">
+        <v>19.1</v>
+      </c>
+      <c r="E1255" s="5">
+        <v>64</v>
+      </c>
+      <c r="F1255" s="5">
+        <v>20</v>
+      </c>
+      <c r="G1255" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1256" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1256" s="5" t="s">
+        <v>482</v>
+      </c>
+      <c r="B1256" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="C1256" s="5" t="s">
+        <v>484</v>
+      </c>
+      <c r="D1256" s="5">
+        <v>20.3</v>
+      </c>
+      <c r="E1256" s="5">
+        <v>61</v>
+      </c>
+      <c r="F1256" s="5">
+        <v>21</v>
+      </c>
+      <c r="G1256" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1257" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1257" s="5" t="s">
+        <v>482</v>
+      </c>
+      <c r="B1257" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="C1257" s="5" t="s">
+        <v>484</v>
+      </c>
+      <c r="D1257" s="5">
+        <v>21.3</v>
+      </c>
+      <c r="E1257" s="5">
+        <v>61</v>
+      </c>
+      <c r="F1257" s="5">
+        <v>22</v>
+      </c>
+      <c r="G1257" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1258" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1258" s="5" t="s">
+        <v>482</v>
+      </c>
+      <c r="B1258" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1258" s="5" t="s">
+        <v>484</v>
+      </c>
+      <c r="D1258" s="5">
+        <v>22.7</v>
+      </c>
+      <c r="E1258" s="5">
+        <v>59</v>
+      </c>
+      <c r="F1258" s="5">
+        <v>23</v>
+      </c>
+      <c r="G1258" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1259" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1259" s="5" t="s">
+        <v>482</v>
+      </c>
+      <c r="B1259" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="C1259" s="5" t="s">
+        <v>484</v>
+      </c>
+      <c r="D1259" s="5">
+        <v>23.2</v>
+      </c>
+      <c r="E1259" s="5">
+        <v>54</v>
+      </c>
+      <c r="F1259" s="5">
+        <v>23</v>
+      </c>
+      <c r="G1259" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>

</xml_diff>

<commit_message>
📊 체감온도 기록: 2026-10-16 20:54 KST
</commit_message>
<xml_diff>
--- a/data/체감온도기록_2026.xlsx
+++ b/data/체감온도기록_2026.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5056" uniqueCount="485">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5068" uniqueCount="486">
   <si>
     <t>성동자이리버뷰 체감온도 기록</t>
   </si>
@@ -1469,6 +1469,9 @@
   </si>
   <si>
     <t>15:22</t>
+  </si>
+  <si>
+    <t>20:54</t>
   </si>
 </sst>
 </file>
@@ -1889,7 +1892,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G1259"/>
+  <dimension ref="A1:G1262"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
@@ -30843,6 +30846,75 @@
         <v>11</v>
       </c>
     </row>
+    <row r="1260" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1260" s="5" t="s">
+        <v>482</v>
+      </c>
+      <c r="B1260" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="C1260" s="5" t="s">
+        <v>485</v>
+      </c>
+      <c r="D1260" s="5">
+        <v>23.4</v>
+      </c>
+      <c r="E1260" s="5">
+        <v>55</v>
+      </c>
+      <c r="F1260" s="5">
+        <v>24</v>
+      </c>
+      <c r="G1260" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1261" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1261" s="5" t="s">
+        <v>482</v>
+      </c>
+      <c r="B1261" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1261" s="5" t="s">
+        <v>485</v>
+      </c>
+      <c r="D1261" s="5">
+        <v>23.6</v>
+      </c>
+      <c r="E1261" s="5">
+        <v>52</v>
+      </c>
+      <c r="F1261" s="5">
+        <v>23</v>
+      </c>
+      <c r="G1261" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1262" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1262" s="5" t="s">
+        <v>482</v>
+      </c>
+      <c r="B1262" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="C1262" s="5" t="s">
+        <v>485</v>
+      </c>
+      <c r="D1262" s="5">
+        <v>23.6</v>
+      </c>
+      <c r="E1262" s="5">
+        <v>52</v>
+      </c>
+      <c r="F1262" s="5">
+        <v>23</v>
+      </c>
+      <c r="G1262" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>

</xml_diff>

<commit_message>
📊 체감온도 기록: 2026-10-17 09:46 KST
</commit_message>
<xml_diff>
--- a/data/체감온도기록_2026.xlsx
+++ b/data/체감온도기록_2026.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5068" uniqueCount="486">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5080" uniqueCount="488">
   <si>
     <t>성동자이리버뷰 체감온도 기록</t>
   </si>
@@ -1472,6 +1472,12 @@
   </si>
   <si>
     <t>20:54</t>
+  </si>
+  <si>
+    <t>2026-10-17</t>
+  </si>
+  <si>
+    <t>09:46</t>
   </si>
 </sst>
 </file>
@@ -1892,7 +1898,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G1262"/>
+  <dimension ref="A1:G1265"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
@@ -30915,6 +30921,75 @@
         <v>11</v>
       </c>
     </row>
+    <row r="1263" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1263" s="5" t="s">
+        <v>486</v>
+      </c>
+      <c r="B1263" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1263" s="5" t="s">
+        <v>487</v>
+      </c>
+      <c r="D1263" s="5">
+        <v>14.8</v>
+      </c>
+      <c r="E1263" s="5">
+        <v>87</v>
+      </c>
+      <c r="F1263" s="5">
+        <v>17</v>
+      </c>
+      <c r="G1263" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1264" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1264" s="5" t="s">
+        <v>486</v>
+      </c>
+      <c r="B1264" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="C1264" s="5" t="s">
+        <v>487</v>
+      </c>
+      <c r="D1264" s="5">
+        <v>16.4</v>
+      </c>
+      <c r="E1264" s="5">
+        <v>79</v>
+      </c>
+      <c r="F1264" s="5">
+        <v>18</v>
+      </c>
+      <c r="G1264" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1265" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1265" s="5" t="s">
+        <v>486</v>
+      </c>
+      <c r="B1265" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="C1265" s="5" t="s">
+        <v>487</v>
+      </c>
+      <c r="D1265" s="5">
+        <v>18.6</v>
+      </c>
+      <c r="E1265" s="5">
+        <v>67</v>
+      </c>
+      <c r="F1265" s="5">
+        <v>20</v>
+      </c>
+      <c r="G1265" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>

</xml_diff>

<commit_message>
📊 체감온도 기록: 2026-10-17 15:11 KST
</commit_message>
<xml_diff>
--- a/data/체감온도기록_2026.xlsx
+++ b/data/체감온도기록_2026.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5080" uniqueCount="488">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5100" uniqueCount="489">
   <si>
     <t>성동자이리버뷰 체감온도 기록</t>
   </si>
@@ -1478,6 +1478,9 @@
   </si>
   <si>
     <t>09:46</t>
+  </si>
+  <si>
+    <t>15:11</t>
   </si>
 </sst>
 </file>
@@ -1898,7 +1901,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G1265"/>
+  <dimension ref="A1:G1270"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
@@ -30990,6 +30993,121 @@
         <v>11</v>
       </c>
     </row>
+    <row r="1266" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1266" s="5" t="s">
+        <v>486</v>
+      </c>
+      <c r="B1266" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1266" s="5" t="s">
+        <v>488</v>
+      </c>
+      <c r="D1266" s="5">
+        <v>19.9</v>
+      </c>
+      <c r="E1266" s="5">
+        <v>59</v>
+      </c>
+      <c r="F1266" s="5">
+        <v>20</v>
+      </c>
+      <c r="G1266" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1267" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1267" s="5" t="s">
+        <v>486</v>
+      </c>
+      <c r="B1267" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="C1267" s="5" t="s">
+        <v>488</v>
+      </c>
+      <c r="D1267" s="5">
+        <v>21.6</v>
+      </c>
+      <c r="E1267" s="5">
+        <v>52</v>
+      </c>
+      <c r="F1267" s="5">
+        <v>22</v>
+      </c>
+      <c r="G1267" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1268" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1268" s="5" t="s">
+        <v>486</v>
+      </c>
+      <c r="B1268" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="C1268" s="5" t="s">
+        <v>488</v>
+      </c>
+      <c r="D1268" s="5">
+        <v>23.5</v>
+      </c>
+      <c r="E1268" s="5">
+        <v>46</v>
+      </c>
+      <c r="F1268" s="5">
+        <v>23</v>
+      </c>
+      <c r="G1268" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1269" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1269" s="5" t="s">
+        <v>486</v>
+      </c>
+      <c r="B1269" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1269" s="5" t="s">
+        <v>488</v>
+      </c>
+      <c r="D1269" s="5">
+        <v>24.1</v>
+      </c>
+      <c r="E1269" s="5">
+        <v>44</v>
+      </c>
+      <c r="F1269" s="5">
+        <v>23</v>
+      </c>
+      <c r="G1269" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1270" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1270" s="5" t="s">
+        <v>486</v>
+      </c>
+      <c r="B1270" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="C1270" s="5" t="s">
+        <v>488</v>
+      </c>
+      <c r="D1270" s="5">
+        <v>25.3</v>
+      </c>
+      <c r="E1270" s="5">
+        <v>41</v>
+      </c>
+      <c r="F1270" s="5">
+        <v>24</v>
+      </c>
+      <c r="G1270" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>

</xml_diff>

<commit_message>
📊 체감온도 기록: 2026-10-17 20:10 KST
</commit_message>
<xml_diff>
--- a/data/체감온도기록_2026.xlsx
+++ b/data/체감온도기록_2026.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5100" uniqueCount="489">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5112" uniqueCount="490">
   <si>
     <t>성동자이리버뷰 체감온도 기록</t>
   </si>
@@ -1481,6 +1481,9 @@
   </si>
   <si>
     <t>15:11</t>
+  </si>
+  <si>
+    <t>20:10</t>
   </si>
 </sst>
 </file>
@@ -1901,7 +1904,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G1270"/>
+  <dimension ref="A1:G1273"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
@@ -31108,6 +31111,75 @@
         <v>11</v>
       </c>
     </row>
+    <row r="1271" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1271" s="5" t="s">
+        <v>486</v>
+      </c>
+      <c r="B1271" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="C1271" s="5" t="s">
+        <v>489</v>
+      </c>
+      <c r="D1271" s="5">
+        <v>25.4</v>
+      </c>
+      <c r="E1271" s="5">
+        <v>41</v>
+      </c>
+      <c r="F1271" s="5">
+        <v>24</v>
+      </c>
+      <c r="G1271" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1272" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1272" s="5" t="s">
+        <v>486</v>
+      </c>
+      <c r="B1272" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1272" s="5" t="s">
+        <v>489</v>
+      </c>
+      <c r="D1272" s="5">
+        <v>25.1</v>
+      </c>
+      <c r="E1272" s="5">
+        <v>42</v>
+      </c>
+      <c r="F1272" s="5">
+        <v>24</v>
+      </c>
+      <c r="G1272" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1273" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1273" s="5" t="s">
+        <v>486</v>
+      </c>
+      <c r="B1273" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="C1273" s="5" t="s">
+        <v>489</v>
+      </c>
+      <c r="D1273" s="5">
+        <v>24.6</v>
+      </c>
+      <c r="E1273" s="5">
+        <v>40</v>
+      </c>
+      <c r="F1273" s="5">
+        <v>23</v>
+      </c>
+      <c r="G1273" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>

</xml_diff>

<commit_message>
📊 체감온도 기록: 2026-10-18 09:19 KST
</commit_message>
<xml_diff>
--- a/data/체감온도기록_2026.xlsx
+++ b/data/체감온도기록_2026.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5112" uniqueCount="490">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5120" uniqueCount="492">
   <si>
     <t>성동자이리버뷰 체감온도 기록</t>
   </si>
@@ -1484,6 +1484,12 @@
   </si>
   <si>
     <t>20:10</t>
+  </si>
+  <si>
+    <t>2026-10-18</t>
+  </si>
+  <si>
+    <t>09:19</t>
   </si>
 </sst>
 </file>
@@ -1904,7 +1910,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G1273"/>
+  <dimension ref="A1:G1275"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
@@ -31180,6 +31186,52 @@
         <v>11</v>
       </c>
     </row>
+    <row r="1274" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1274" s="5" t="s">
+        <v>490</v>
+      </c>
+      <c r="B1274" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1274" s="5" t="s">
+        <v>491</v>
+      </c>
+      <c r="D1274" s="5">
+        <v>20.1</v>
+      </c>
+      <c r="E1274" s="5">
+        <v>53</v>
+      </c>
+      <c r="F1274" s="5">
+        <v>20</v>
+      </c>
+      <c r="G1274" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1275" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1275" s="5" t="s">
+        <v>490</v>
+      </c>
+      <c r="B1275" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="C1275" s="5" t="s">
+        <v>491</v>
+      </c>
+      <c r="D1275" s="5">
+        <v>20.4</v>
+      </c>
+      <c r="E1275" s="5">
+        <v>53</v>
+      </c>
+      <c r="F1275" s="5">
+        <v>20</v>
+      </c>
+      <c r="G1275" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>

</xml_diff>

<commit_message>
📊 체감온도 기록: 2026-10-18 14:09 KST
</commit_message>
<xml_diff>
--- a/data/체감온도기록_2026.xlsx
+++ b/data/체감온도기록_2026.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5120" uniqueCount="492">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5140" uniqueCount="492">
   <si>
     <t>성동자이리버뷰 체감온도 기록</t>
   </si>
@@ -1910,7 +1910,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G1275"/>
+  <dimension ref="A1:G1280"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
@@ -31232,6 +31232,121 @@
         <v>11</v>
       </c>
     </row>
+    <row r="1276" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1276" s="5" t="s">
+        <v>490</v>
+      </c>
+      <c r="B1276" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="C1276" s="5" t="s">
+        <v>286</v>
+      </c>
+      <c r="D1276" s="5">
+        <v>20.6</v>
+      </c>
+      <c r="E1276" s="5">
+        <v>55</v>
+      </c>
+      <c r="F1276" s="5">
+        <v>21</v>
+      </c>
+      <c r="G1276" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1277" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1277" s="5" t="s">
+        <v>490</v>
+      </c>
+      <c r="B1277" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1277" s="5" t="s">
+        <v>286</v>
+      </c>
+      <c r="D1277" s="5">
+        <v>20.2</v>
+      </c>
+      <c r="E1277" s="5">
+        <v>65</v>
+      </c>
+      <c r="F1277" s="5">
+        <v>21</v>
+      </c>
+      <c r="G1277" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1278" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1278" s="5" t="s">
+        <v>490</v>
+      </c>
+      <c r="B1278" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="C1278" s="5" t="s">
+        <v>286</v>
+      </c>
+      <c r="D1278" s="5">
+        <v>20.4</v>
+      </c>
+      <c r="E1278" s="5">
+        <v>69</v>
+      </c>
+      <c r="F1278" s="5">
+        <v>22</v>
+      </c>
+      <c r="G1278" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1279" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1279" s="5" t="s">
+        <v>490</v>
+      </c>
+      <c r="B1279" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="C1279" s="5" t="s">
+        <v>286</v>
+      </c>
+      <c r="D1279" s="5">
+        <v>21.2</v>
+      </c>
+      <c r="E1279" s="5">
+        <v>72</v>
+      </c>
+      <c r="F1279" s="5">
+        <v>23</v>
+      </c>
+      <c r="G1279" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1280" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1280" s="5" t="s">
+        <v>490</v>
+      </c>
+      <c r="B1280" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1280" s="5" t="s">
+        <v>286</v>
+      </c>
+      <c r="D1280" s="5">
+        <v>20.4</v>
+      </c>
+      <c r="E1280" s="5">
+        <v>84</v>
+      </c>
+      <c r="F1280" s="5">
+        <v>23</v>
+      </c>
+      <c r="G1280" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>

</xml_diff>

<commit_message>
📊 체감온도 기록: 2026-10-18 18:56 KST
</commit_message>
<xml_diff>
--- a/data/체감온도기록_2026.xlsx
+++ b/data/체감온도기록_2026.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5140" uniqueCount="492">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5156" uniqueCount="492">
   <si>
     <t>성동자이리버뷰 체감온도 기록</t>
   </si>
@@ -1910,7 +1910,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G1280"/>
+  <dimension ref="A1:G1284"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
@@ -31347,6 +31347,98 @@
         <v>11</v>
       </c>
     </row>
+    <row r="1281" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1281" s="5" t="s">
+        <v>490</v>
+      </c>
+      <c r="B1281" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="C1281" s="5" t="s">
+        <v>378</v>
+      </c>
+      <c r="D1281" s="5">
+        <v>20.6</v>
+      </c>
+      <c r="E1281" s="5">
+        <v>91</v>
+      </c>
+      <c r="F1281" s="5">
+        <v>23</v>
+      </c>
+      <c r="G1281" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1282" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1282" s="5" t="s">
+        <v>490</v>
+      </c>
+      <c r="B1282" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="C1282" s="5" t="s">
+        <v>378</v>
+      </c>
+      <c r="D1282" s="5">
+        <v>20.5</v>
+      </c>
+      <c r="E1282" s="5">
+        <v>95</v>
+      </c>
+      <c r="F1282" s="5">
+        <v>23</v>
+      </c>
+      <c r="G1282" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1283" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1283" s="5" t="s">
+        <v>490</v>
+      </c>
+      <c r="B1283" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1283" s="5" t="s">
+        <v>378</v>
+      </c>
+      <c r="D1283" s="5">
+        <v>20.4</v>
+      </c>
+      <c r="E1283" s="5">
+        <v>94</v>
+      </c>
+      <c r="F1283" s="5">
+        <v>23</v>
+      </c>
+      <c r="G1283" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1284" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1284" s="5" t="s">
+        <v>490</v>
+      </c>
+      <c r="B1284" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="C1284" s="5" t="s">
+        <v>378</v>
+      </c>
+      <c r="D1284" s="5">
+        <v>19.5</v>
+      </c>
+      <c r="E1284" s="5">
+        <v>94</v>
+      </c>
+      <c r="F1284" s="5">
+        <v>22</v>
+      </c>
+      <c r="G1284" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>

</xml_diff>

<commit_message>
📊 체감온도 기록: 2026-10-19 09:31 KST
</commit_message>
<xml_diff>
--- a/data/체감온도기록_2026.xlsx
+++ b/data/체감온도기록_2026.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5156" uniqueCount="492">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5164" uniqueCount="494">
   <si>
     <t>성동자이리버뷰 체감온도 기록</t>
   </si>
@@ -1490,6 +1490,12 @@
   </si>
   <si>
     <t>09:19</t>
+  </si>
+  <si>
+    <t>2026-10-19</t>
+  </si>
+  <si>
+    <t>09:30</t>
   </si>
 </sst>
 </file>
@@ -1910,7 +1916,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G1284"/>
+  <dimension ref="A1:G1286"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
@@ -31439,6 +31445,52 @@
         <v>11</v>
       </c>
     </row>
+    <row r="1285" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1285" s="5" t="s">
+        <v>492</v>
+      </c>
+      <c r="B1285" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1285" s="5" t="s">
+        <v>493</v>
+      </c>
+      <c r="D1285" s="5">
+        <v>12.8</v>
+      </c>
+      <c r="E1285" s="5">
+        <v>86</v>
+      </c>
+      <c r="F1285" s="5">
+        <v>15</v>
+      </c>
+      <c r="G1285" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1286" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1286" s="5" t="s">
+        <v>492</v>
+      </c>
+      <c r="B1286" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="C1286" s="5" t="s">
+        <v>493</v>
+      </c>
+      <c r="D1286" s="5">
+        <v>13.6</v>
+      </c>
+      <c r="E1286" s="5">
+        <v>81</v>
+      </c>
+      <c r="F1286" s="5">
+        <v>16</v>
+      </c>
+      <c r="G1286" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>

</xml_diff>

<commit_message>
📊 체감온도 기록: 2026-10-19 20:15 KST
</commit_message>
<xml_diff>
--- a/data/체감온도기록_2026.xlsx
+++ b/data/체감온도기록_2026.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5164" uniqueCount="494">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5200" uniqueCount="495">
   <si>
     <t>성동자이리버뷰 체감온도 기록</t>
   </si>
@@ -1496,6 +1496,9 @@
   </si>
   <si>
     <t>09:30</t>
+  </si>
+  <si>
+    <t>20:15</t>
   </si>
 </sst>
 </file>
@@ -1916,7 +1919,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G1286"/>
+  <dimension ref="A1:G1295"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
@@ -31491,6 +31494,213 @@
         <v>11</v>
       </c>
     </row>
+    <row r="1287" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1287" s="5" t="s">
+        <v>492</v>
+      </c>
+      <c r="B1287" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="C1287" s="5" t="s">
+        <v>494</v>
+      </c>
+      <c r="D1287" s="5">
+        <v>14.6</v>
+      </c>
+      <c r="E1287" s="5">
+        <v>74</v>
+      </c>
+      <c r="F1287" s="5">
+        <v>16</v>
+      </c>
+      <c r="G1287" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1288" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1288" s="5" t="s">
+        <v>492</v>
+      </c>
+      <c r="B1288" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1288" s="5" t="s">
+        <v>494</v>
+      </c>
+      <c r="D1288" s="5">
+        <v>16.5</v>
+      </c>
+      <c r="E1288" s="5">
+        <v>67</v>
+      </c>
+      <c r="F1288" s="5">
+        <v>18</v>
+      </c>
+      <c r="G1288" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1289" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1289" s="5" t="s">
+        <v>492</v>
+      </c>
+      <c r="B1289" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="C1289" s="5" t="s">
+        <v>494</v>
+      </c>
+      <c r="D1289" s="5">
+        <v>17.2</v>
+      </c>
+      <c r="E1289" s="5">
+        <v>59</v>
+      </c>
+      <c r="F1289" s="5">
+        <v>18</v>
+      </c>
+      <c r="G1289" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1290" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1290" s="5" t="s">
+        <v>492</v>
+      </c>
+      <c r="B1290" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="C1290" s="5" t="s">
+        <v>494</v>
+      </c>
+      <c r="D1290" s="5">
+        <v>18.4</v>
+      </c>
+      <c r="E1290" s="5">
+        <v>48</v>
+      </c>
+      <c r="F1290" s="5">
+        <v>18</v>
+      </c>
+      <c r="G1290" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1291" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1291" s="5" t="s">
+        <v>492</v>
+      </c>
+      <c r="B1291" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1291" s="5" t="s">
+        <v>494</v>
+      </c>
+      <c r="D1291" s="5">
+        <v>18.6</v>
+      </c>
+      <c r="E1291" s="5">
+        <v>54</v>
+      </c>
+      <c r="F1291" s="5">
+        <v>19</v>
+      </c>
+      <c r="G1291" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1292" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1292" s="5" t="s">
+        <v>492</v>
+      </c>
+      <c r="B1292" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="C1292" s="5" t="s">
+        <v>494</v>
+      </c>
+      <c r="D1292" s="5">
+        <v>18.1</v>
+      </c>
+      <c r="E1292" s="5">
+        <v>50</v>
+      </c>
+      <c r="F1292" s="5">
+        <v>18</v>
+      </c>
+      <c r="G1292" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1293" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1293" s="5" t="s">
+        <v>492</v>
+      </c>
+      <c r="B1293" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="C1293" s="5" t="s">
+        <v>494</v>
+      </c>
+      <c r="D1293" s="5">
+        <v>17.9</v>
+      </c>
+      <c r="E1293" s="5">
+        <v>50</v>
+      </c>
+      <c r="F1293" s="5">
+        <v>18</v>
+      </c>
+      <c r="G1293" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1294" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1294" s="5" t="s">
+        <v>492</v>
+      </c>
+      <c r="B1294" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1294" s="5" t="s">
+        <v>494</v>
+      </c>
+      <c r="D1294" s="5">
+        <v>18.2</v>
+      </c>
+      <c r="E1294" s="5">
+        <v>51</v>
+      </c>
+      <c r="F1294" s="5">
+        <v>18</v>
+      </c>
+      <c r="G1294" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1295" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1295" s="5" t="s">
+        <v>492</v>
+      </c>
+      <c r="B1295" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="C1295" s="5" t="s">
+        <v>494</v>
+      </c>
+      <c r="D1295" s="5">
+        <v>17.9</v>
+      </c>
+      <c r="E1295" s="5">
+        <v>52</v>
+      </c>
+      <c r="F1295" s="5">
+        <v>18</v>
+      </c>
+      <c r="G1295" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>

</xml_diff>

<commit_message>
📊 체감온도 기록: 2026-10-20 10:16 KST
</commit_message>
<xml_diff>
--- a/data/체감온도기록_2026.xlsx
+++ b/data/체감온도기록_2026.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5200" uniqueCount="495">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5212" uniqueCount="496">
   <si>
     <t>성동자이리버뷰 체감온도 기록</t>
   </si>
@@ -1499,6 +1499,9 @@
   </si>
   <si>
     <t>20:15</t>
+  </si>
+  <si>
+    <t>2026-10-20</t>
   </si>
 </sst>
 </file>
@@ -1919,7 +1922,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G1295"/>
+  <dimension ref="A1:G1298"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
@@ -31701,6 +31704,75 @@
         <v>11</v>
       </c>
     </row>
+    <row r="1296" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1296" s="5" t="s">
+        <v>495</v>
+      </c>
+      <c r="B1296" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1296" s="5" t="s">
+        <v>457</v>
+      </c>
+      <c r="D1296" s="5">
+        <v>13.5</v>
+      </c>
+      <c r="E1296" s="5">
+        <v>75</v>
+      </c>
+      <c r="F1296" s="5">
+        <v>15</v>
+      </c>
+      <c r="G1296" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1297" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1297" s="5" t="s">
+        <v>495</v>
+      </c>
+      <c r="B1297" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="C1297" s="5" t="s">
+        <v>457</v>
+      </c>
+      <c r="D1297" s="5">
+        <v>14.5</v>
+      </c>
+      <c r="E1297" s="5">
+        <v>72</v>
+      </c>
+      <c r="F1297" s="5">
+        <v>16</v>
+      </c>
+      <c r="G1297" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1298" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1298" s="5" t="s">
+        <v>495</v>
+      </c>
+      <c r="B1298" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="C1298" s="5" t="s">
+        <v>457</v>
+      </c>
+      <c r="D1298" s="5">
+        <v>14.8</v>
+      </c>
+      <c r="E1298" s="5">
+        <v>70</v>
+      </c>
+      <c r="F1298" s="5">
+        <v>16</v>
+      </c>
+      <c r="G1298" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>

</xml_diff>

<commit_message>
📊 체감온도 기록: 2026-10-20 15:36 KST
</commit_message>
<xml_diff>
--- a/data/체감온도기록_2026.xlsx
+++ b/data/체감온도기록_2026.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5212" uniqueCount="496">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5232" uniqueCount="496">
   <si>
     <t>성동자이리버뷰 체감온도 기록</t>
   </si>
@@ -1922,7 +1922,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G1298"/>
+  <dimension ref="A1:G1303"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
@@ -31773,6 +31773,121 @@
         <v>11</v>
       </c>
     </row>
+    <row r="1299" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1299" s="5" t="s">
+        <v>495</v>
+      </c>
+      <c r="B1299" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1299" s="5" t="s">
+        <v>434</v>
+      </c>
+      <c r="D1299" s="5">
+        <v>17.4</v>
+      </c>
+      <c r="E1299" s="5">
+        <v>61</v>
+      </c>
+      <c r="F1299" s="5">
+        <v>18</v>
+      </c>
+      <c r="G1299" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1300" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1300" s="5" t="s">
+        <v>495</v>
+      </c>
+      <c r="B1300" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="C1300" s="5" t="s">
+        <v>434</v>
+      </c>
+      <c r="D1300" s="5">
+        <v>20.3</v>
+      </c>
+      <c r="E1300" s="5">
+        <v>54</v>
+      </c>
+      <c r="F1300" s="5">
+        <v>20</v>
+      </c>
+      <c r="G1300" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1301" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1301" s="5" t="s">
+        <v>495</v>
+      </c>
+      <c r="B1301" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="C1301" s="5" t="s">
+        <v>434</v>
+      </c>
+      <c r="D1301" s="5">
+        <v>20.5</v>
+      </c>
+      <c r="E1301" s="5">
+        <v>48</v>
+      </c>
+      <c r="F1301" s="5">
+        <v>20</v>
+      </c>
+      <c r="G1301" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1302" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1302" s="5" t="s">
+        <v>495</v>
+      </c>
+      <c r="B1302" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1302" s="5" t="s">
+        <v>434</v>
+      </c>
+      <c r="D1302" s="5">
+        <v>22.3</v>
+      </c>
+      <c r="E1302" s="5">
+        <v>43</v>
+      </c>
+      <c r="F1302" s="5">
+        <v>22</v>
+      </c>
+      <c r="G1302" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1303" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1303" s="5" t="s">
+        <v>495</v>
+      </c>
+      <c r="B1303" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="C1303" s="5" t="s">
+        <v>434</v>
+      </c>
+      <c r="D1303" s="5">
+        <v>22.5</v>
+      </c>
+      <c r="E1303" s="5">
+        <v>34</v>
+      </c>
+      <c r="F1303" s="5">
+        <v>21</v>
+      </c>
+      <c r="G1303" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>

</xml_diff>

<commit_message>
📊 체감온도 기록: 2026-10-20 21:12 KST
</commit_message>
<xml_diff>
--- a/data/체감온도기록_2026.xlsx
+++ b/data/체감온도기록_2026.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5232" uniqueCount="496">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5244" uniqueCount="497">
   <si>
     <t>성동자이리버뷰 체감온도 기록</t>
   </si>
@@ -1502,6 +1502,9 @@
   </si>
   <si>
     <t>2026-10-20</t>
+  </si>
+  <si>
+    <t>21:11</t>
   </si>
 </sst>
 </file>
@@ -1922,7 +1925,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G1303"/>
+  <dimension ref="A1:G1306"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
@@ -31888,6 +31891,75 @@
         <v>11</v>
       </c>
     </row>
+    <row r="1304" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1304" s="5" t="s">
+        <v>495</v>
+      </c>
+      <c r="B1304" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="C1304" s="5" t="s">
+        <v>496</v>
+      </c>
+      <c r="D1304" s="5">
+        <v>23</v>
+      </c>
+      <c r="E1304" s="5">
+        <v>34</v>
+      </c>
+      <c r="F1304" s="5">
+        <v>21</v>
+      </c>
+      <c r="G1304" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1305" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1305" s="5" t="s">
+        <v>495</v>
+      </c>
+      <c r="B1305" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1305" s="5" t="s">
+        <v>496</v>
+      </c>
+      <c r="D1305" s="5">
+        <v>22.4</v>
+      </c>
+      <c r="E1305" s="5">
+        <v>35</v>
+      </c>
+      <c r="F1305" s="5">
+        <v>21</v>
+      </c>
+      <c r="G1305" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1306" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1306" s="5" t="s">
+        <v>495</v>
+      </c>
+      <c r="B1306" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="C1306" s="5" t="s">
+        <v>496</v>
+      </c>
+      <c r="D1306" s="5">
+        <v>21.3</v>
+      </c>
+      <c r="E1306" s="5">
+        <v>45</v>
+      </c>
+      <c r="F1306" s="5">
+        <v>21</v>
+      </c>
+      <c r="G1306" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>

</xml_diff>

<commit_message>
📊 체감온도 기록: 2026-10-21 09:57 KST
</commit_message>
<xml_diff>
--- a/data/체감온도기록_2026.xlsx
+++ b/data/체감온도기록_2026.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5244" uniqueCount="497">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5256" uniqueCount="499">
   <si>
     <t>성동자이리버뷰 체감온도 기록</t>
   </si>
@@ -1505,6 +1505,12 @@
   </si>
   <si>
     <t>21:11</t>
+  </si>
+  <si>
+    <t>2026-10-21</t>
+  </si>
+  <si>
+    <t>09:57</t>
   </si>
 </sst>
 </file>
@@ -1925,7 +1931,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G1306"/>
+  <dimension ref="A1:G1309"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
@@ -31960,6 +31966,75 @@
         <v>11</v>
       </c>
     </row>
+    <row r="1307" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1307" s="5" t="s">
+        <v>497</v>
+      </c>
+      <c r="B1307" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1307" s="5" t="s">
+        <v>498</v>
+      </c>
+      <c r="D1307" s="5">
+        <v>16.1</v>
+      </c>
+      <c r="E1307" s="5">
+        <v>69</v>
+      </c>
+      <c r="F1307" s="5">
+        <v>17</v>
+      </c>
+      <c r="G1307" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1308" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1308" s="5" t="s">
+        <v>497</v>
+      </c>
+      <c r="B1308" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="C1308" s="5" t="s">
+        <v>498</v>
+      </c>
+      <c r="D1308" s="5">
+        <v>15.7</v>
+      </c>
+      <c r="E1308" s="5">
+        <v>78</v>
+      </c>
+      <c r="F1308" s="5">
+        <v>17</v>
+      </c>
+      <c r="G1308" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1309" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1309" s="5" t="s">
+        <v>497</v>
+      </c>
+      <c r="B1309" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="C1309" s="5" t="s">
+        <v>498</v>
+      </c>
+      <c r="D1309" s="5">
+        <v>15</v>
+      </c>
+      <c r="E1309" s="5">
+        <v>73</v>
+      </c>
+      <c r="F1309" s="5">
+        <v>16</v>
+      </c>
+      <c r="G1309" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>

</xml_diff>

<commit_message>
📊 체감온도 기록: 2026-10-21 15:34 KST
</commit_message>
<xml_diff>
--- a/data/체감온도기록_2026.xlsx
+++ b/data/체감온도기록_2026.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5256" uniqueCount="499">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5276" uniqueCount="499">
   <si>
     <t>성동자이리버뷰 체감온도 기록</t>
   </si>
@@ -1931,7 +1931,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G1309"/>
+  <dimension ref="A1:G1314"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
@@ -32035,6 +32035,121 @@
         <v>11</v>
       </c>
     </row>
+    <row r="1310" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1310" s="5" t="s">
+        <v>497</v>
+      </c>
+      <c r="B1310" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1310" s="5" t="s">
+        <v>289</v>
+      </c>
+      <c r="D1310" s="5">
+        <v>15</v>
+      </c>
+      <c r="E1310" s="5">
+        <v>71</v>
+      </c>
+      <c r="F1310" s="5">
+        <v>16</v>
+      </c>
+      <c r="G1310" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1311" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1311" s="5" t="s">
+        <v>497</v>
+      </c>
+      <c r="B1311" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="C1311" s="5" t="s">
+        <v>289</v>
+      </c>
+      <c r="D1311" s="5">
+        <v>16.1</v>
+      </c>
+      <c r="E1311" s="5">
+        <v>49</v>
+      </c>
+      <c r="F1311" s="5">
+        <v>16</v>
+      </c>
+      <c r="G1311" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1312" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1312" s="5" t="s">
+        <v>497</v>
+      </c>
+      <c r="B1312" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="C1312" s="5" t="s">
+        <v>289</v>
+      </c>
+      <c r="D1312" s="5">
+        <v>16.5</v>
+      </c>
+      <c r="E1312" s="5">
+        <v>41</v>
+      </c>
+      <c r="F1312" s="5">
+        <v>16</v>
+      </c>
+      <c r="G1312" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1313" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1313" s="5" t="s">
+        <v>497</v>
+      </c>
+      <c r="B1313" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1313" s="5" t="s">
+        <v>289</v>
+      </c>
+      <c r="D1313" s="5">
+        <v>15.6</v>
+      </c>
+      <c r="E1313" s="5">
+        <v>41</v>
+      </c>
+      <c r="F1313" s="5">
+        <v>15</v>
+      </c>
+      <c r="G1313" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1314" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1314" s="5" t="s">
+        <v>497</v>
+      </c>
+      <c r="B1314" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="C1314" s="5" t="s">
+        <v>289</v>
+      </c>
+      <c r="D1314" s="5">
+        <v>15.3</v>
+      </c>
+      <c r="E1314" s="5">
+        <v>29</v>
+      </c>
+      <c r="F1314" s="5">
+        <v>14</v>
+      </c>
+      <c r="G1314" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>

</xml_diff>

<commit_message>
📊 체감온도 기록: 2026-10-21 21:25 KST
</commit_message>
<xml_diff>
--- a/data/체감온도기록_2026.xlsx
+++ b/data/체감온도기록_2026.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5276" uniqueCount="499">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5288" uniqueCount="500">
   <si>
     <t>성동자이리버뷰 체감온도 기록</t>
   </si>
@@ -1511,6 +1511,9 @@
   </si>
   <si>
     <t>09:57</t>
+  </si>
+  <si>
+    <t>21:25</t>
   </si>
 </sst>
 </file>
@@ -1931,7 +1934,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G1314"/>
+  <dimension ref="A1:G1317"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
@@ -32150,6 +32153,75 @@
         <v>11</v>
       </c>
     </row>
+    <row r="1315" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1315" s="5" t="s">
+        <v>497</v>
+      </c>
+      <c r="B1315" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="C1315" s="5" t="s">
+        <v>499</v>
+      </c>
+      <c r="D1315" s="5">
+        <v>14.6</v>
+      </c>
+      <c r="E1315" s="5">
+        <v>28</v>
+      </c>
+      <c r="F1315" s="5">
+        <v>13</v>
+      </c>
+      <c r="G1315" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1316" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1316" s="5" t="s">
+        <v>497</v>
+      </c>
+      <c r="B1316" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1316" s="5" t="s">
+        <v>499</v>
+      </c>
+      <c r="D1316" s="5">
+        <v>14.1</v>
+      </c>
+      <c r="E1316" s="5">
+        <v>32</v>
+      </c>
+      <c r="F1316" s="5">
+        <v>13</v>
+      </c>
+      <c r="G1316" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1317" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1317" s="5" t="s">
+        <v>497</v>
+      </c>
+      <c r="B1317" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="C1317" s="5" t="s">
+        <v>499</v>
+      </c>
+      <c r="D1317" s="5">
+        <v>13.7</v>
+      </c>
+      <c r="E1317" s="5">
+        <v>34</v>
+      </c>
+      <c r="F1317" s="5">
+        <v>13</v>
+      </c>
+      <c r="G1317" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>

</xml_diff>

<commit_message>
📊 체감온도 기록: 2026-10-22 09:54 KST
</commit_message>
<xml_diff>
--- a/data/체감온도기록_2026.xlsx
+++ b/data/체감온도기록_2026.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5288" uniqueCount="500">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5300" uniqueCount="502">
   <si>
     <t>성동자이리버뷰 체감온도 기록</t>
   </si>
@@ -1514,6 +1514,12 @@
   </si>
   <si>
     <t>21:25</t>
+  </si>
+  <si>
+    <t>2026-10-22</t>
+  </si>
+  <si>
+    <t>09:53</t>
   </si>
 </sst>
 </file>
@@ -1934,7 +1940,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G1317"/>
+  <dimension ref="A1:G1320"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
@@ -32222,6 +32228,75 @@
         <v>11</v>
       </c>
     </row>
+    <row r="1318" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1318" s="5" t="s">
+        <v>500</v>
+      </c>
+      <c r="B1318" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1318" s="5" t="s">
+        <v>501</v>
+      </c>
+      <c r="D1318" s="5">
+        <v>6.8</v>
+      </c>
+      <c r="E1318" s="5">
+        <v>61</v>
+      </c>
+      <c r="F1318" s="5">
+        <v>8</v>
+      </c>
+      <c r="G1318" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1319" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1319" s="5" t="s">
+        <v>500</v>
+      </c>
+      <c r="B1319" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="C1319" s="5" t="s">
+        <v>501</v>
+      </c>
+      <c r="D1319" s="5">
+        <v>7.7</v>
+      </c>
+      <c r="E1319" s="5">
+        <v>57</v>
+      </c>
+      <c r="F1319" s="5">
+        <v>8</v>
+      </c>
+      <c r="G1319" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1320" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1320" s="5" t="s">
+        <v>500</v>
+      </c>
+      <c r="B1320" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="C1320" s="5" t="s">
+        <v>501</v>
+      </c>
+      <c r="D1320" s="5">
+        <v>9</v>
+      </c>
+      <c r="E1320" s="5">
+        <v>44</v>
+      </c>
+      <c r="F1320" s="5">
+        <v>9</v>
+      </c>
+      <c r="G1320" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>

</xml_diff>

<commit_message>
📊 체감온도 기록: 2026-10-22 15:34 KST
</commit_message>
<xml_diff>
--- a/data/체감온도기록_2026.xlsx
+++ b/data/체감온도기록_2026.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5300" uniqueCount="502">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5320" uniqueCount="502">
   <si>
     <t>성동자이리버뷰 체감온도 기록</t>
   </si>
@@ -1940,7 +1940,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G1320"/>
+  <dimension ref="A1:G1325"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
@@ -32297,6 +32297,121 @@
         <v>11</v>
       </c>
     </row>
+    <row r="1321" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1321" s="5" t="s">
+        <v>500</v>
+      </c>
+      <c r="B1321" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1321" s="5" t="s">
+        <v>289</v>
+      </c>
+      <c r="D1321" s="5">
+        <v>9.9</v>
+      </c>
+      <c r="E1321" s="5">
+        <v>34</v>
+      </c>
+      <c r="F1321" s="5">
+        <v>9</v>
+      </c>
+      <c r="G1321" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1322" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1322" s="5" t="s">
+        <v>500</v>
+      </c>
+      <c r="B1322" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="C1322" s="5" t="s">
+        <v>289</v>
+      </c>
+      <c r="D1322" s="5">
+        <v>11.9</v>
+      </c>
+      <c r="E1322" s="5">
+        <v>24</v>
+      </c>
+      <c r="F1322" s="5">
+        <v>11</v>
+      </c>
+      <c r="G1322" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1323" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1323" s="5" t="s">
+        <v>500</v>
+      </c>
+      <c r="B1323" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="C1323" s="5" t="s">
+        <v>289</v>
+      </c>
+      <c r="D1323" s="5">
+        <v>13.5</v>
+      </c>
+      <c r="E1323" s="5">
+        <v>26</v>
+      </c>
+      <c r="F1323" s="5">
+        <v>12</v>
+      </c>
+      <c r="G1323" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1324" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1324" s="5" t="s">
+        <v>500</v>
+      </c>
+      <c r="B1324" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1324" s="5" t="s">
+        <v>289</v>
+      </c>
+      <c r="D1324" s="5">
+        <v>13.4</v>
+      </c>
+      <c r="E1324" s="5">
+        <v>26</v>
+      </c>
+      <c r="F1324" s="5">
+        <v>12</v>
+      </c>
+      <c r="G1324" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1325" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1325" s="5" t="s">
+        <v>500</v>
+      </c>
+      <c r="B1325" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="C1325" s="5" t="s">
+        <v>289</v>
+      </c>
+      <c r="D1325" s="5">
+        <v>14.7</v>
+      </c>
+      <c r="E1325" s="5">
+        <v>25</v>
+      </c>
+      <c r="F1325" s="5">
+        <v>13</v>
+      </c>
+      <c r="G1325" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>

</xml_diff>

<commit_message>
📊 체감온도 기록: 2026-10-22 21:26 KST
</commit_message>
<xml_diff>
--- a/data/체감온도기록_2026.xlsx
+++ b/data/체감온도기록_2026.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5320" uniqueCount="502">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5332" uniqueCount="502">
   <si>
     <t>성동자이리버뷰 체감온도 기록</t>
   </si>
@@ -1940,7 +1940,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G1325"/>
+  <dimension ref="A1:G1328"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
@@ -32412,6 +32412,75 @@
         <v>11</v>
       </c>
     </row>
+    <row r="1326" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1326" s="5" t="s">
+        <v>500</v>
+      </c>
+      <c r="B1326" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="C1326" s="5" t="s">
+        <v>499</v>
+      </c>
+      <c r="D1326" s="5">
+        <v>15.5</v>
+      </c>
+      <c r="E1326" s="5">
+        <v>24</v>
+      </c>
+      <c r="F1326" s="5">
+        <v>14</v>
+      </c>
+      <c r="G1326" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1327" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1327" s="5" t="s">
+        <v>500</v>
+      </c>
+      <c r="B1327" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1327" s="5" t="s">
+        <v>499</v>
+      </c>
+      <c r="D1327" s="5">
+        <v>15.2</v>
+      </c>
+      <c r="E1327" s="5">
+        <v>21</v>
+      </c>
+      <c r="F1327" s="5">
+        <v>13</v>
+      </c>
+      <c r="G1327" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1328" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1328" s="5" t="s">
+        <v>500</v>
+      </c>
+      <c r="B1328" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="C1328" s="5" t="s">
+        <v>499</v>
+      </c>
+      <c r="D1328" s="5">
+        <v>15</v>
+      </c>
+      <c r="E1328" s="5">
+        <v>24</v>
+      </c>
+      <c r="F1328" s="5">
+        <v>13</v>
+      </c>
+      <c r="G1328" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>

</xml_diff>

<commit_message>
📊 체감온도 기록: 2026-10-23 09:56 KST
</commit_message>
<xml_diff>
--- a/data/체감온도기록_2026.xlsx
+++ b/data/체감온도기록_2026.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5332" uniqueCount="502">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5344" uniqueCount="503">
   <si>
     <t>성동자이리버뷰 체감온도 기록</t>
   </si>
@@ -1520,6 +1520,9 @@
   </si>
   <si>
     <t>09:53</t>
+  </si>
+  <si>
+    <t>2026-10-23</t>
   </si>
 </sst>
 </file>
@@ -1940,7 +1943,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G1328"/>
+  <dimension ref="A1:G1331"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
@@ -32481,6 +32484,75 @@
         <v>11</v>
       </c>
     </row>
+    <row r="1329" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1329" s="5" t="s">
+        <v>502</v>
+      </c>
+      <c r="B1329" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1329" s="5" t="s">
+        <v>429</v>
+      </c>
+      <c r="D1329" s="5">
+        <v>8.4</v>
+      </c>
+      <c r="E1329" s="5">
+        <v>62</v>
+      </c>
+      <c r="F1329" s="5">
+        <v>9</v>
+      </c>
+      <c r="G1329" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1330" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1330" s="5" t="s">
+        <v>502</v>
+      </c>
+      <c r="B1330" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="C1330" s="5" t="s">
+        <v>429</v>
+      </c>
+      <c r="D1330" s="5">
+        <v>9.9</v>
+      </c>
+      <c r="E1330" s="5">
+        <v>59</v>
+      </c>
+      <c r="F1330" s="5">
+        <v>11</v>
+      </c>
+      <c r="G1330" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1331" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1331" s="5" t="s">
+        <v>502</v>
+      </c>
+      <c r="B1331" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="C1331" s="5" t="s">
+        <v>429</v>
+      </c>
+      <c r="D1331" s="5">
+        <v>11.1</v>
+      </c>
+      <c r="E1331" s="5">
+        <v>53</v>
+      </c>
+      <c r="F1331" s="5">
+        <v>11</v>
+      </c>
+      <c r="G1331" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>

</xml_diff>

<commit_message>
📊 체감온도 기록: 2026-10-23 15:28 KST
</commit_message>
<xml_diff>
--- a/data/체감온도기록_2026.xlsx
+++ b/data/체감온도기록_2026.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5344" uniqueCount="503">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5364" uniqueCount="504">
   <si>
     <t>성동자이리버뷰 체감온도 기록</t>
   </si>
@@ -1523,6 +1523,9 @@
   </si>
   <si>
     <t>2026-10-23</t>
+  </si>
+  <si>
+    <t>15:28</t>
   </si>
 </sst>
 </file>
@@ -1943,7 +1946,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G1331"/>
+  <dimension ref="A1:G1336"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
@@ -32553,6 +32556,121 @@
         <v>11</v>
       </c>
     </row>
+    <row r="1332" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1332" s="5" t="s">
+        <v>502</v>
+      </c>
+      <c r="B1332" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1332" s="5" t="s">
+        <v>503</v>
+      </c>
+      <c r="D1332" s="5">
+        <v>13.9</v>
+      </c>
+      <c r="E1332" s="5">
+        <v>47</v>
+      </c>
+      <c r="F1332" s="5">
+        <v>14</v>
+      </c>
+      <c r="G1332" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1333" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1333" s="5" t="s">
+        <v>502</v>
+      </c>
+      <c r="B1333" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="C1333" s="5" t="s">
+        <v>503</v>
+      </c>
+      <c r="D1333" s="5">
+        <v>15.8</v>
+      </c>
+      <c r="E1333" s="5">
+        <v>45</v>
+      </c>
+      <c r="F1333" s="5">
+        <v>15</v>
+      </c>
+      <c r="G1333" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1334" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1334" s="5" t="s">
+        <v>502</v>
+      </c>
+      <c r="B1334" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="C1334" s="5" t="s">
+        <v>503</v>
+      </c>
+      <c r="D1334" s="5">
+        <v>17.8</v>
+      </c>
+      <c r="E1334" s="5">
+        <v>45</v>
+      </c>
+      <c r="F1334" s="5">
+        <v>17</v>
+      </c>
+      <c r="G1334" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1335" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1335" s="5" t="s">
+        <v>502</v>
+      </c>
+      <c r="B1335" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1335" s="5" t="s">
+        <v>503</v>
+      </c>
+      <c r="D1335" s="5">
+        <v>18.6</v>
+      </c>
+      <c r="E1335" s="5">
+        <v>48</v>
+      </c>
+      <c r="F1335" s="5">
+        <v>18</v>
+      </c>
+      <c r="G1335" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1336" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1336" s="5" t="s">
+        <v>502</v>
+      </c>
+      <c r="B1336" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="C1336" s="5" t="s">
+        <v>503</v>
+      </c>
+      <c r="D1336" s="5">
+        <v>20.4</v>
+      </c>
+      <c r="E1336" s="5">
+        <v>47</v>
+      </c>
+      <c r="F1336" s="5">
+        <v>20</v>
+      </c>
+      <c r="G1336" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>

</xml_diff>

<commit_message>
📊 체감온도 기록: 2026-10-23 21:07 KST
</commit_message>
<xml_diff>
--- a/data/체감온도기록_2026.xlsx
+++ b/data/체감온도기록_2026.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5364" uniqueCount="504">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5376" uniqueCount="504">
   <si>
     <t>성동자이리버뷰 체감온도 기록</t>
   </si>
@@ -1946,7 +1946,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G1336"/>
+  <dimension ref="A1:G1339"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
@@ -32671,6 +32671,75 @@
         <v>11</v>
       </c>
     </row>
+    <row r="1337" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1337" s="5" t="s">
+        <v>502</v>
+      </c>
+      <c r="B1337" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="C1337" s="5" t="s">
+        <v>481</v>
+      </c>
+      <c r="D1337" s="5">
+        <v>21.6</v>
+      </c>
+      <c r="E1337" s="5">
+        <v>45</v>
+      </c>
+      <c r="F1337" s="5">
+        <v>21</v>
+      </c>
+      <c r="G1337" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1338" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1338" s="5" t="s">
+        <v>502</v>
+      </c>
+      <c r="B1338" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1338" s="5" t="s">
+        <v>481</v>
+      </c>
+      <c r="D1338" s="5">
+        <v>21.1</v>
+      </c>
+      <c r="E1338" s="5">
+        <v>49</v>
+      </c>
+      <c r="F1338" s="5">
+        <v>21</v>
+      </c>
+      <c r="G1338" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1339" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1339" s="5" t="s">
+        <v>502</v>
+      </c>
+      <c r="B1339" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="C1339" s="5" t="s">
+        <v>481</v>
+      </c>
+      <c r="D1339" s="5">
+        <v>20.4</v>
+      </c>
+      <c r="E1339" s="5">
+        <v>50</v>
+      </c>
+      <c r="F1339" s="5">
+        <v>20</v>
+      </c>
+      <c r="G1339" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>

</xml_diff>

<commit_message>
📊 체감온도 기록: 2026-10-24 10:05 KST
</commit_message>
<xml_diff>
--- a/data/체감온도기록_2026.xlsx
+++ b/data/체감온도기록_2026.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5376" uniqueCount="504">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5388" uniqueCount="506">
   <si>
     <t>성동자이리버뷰 체감온도 기록</t>
   </si>
@@ -1526,6 +1526,12 @@
   </si>
   <si>
     <t>15:28</t>
+  </si>
+  <si>
+    <t>2026-10-24</t>
+  </si>
+  <si>
+    <t>10:05</t>
   </si>
 </sst>
 </file>
@@ -1946,7 +1952,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G1339"/>
+  <dimension ref="A1:G1342"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
@@ -32740,6 +32746,75 @@
         <v>11</v>
       </c>
     </row>
+    <row r="1340" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1340" s="5" t="s">
+        <v>504</v>
+      </c>
+      <c r="B1340" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1340" s="5" t="s">
+        <v>505</v>
+      </c>
+      <c r="D1340" s="5">
+        <v>15.3</v>
+      </c>
+      <c r="E1340" s="5">
+        <v>78</v>
+      </c>
+      <c r="F1340" s="5">
+        <v>17</v>
+      </c>
+      <c r="G1340" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1341" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1341" s="5" t="s">
+        <v>504</v>
+      </c>
+      <c r="B1341" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="C1341" s="5" t="s">
+        <v>505</v>
+      </c>
+      <c r="D1341" s="5">
+        <v>15.4</v>
+      </c>
+      <c r="E1341" s="5">
+        <v>77</v>
+      </c>
+      <c r="F1341" s="5">
+        <v>17</v>
+      </c>
+      <c r="G1341" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1342" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1342" s="5" t="s">
+        <v>504</v>
+      </c>
+      <c r="B1342" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="C1342" s="5" t="s">
+        <v>505</v>
+      </c>
+      <c r="D1342" s="5">
+        <v>15.8</v>
+      </c>
+      <c r="E1342" s="5">
+        <v>73</v>
+      </c>
+      <c r="F1342" s="5">
+        <v>17</v>
+      </c>
+      <c r="G1342" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>

</xml_diff>

<commit_message>
📊 체감온도 기록: 2026-10-24 15:28 KST
</commit_message>
<xml_diff>
--- a/data/체감온도기록_2026.xlsx
+++ b/data/체감온도기록_2026.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5388" uniqueCount="506">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5408" uniqueCount="506">
   <si>
     <t>성동자이리버뷰 체감온도 기록</t>
   </si>
@@ -1952,7 +1952,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G1342"/>
+  <dimension ref="A1:G1347"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
@@ -32815,6 +32815,121 @@
         <v>11</v>
       </c>
     </row>
+    <row r="1343" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1343" s="5" t="s">
+        <v>504</v>
+      </c>
+      <c r="B1343" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1343" s="5" t="s">
+        <v>283</v>
+      </c>
+      <c r="D1343" s="5">
+        <v>16.3</v>
+      </c>
+      <c r="E1343" s="5">
+        <v>72</v>
+      </c>
+      <c r="F1343" s="5">
+        <v>18</v>
+      </c>
+      <c r="G1343" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1344" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1344" s="5" t="s">
+        <v>504</v>
+      </c>
+      <c r="B1344" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="C1344" s="5" t="s">
+        <v>283</v>
+      </c>
+      <c r="D1344" s="5">
+        <v>16.9</v>
+      </c>
+      <c r="E1344" s="5">
+        <v>70</v>
+      </c>
+      <c r="F1344" s="5">
+        <v>18</v>
+      </c>
+      <c r="G1344" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1345" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1345" s="5" t="s">
+        <v>504</v>
+      </c>
+      <c r="B1345" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="C1345" s="5" t="s">
+        <v>283</v>
+      </c>
+      <c r="D1345" s="5">
+        <v>17.2</v>
+      </c>
+      <c r="E1345" s="5">
+        <v>68</v>
+      </c>
+      <c r="F1345" s="5">
+        <v>18</v>
+      </c>
+      <c r="G1345" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1346" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1346" s="5" t="s">
+        <v>504</v>
+      </c>
+      <c r="B1346" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1346" s="5" t="s">
+        <v>283</v>
+      </c>
+      <c r="D1346" s="5">
+        <v>18</v>
+      </c>
+      <c r="E1346" s="5">
+        <v>66</v>
+      </c>
+      <c r="F1346" s="5">
+        <v>19</v>
+      </c>
+      <c r="G1346" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1347" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1347" s="5" t="s">
+        <v>504</v>
+      </c>
+      <c r="B1347" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="C1347" s="5" t="s">
+        <v>283</v>
+      </c>
+      <c r="D1347" s="5">
+        <v>17.7</v>
+      </c>
+      <c r="E1347" s="5">
+        <v>68</v>
+      </c>
+      <c r="F1347" s="5">
+        <v>19</v>
+      </c>
+      <c r="G1347" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>

</xml_diff>

<commit_message>
📊 체감온도 기록: 2026-10-24 20:38 KST
</commit_message>
<xml_diff>
--- a/data/체감온도기록_2026.xlsx
+++ b/data/체감온도기록_2026.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5408" uniqueCount="506">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5420" uniqueCount="507">
   <si>
     <t>성동자이리버뷰 체감온도 기록</t>
   </si>
@@ -1532,6 +1532,9 @@
   </si>
   <si>
     <t>10:05</t>
+  </si>
+  <si>
+    <t>20:38</t>
   </si>
 </sst>
 </file>
@@ -1952,7 +1955,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G1347"/>
+  <dimension ref="A1:G1350"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
@@ -32930,6 +32933,75 @@
         <v>11</v>
       </c>
     </row>
+    <row r="1348" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1348" s="5" t="s">
+        <v>504</v>
+      </c>
+      <c r="B1348" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="C1348" s="5" t="s">
+        <v>506</v>
+      </c>
+      <c r="D1348" s="5">
+        <v>17.9</v>
+      </c>
+      <c r="E1348" s="5">
+        <v>68</v>
+      </c>
+      <c r="F1348" s="5">
+        <v>19</v>
+      </c>
+      <c r="G1348" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1349" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1349" s="5" t="s">
+        <v>504</v>
+      </c>
+      <c r="B1349" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1349" s="5" t="s">
+        <v>506</v>
+      </c>
+      <c r="D1349" s="5">
+        <v>17.5</v>
+      </c>
+      <c r="E1349" s="5">
+        <v>71</v>
+      </c>
+      <c r="F1349" s="5">
+        <v>19</v>
+      </c>
+      <c r="G1349" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1350" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1350" s="5" t="s">
+        <v>504</v>
+      </c>
+      <c r="B1350" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="C1350" s="5" t="s">
+        <v>506</v>
+      </c>
+      <c r="D1350" s="5">
+        <v>17.5</v>
+      </c>
+      <c r="E1350" s="5">
+        <v>72</v>
+      </c>
+      <c r="F1350" s="5">
+        <v>19</v>
+      </c>
+      <c r="G1350" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>

</xml_diff>

<commit_message>
📊 체감온도 기록: 2026-10-25 09:31 KST
</commit_message>
<xml_diff>
--- a/data/체감온도기록_2026.xlsx
+++ b/data/체감온도기록_2026.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5420" uniqueCount="507">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5428" uniqueCount="509">
   <si>
     <t>성동자이리버뷰 체감온도 기록</t>
   </si>
@@ -1535,6 +1535,12 @@
   </si>
   <si>
     <t>20:38</t>
+  </si>
+  <si>
+    <t>2026-10-25</t>
+  </si>
+  <si>
+    <t>09:31</t>
   </si>
 </sst>
 </file>
@@ -1955,7 +1961,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G1350"/>
+  <dimension ref="A1:G1352"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
@@ -33002,6 +33008,52 @@
         <v>11</v>
       </c>
     </row>
+    <row r="1351" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1351" s="5" t="s">
+        <v>507</v>
+      </c>
+      <c r="B1351" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1351" s="5" t="s">
+        <v>508</v>
+      </c>
+      <c r="D1351" s="5">
+        <v>13.3</v>
+      </c>
+      <c r="E1351" s="5">
+        <v>87</v>
+      </c>
+      <c r="F1351" s="5">
+        <v>16</v>
+      </c>
+      <c r="G1351" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1352" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1352" s="5" t="s">
+        <v>507</v>
+      </c>
+      <c r="B1352" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="C1352" s="5" t="s">
+        <v>508</v>
+      </c>
+      <c r="D1352" s="5">
+        <v>14</v>
+      </c>
+      <c r="E1352" s="5">
+        <v>83</v>
+      </c>
+      <c r="F1352" s="5">
+        <v>16</v>
+      </c>
+      <c r="G1352" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>

</xml_diff>

<commit_message>
📊 체감온도 기록: 2026-10-25 14:18 KST
</commit_message>
<xml_diff>
--- a/data/체감온도기록_2026.xlsx
+++ b/data/체감온도기록_2026.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5428" uniqueCount="509">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5448" uniqueCount="509">
   <si>
     <t>성동자이리버뷰 체감온도 기록</t>
   </si>
@@ -1961,7 +1961,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G1352"/>
+  <dimension ref="A1:G1357"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
@@ -33054,6 +33054,121 @@
         <v>11</v>
       </c>
     </row>
+    <row r="1353" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1353" s="5" t="s">
+        <v>507</v>
+      </c>
+      <c r="B1353" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="C1353" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="D1353" s="5">
+        <v>14.7</v>
+      </c>
+      <c r="E1353" s="5">
+        <v>79</v>
+      </c>
+      <c r="F1353" s="5">
+        <v>16</v>
+      </c>
+      <c r="G1353" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1354" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1354" s="5" t="s">
+        <v>507</v>
+      </c>
+      <c r="B1354" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1354" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="D1354" s="5">
+        <v>15.7</v>
+      </c>
+      <c r="E1354" s="5">
+        <v>74</v>
+      </c>
+      <c r="F1354" s="5">
+        <v>17</v>
+      </c>
+      <c r="G1354" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1355" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1355" s="5" t="s">
+        <v>507</v>
+      </c>
+      <c r="B1355" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="C1355" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="D1355" s="5">
+        <v>17.9</v>
+      </c>
+      <c r="E1355" s="5">
+        <v>64</v>
+      </c>
+      <c r="F1355" s="5">
+        <v>19</v>
+      </c>
+      <c r="G1355" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1356" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1356" s="5" t="s">
+        <v>507</v>
+      </c>
+      <c r="B1356" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="C1356" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="D1356" s="5">
+        <v>21.1</v>
+      </c>
+      <c r="E1356" s="5">
+        <v>53</v>
+      </c>
+      <c r="F1356" s="5">
+        <v>21</v>
+      </c>
+      <c r="G1356" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1357" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1357" s="5" t="s">
+        <v>507</v>
+      </c>
+      <c r="B1357" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1357" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="D1357" s="5">
+        <v>21.6</v>
+      </c>
+      <c r="E1357" s="5">
+        <v>52</v>
+      </c>
+      <c r="F1357" s="5">
+        <v>22</v>
+      </c>
+      <c r="G1357" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>

</xml_diff>

<commit_message>
📊 체감온도 기록: 2026-10-25 19:08 KST
</commit_message>
<xml_diff>
--- a/data/체감온도기록_2026.xlsx
+++ b/data/체감온도기록_2026.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5448" uniqueCount="509">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5464" uniqueCount="509">
   <si>
     <t>성동자이리버뷰 체감온도 기록</t>
   </si>
@@ -1961,7 +1961,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G1357"/>
+  <dimension ref="A1:G1361"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
@@ -33169,6 +33169,98 @@
         <v>11</v>
       </c>
     </row>
+    <row r="1358" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1358" s="5" t="s">
+        <v>507</v>
+      </c>
+      <c r="B1358" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="C1358" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="D1358" s="5">
+        <v>22</v>
+      </c>
+      <c r="E1358" s="5">
+        <v>53</v>
+      </c>
+      <c r="F1358" s="5">
+        <v>22</v>
+      </c>
+      <c r="G1358" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1359" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1359" s="5" t="s">
+        <v>507</v>
+      </c>
+      <c r="B1359" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="C1359" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="D1359" s="5">
+        <v>22.3</v>
+      </c>
+      <c r="E1359" s="5">
+        <v>54</v>
+      </c>
+      <c r="F1359" s="5">
+        <v>22</v>
+      </c>
+      <c r="G1359" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1360" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1360" s="5" t="s">
+        <v>507</v>
+      </c>
+      <c r="B1360" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1360" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="D1360" s="5">
+        <v>22.1</v>
+      </c>
+      <c r="E1360" s="5">
+        <v>54</v>
+      </c>
+      <c r="F1360" s="5">
+        <v>22</v>
+      </c>
+      <c r="G1360" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1361" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1361" s="5" t="s">
+        <v>507</v>
+      </c>
+      <c r="B1361" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="C1361" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="D1361" s="5">
+        <v>21.7</v>
+      </c>
+      <c r="E1361" s="5">
+        <v>51</v>
+      </c>
+      <c r="F1361" s="5">
+        <v>22</v>
+      </c>
+      <c r="G1361" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>

</xml_diff>

<commit_message>
📊 체감온도 기록: 2026-10-26 09:43 KST
</commit_message>
<xml_diff>
--- a/data/체감온도기록_2026.xlsx
+++ b/data/체감온도기록_2026.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5464" uniqueCount="509">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5476" uniqueCount="510">
   <si>
     <t>성동자이리버뷰 체감온도 기록</t>
   </si>
@@ -1541,6 +1541,9 @@
   </si>
   <si>
     <t>09:31</t>
+  </si>
+  <si>
+    <t>2026-10-26</t>
   </si>
 </sst>
 </file>
@@ -1961,7 +1964,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G1361"/>
+  <dimension ref="A1:G1364"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
@@ -33261,6 +33264,75 @@
         <v>11</v>
       </c>
     </row>
+    <row r="1362" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1362" s="5" t="s">
+        <v>509</v>
+      </c>
+      <c r="B1362" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1362" s="5" t="s">
+        <v>295</v>
+      </c>
+      <c r="D1362" s="5">
+        <v>13.8</v>
+      </c>
+      <c r="E1362" s="5">
+        <v>82</v>
+      </c>
+      <c r="F1362" s="5">
+        <v>16</v>
+      </c>
+      <c r="G1362" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1363" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1363" s="5" t="s">
+        <v>509</v>
+      </c>
+      <c r="B1363" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="C1363" s="5" t="s">
+        <v>295</v>
+      </c>
+      <c r="D1363" s="5">
+        <v>13.7</v>
+      </c>
+      <c r="E1363" s="5">
+        <v>80</v>
+      </c>
+      <c r="F1363" s="5">
+        <v>16</v>
+      </c>
+      <c r="G1363" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1364" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1364" s="5" t="s">
+        <v>509</v>
+      </c>
+      <c r="B1364" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="C1364" s="5" t="s">
+        <v>295</v>
+      </c>
+      <c r="D1364" s="5">
+        <v>14.6</v>
+      </c>
+      <c r="E1364" s="5">
+        <v>76</v>
+      </c>
+      <c r="F1364" s="5">
+        <v>16</v>
+      </c>
+      <c r="G1364" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>

</xml_diff>

<commit_message>
📊 체감온도 기록: 2026-10-26 14:21 KST
</commit_message>
<xml_diff>
--- a/data/체감온도기록_2026.xlsx
+++ b/data/체감온도기록_2026.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5476" uniqueCount="510">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5492" uniqueCount="510">
   <si>
     <t>성동자이리버뷰 체감온도 기록</t>
   </si>
@@ -1964,7 +1964,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G1364"/>
+  <dimension ref="A1:G1368"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
@@ -33333,6 +33333,98 @@
         <v>11</v>
       </c>
     </row>
+    <row r="1365" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1365" s="5" t="s">
+        <v>509</v>
+      </c>
+      <c r="B1365" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1365" s="5" t="s">
+        <v>402</v>
+      </c>
+      <c r="D1365" s="5">
+        <v>15.8</v>
+      </c>
+      <c r="E1365" s="5">
+        <v>71</v>
+      </c>
+      <c r="F1365" s="5">
+        <v>17</v>
+      </c>
+      <c r="G1365" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1366" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1366" s="5" t="s">
+        <v>509</v>
+      </c>
+      <c r="B1366" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="C1366" s="5" t="s">
+        <v>402</v>
+      </c>
+      <c r="D1366" s="5">
+        <v>16.5</v>
+      </c>
+      <c r="E1366" s="5">
+        <v>68</v>
+      </c>
+      <c r="F1366" s="5">
+        <v>18</v>
+      </c>
+      <c r="G1366" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1367" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1367" s="5" t="s">
+        <v>509</v>
+      </c>
+      <c r="B1367" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="C1367" s="5" t="s">
+        <v>402</v>
+      </c>
+      <c r="D1367" s="5">
+        <v>17.6</v>
+      </c>
+      <c r="E1367" s="5">
+        <v>65</v>
+      </c>
+      <c r="F1367" s="5">
+        <v>19</v>
+      </c>
+      <c r="G1367" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1368" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1368" s="5" t="s">
+        <v>509</v>
+      </c>
+      <c r="B1368" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1368" s="5" t="s">
+        <v>402</v>
+      </c>
+      <c r="D1368" s="5">
+        <v>18.2</v>
+      </c>
+      <c r="E1368" s="5">
+        <v>62</v>
+      </c>
+      <c r="F1368" s="5">
+        <v>19</v>
+      </c>
+      <c r="G1368" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>

</xml_diff>

<commit_message>
📊 체감온도 기록: 2026-10-26 20:36 KST
</commit_message>
<xml_diff>
--- a/data/체감온도기록_2026.xlsx
+++ b/data/체감온도기록_2026.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5492" uniqueCount="510">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5508" uniqueCount="511">
   <si>
     <t>성동자이리버뷰 체감온도 기록</t>
   </si>
@@ -1544,6 +1544,9 @@
   </si>
   <si>
     <t>2026-10-26</t>
+  </si>
+  <si>
+    <t>20:36</t>
   </si>
 </sst>
 </file>
@@ -1964,7 +1967,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G1368"/>
+  <dimension ref="A1:G1372"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
@@ -33425,6 +33428,98 @@
         <v>11</v>
       </c>
     </row>
+    <row r="1369" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1369" s="5" t="s">
+        <v>509</v>
+      </c>
+      <c r="B1369" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="C1369" s="5" t="s">
+        <v>510</v>
+      </c>
+      <c r="D1369" s="5">
+        <v>19.7</v>
+      </c>
+      <c r="E1369" s="5">
+        <v>58</v>
+      </c>
+      <c r="F1369" s="5">
+        <v>20</v>
+      </c>
+      <c r="G1369" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1370" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1370" s="5" t="s">
+        <v>509</v>
+      </c>
+      <c r="B1370" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="C1370" s="5" t="s">
+        <v>510</v>
+      </c>
+      <c r="D1370" s="5">
+        <v>21.2</v>
+      </c>
+      <c r="E1370" s="5">
+        <v>55</v>
+      </c>
+      <c r="F1370" s="5">
+        <v>21</v>
+      </c>
+      <c r="G1370" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1371" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1371" s="5" t="s">
+        <v>509</v>
+      </c>
+      <c r="B1371" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1371" s="5" t="s">
+        <v>510</v>
+      </c>
+      <c r="D1371" s="5">
+        <v>20.5</v>
+      </c>
+      <c r="E1371" s="5">
+        <v>57</v>
+      </c>
+      <c r="F1371" s="5">
+        <v>21</v>
+      </c>
+      <c r="G1371" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1372" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1372" s="5" t="s">
+        <v>509</v>
+      </c>
+      <c r="B1372" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="C1372" s="5" t="s">
+        <v>510</v>
+      </c>
+      <c r="D1372" s="5">
+        <v>19.7</v>
+      </c>
+      <c r="E1372" s="5">
+        <v>60</v>
+      </c>
+      <c r="F1372" s="5">
+        <v>20</v>
+      </c>
+      <c r="G1372" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>

</xml_diff>

<commit_message>
📊 체감온도 기록: 2026-10-27 10:37 KST
</commit_message>
<xml_diff>
--- a/data/체감온도기록_2026.xlsx
+++ b/data/체감온도기록_2026.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5508" uniqueCount="511">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5520" uniqueCount="512">
   <si>
     <t>성동자이리버뷰 체감온도 기록</t>
   </si>
@@ -1547,6 +1547,9 @@
   </si>
   <si>
     <t>20:36</t>
+  </si>
+  <si>
+    <t>2026-10-27</t>
   </si>
 </sst>
 </file>
@@ -1967,7 +1970,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G1372"/>
+  <dimension ref="A1:G1375"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
@@ -33520,6 +33523,75 @@
         <v>11</v>
       </c>
     </row>
+    <row r="1373" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1373" s="5" t="s">
+        <v>511</v>
+      </c>
+      <c r="B1373" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1373" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="D1373" s="5">
+        <v>12</v>
+      </c>
+      <c r="E1373" s="5">
+        <v>36</v>
+      </c>
+      <c r="F1373" s="5">
+        <v>11</v>
+      </c>
+      <c r="G1373" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1374" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1374" s="5" t="s">
+        <v>511</v>
+      </c>
+      <c r="B1374" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="C1374" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="D1374" s="5">
+        <v>12.2</v>
+      </c>
+      <c r="E1374" s="5">
+        <v>28</v>
+      </c>
+      <c r="F1374" s="5">
+        <v>11</v>
+      </c>
+      <c r="G1374" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1375" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1375" s="5" t="s">
+        <v>511</v>
+      </c>
+      <c r="B1375" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="C1375" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="D1375" s="5">
+        <v>13.2</v>
+      </c>
+      <c r="E1375" s="5">
+        <v>26</v>
+      </c>
+      <c r="F1375" s="5">
+        <v>12</v>
+      </c>
+      <c r="G1375" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>

</xml_diff>

<commit_message>
📊 체감온도 기록: 2026-10-27 22:34 KST
</commit_message>
<xml_diff>
--- a/data/체감온도기록_2026.xlsx
+++ b/data/체감온도기록_2026.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5520" uniqueCount="512">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5552" uniqueCount="513">
   <si>
     <t>성동자이리버뷰 체감온도 기록</t>
   </si>
@@ -1550,6 +1550,9 @@
   </si>
   <si>
     <t>2026-10-27</t>
+  </si>
+  <si>
+    <t>22:33</t>
   </si>
 </sst>
 </file>
@@ -1970,7 +1973,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G1375"/>
+  <dimension ref="A1:G1383"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
@@ -33592,6 +33595,190 @@
         <v>11</v>
       </c>
     </row>
+    <row r="1376" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1376" s="5" t="s">
+        <v>511</v>
+      </c>
+      <c r="B1376" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1376" s="5" t="s">
+        <v>512</v>
+      </c>
+      <c r="D1376" s="5">
+        <v>13.9</v>
+      </c>
+      <c r="E1376" s="5">
+        <v>24</v>
+      </c>
+      <c r="F1376" s="5">
+        <v>12</v>
+      </c>
+      <c r="G1376" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1377" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1377" s="5" t="s">
+        <v>511</v>
+      </c>
+      <c r="B1377" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="C1377" s="5" t="s">
+        <v>512</v>
+      </c>
+      <c r="D1377" s="5">
+        <v>14.5</v>
+      </c>
+      <c r="E1377" s="5">
+        <v>28</v>
+      </c>
+      <c r="F1377" s="5">
+        <v>13</v>
+      </c>
+      <c r="G1377" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1378" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1378" s="5" t="s">
+        <v>511</v>
+      </c>
+      <c r="B1378" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="C1378" s="5" t="s">
+        <v>512</v>
+      </c>
+      <c r="D1378" s="5">
+        <v>15.8</v>
+      </c>
+      <c r="E1378" s="5">
+        <v>28</v>
+      </c>
+      <c r="F1378" s="5">
+        <v>14</v>
+      </c>
+      <c r="G1378" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1379" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1379" s="5" t="s">
+        <v>511</v>
+      </c>
+      <c r="B1379" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1379" s="5" t="s">
+        <v>512</v>
+      </c>
+      <c r="D1379" s="5">
+        <v>16.3</v>
+      </c>
+      <c r="E1379" s="5">
+        <v>31</v>
+      </c>
+      <c r="F1379" s="5">
+        <v>15</v>
+      </c>
+      <c r="G1379" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1380" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1380" s="5" t="s">
+        <v>511</v>
+      </c>
+      <c r="B1380" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="C1380" s="5" t="s">
+        <v>512</v>
+      </c>
+      <c r="D1380" s="5">
+        <v>16.1</v>
+      </c>
+      <c r="E1380" s="5">
+        <v>23</v>
+      </c>
+      <c r="F1380" s="5">
+        <v>14</v>
+      </c>
+      <c r="G1380" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1381" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1381" s="5" t="s">
+        <v>511</v>
+      </c>
+      <c r="B1381" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="C1381" s="5" t="s">
+        <v>512</v>
+      </c>
+      <c r="D1381" s="5">
+        <v>15.5</v>
+      </c>
+      <c r="E1381" s="5">
+        <v>21</v>
+      </c>
+      <c r="F1381" s="5">
+        <v>13</v>
+      </c>
+      <c r="G1381" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1382" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1382" s="5" t="s">
+        <v>511</v>
+      </c>
+      <c r="B1382" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1382" s="5" t="s">
+        <v>512</v>
+      </c>
+      <c r="D1382" s="5">
+        <v>14.5</v>
+      </c>
+      <c r="E1382" s="5">
+        <v>20</v>
+      </c>
+      <c r="F1382" s="5">
+        <v>13</v>
+      </c>
+      <c r="G1382" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1383" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1383" s="5" t="s">
+        <v>511</v>
+      </c>
+      <c r="B1383" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="C1383" s="5" t="s">
+        <v>512</v>
+      </c>
+      <c r="D1383" s="5">
+        <v>13</v>
+      </c>
+      <c r="E1383" s="5">
+        <v>21</v>
+      </c>
+      <c r="F1383" s="5">
+        <v>11</v>
+      </c>
+      <c r="G1383" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>

</xml_diff>

<commit_message>
📊 체감온도 기록: 2026-10-28 10:43 KST
</commit_message>
<xml_diff>
--- a/data/체감온도기록_2026.xlsx
+++ b/data/체감온도기록_2026.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5552" uniqueCount="513">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5568" uniqueCount="515">
   <si>
     <t>성동자이리버뷰 체감온도 기록</t>
   </si>
@@ -1553,6 +1553,12 @@
   </si>
   <si>
     <t>22:33</t>
+  </si>
+  <si>
+    <t>2026-10-28</t>
+  </si>
+  <si>
+    <t>10:43</t>
   </si>
 </sst>
 </file>
@@ -1973,7 +1979,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G1383"/>
+  <dimension ref="A1:G1387"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
@@ -33779,6 +33785,98 @@
         <v>11</v>
       </c>
     </row>
+    <row r="1384" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1384" s="5" t="s">
+        <v>513</v>
+      </c>
+      <c r="B1384" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1384" s="5" t="s">
+        <v>514</v>
+      </c>
+      <c r="D1384" s="5">
+        <v>5.4</v>
+      </c>
+      <c r="E1384" s="5">
+        <v>24</v>
+      </c>
+      <c r="F1384" s="5">
+        <v>5</v>
+      </c>
+      <c r="G1384" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1385" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1385" s="5" t="s">
+        <v>513</v>
+      </c>
+      <c r="B1385" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="C1385" s="5" t="s">
+        <v>514</v>
+      </c>
+      <c r="D1385" s="5">
+        <v>5.9</v>
+      </c>
+      <c r="E1385" s="5">
+        <v>23</v>
+      </c>
+      <c r="F1385" s="5">
+        <v>5</v>
+      </c>
+      <c r="G1385" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1386" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1386" s="5" t="s">
+        <v>513</v>
+      </c>
+      <c r="B1386" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="C1386" s="5" t="s">
+        <v>514</v>
+      </c>
+      <c r="D1386" s="5">
+        <v>6.5</v>
+      </c>
+      <c r="E1386" s="5">
+        <v>21</v>
+      </c>
+      <c r="F1386" s="5">
+        <v>6</v>
+      </c>
+      <c r="G1386" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1387" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1387" s="5" t="s">
+        <v>513</v>
+      </c>
+      <c r="B1387" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1387" s="5" t="s">
+        <v>514</v>
+      </c>
+      <c r="D1387" s="5">
+        <v>7.7</v>
+      </c>
+      <c r="E1387" s="5">
+        <v>19</v>
+      </c>
+      <c r="F1387" s="5">
+        <v>7</v>
+      </c>
+      <c r="G1387" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>

</xml_diff>

<commit_message>
📊 체감온도 기록: 2026-10-28 16:28 KST
</commit_message>
<xml_diff>
--- a/data/체감온도기록_2026.xlsx
+++ b/data/체감온도기록_2026.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5568" uniqueCount="515">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5588" uniqueCount="515">
   <si>
     <t>성동자이리버뷰 체감온도 기록</t>
   </si>
@@ -1979,7 +1979,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G1387"/>
+  <dimension ref="A1:G1392"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
@@ -33877,6 +33877,121 @@
         <v>11</v>
       </c>
     </row>
+    <row r="1388" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1388" s="5" t="s">
+        <v>513</v>
+      </c>
+      <c r="B1388" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="C1388" s="5" t="s">
+        <v>338</v>
+      </c>
+      <c r="D1388" s="5">
+        <v>9</v>
+      </c>
+      <c r="E1388" s="5">
+        <v>17</v>
+      </c>
+      <c r="F1388" s="5">
+        <v>8</v>
+      </c>
+      <c r="G1388" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1389" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1389" s="5" t="s">
+        <v>513</v>
+      </c>
+      <c r="B1389" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="C1389" s="5" t="s">
+        <v>338</v>
+      </c>
+      <c r="D1389" s="5">
+        <v>11.9</v>
+      </c>
+      <c r="E1389" s="5">
+        <v>16</v>
+      </c>
+      <c r="F1389" s="5">
+        <v>10</v>
+      </c>
+      <c r="G1389" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1390" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1390" s="5" t="s">
+        <v>513</v>
+      </c>
+      <c r="B1390" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1390" s="5" t="s">
+        <v>338</v>
+      </c>
+      <c r="D1390" s="5">
+        <v>12.7</v>
+      </c>
+      <c r="E1390" s="5">
+        <v>13</v>
+      </c>
+      <c r="F1390" s="5">
+        <v>10</v>
+      </c>
+      <c r="G1390" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1391" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1391" s="5" t="s">
+        <v>513</v>
+      </c>
+      <c r="B1391" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="C1391" s="5" t="s">
+        <v>338</v>
+      </c>
+      <c r="D1391" s="5">
+        <v>13.6</v>
+      </c>
+      <c r="E1391" s="5">
+        <v>13</v>
+      </c>
+      <c r="F1391" s="5">
+        <v>11</v>
+      </c>
+      <c r="G1391" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1392" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1392" s="5" t="s">
+        <v>513</v>
+      </c>
+      <c r="B1392" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="C1392" s="5" t="s">
+        <v>338</v>
+      </c>
+      <c r="D1392" s="5">
+        <v>13.9</v>
+      </c>
+      <c r="E1392" s="5">
+        <v>14</v>
+      </c>
+      <c r="F1392" s="5">
+        <v>12</v>
+      </c>
+      <c r="G1392" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>

</xml_diff>

<commit_message>
📊 체감온도 기록: 2026-10-28 23:30 KST
</commit_message>
<xml_diff>
--- a/data/체감온도기록_2026.xlsx
+++ b/data/체감온도기록_2026.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5588" uniqueCount="515">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5596" uniqueCount="516">
   <si>
     <t>성동자이리버뷰 체감온도 기록</t>
   </si>
@@ -1559,6 +1559,9 @@
   </si>
   <si>
     <t>10:43</t>
+  </si>
+  <si>
+    <t>23:30</t>
   </si>
 </sst>
 </file>
@@ -1979,7 +1982,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G1392"/>
+  <dimension ref="A1:G1394"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
@@ -33992,6 +33995,52 @@
         <v>11</v>
       </c>
     </row>
+    <row r="1393" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1393" s="5" t="s">
+        <v>513</v>
+      </c>
+      <c r="B1393" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1393" s="5" t="s">
+        <v>515</v>
+      </c>
+      <c r="D1393" s="5">
+        <v>14.1</v>
+      </c>
+      <c r="E1393" s="5">
+        <v>16</v>
+      </c>
+      <c r="F1393" s="5">
+        <v>12</v>
+      </c>
+      <c r="G1393" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1394" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1394" s="5" t="s">
+        <v>513</v>
+      </c>
+      <c r="B1394" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="C1394" s="5" t="s">
+        <v>515</v>
+      </c>
+      <c r="D1394" s="5">
+        <v>12.5</v>
+      </c>
+      <c r="E1394" s="5">
+        <v>20</v>
+      </c>
+      <c r="F1394" s="5">
+        <v>11</v>
+      </c>
+      <c r="G1394" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>

</xml_diff>

<commit_message>
📊 체감온도 기록: 2026-10-29 10:56 KST
</commit_message>
<xml_diff>
--- a/data/체감온도기록_2026.xlsx
+++ b/data/체감온도기록_2026.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5596" uniqueCount="516">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5612" uniqueCount="518">
   <si>
     <t>성동자이리버뷰 체감온도 기록</t>
   </si>
@@ -1562,6 +1562,12 @@
   </si>
   <si>
     <t>23:30</t>
+  </si>
+  <si>
+    <t>2026-10-29</t>
+  </si>
+  <si>
+    <t>10:56</t>
   </si>
 </sst>
 </file>
@@ -1982,7 +1988,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G1394"/>
+  <dimension ref="A1:G1398"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
@@ -34041,6 +34047,98 @@
         <v>11</v>
       </c>
     </row>
+    <row r="1395" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1395" s="5" t="s">
+        <v>516</v>
+      </c>
+      <c r="B1395" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1395" s="5" t="s">
+        <v>517</v>
+      </c>
+      <c r="D1395" s="5">
+        <v>6.4</v>
+      </c>
+      <c r="E1395" s="5">
+        <v>59</v>
+      </c>
+      <c r="F1395" s="5">
+        <v>7</v>
+      </c>
+      <c r="G1395" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1396" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1396" s="5" t="s">
+        <v>516</v>
+      </c>
+      <c r="B1396" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="C1396" s="5" t="s">
+        <v>517</v>
+      </c>
+      <c r="D1396" s="5">
+        <v>6.9</v>
+      </c>
+      <c r="E1396" s="5">
+        <v>57</v>
+      </c>
+      <c r="F1396" s="5">
+        <v>8</v>
+      </c>
+      <c r="G1396" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1397" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1397" s="5" t="s">
+        <v>516</v>
+      </c>
+      <c r="B1397" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="C1397" s="5" t="s">
+        <v>517</v>
+      </c>
+      <c r="D1397" s="5">
+        <v>7.5</v>
+      </c>
+      <c r="E1397" s="5">
+        <v>54</v>
+      </c>
+      <c r="F1397" s="5">
+        <v>8</v>
+      </c>
+      <c r="G1397" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1398" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1398" s="5" t="s">
+        <v>516</v>
+      </c>
+      <c r="B1398" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1398" s="5" t="s">
+        <v>517</v>
+      </c>
+      <c r="D1398" s="5">
+        <v>7.9</v>
+      </c>
+      <c r="E1398" s="5">
+        <v>51</v>
+      </c>
+      <c r="F1398" s="5">
+        <v>8</v>
+      </c>
+      <c r="G1398" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>

</xml_diff>

<commit_message>
📊 체감온도 기록: 2026-10-29 17:54 KST
</commit_message>
<xml_diff>
--- a/data/체감온도기록_2026.xlsx
+++ b/data/체감온도기록_2026.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5612" uniqueCount="518">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5640" uniqueCount="518">
   <si>
     <t>성동자이리버뷰 체감온도 기록</t>
   </si>
@@ -1988,7 +1988,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G1398"/>
+  <dimension ref="A1:G1405"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
@@ -34139,6 +34139,167 @@
         <v>11</v>
       </c>
     </row>
+    <row r="1399" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1399" s="5" t="s">
+        <v>516</v>
+      </c>
+      <c r="B1399" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="C1399" s="5" t="s">
+        <v>297</v>
+      </c>
+      <c r="D1399" s="5">
+        <v>7.8</v>
+      </c>
+      <c r="E1399" s="5">
+        <v>56</v>
+      </c>
+      <c r="F1399" s="5">
+        <v>8</v>
+      </c>
+      <c r="G1399" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1400" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1400" s="5" t="s">
+        <v>516</v>
+      </c>
+      <c r="B1400" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="C1400" s="5" t="s">
+        <v>297</v>
+      </c>
+      <c r="D1400" s="5">
+        <v>8.9</v>
+      </c>
+      <c r="E1400" s="5">
+        <v>55</v>
+      </c>
+      <c r="F1400" s="5">
+        <v>9</v>
+      </c>
+      <c r="G1400" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1401" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1401" s="5" t="s">
+        <v>516</v>
+      </c>
+      <c r="B1401" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1401" s="5" t="s">
+        <v>297</v>
+      </c>
+      <c r="D1401" s="5">
+        <v>8.8</v>
+      </c>
+      <c r="E1401" s="5">
+        <v>53</v>
+      </c>
+      <c r="F1401" s="5">
+        <v>9</v>
+      </c>
+      <c r="G1401" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1402" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1402" s="5" t="s">
+        <v>516</v>
+      </c>
+      <c r="B1402" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="C1402" s="5" t="s">
+        <v>297</v>
+      </c>
+      <c r="D1402" s="5">
+        <v>9.3</v>
+      </c>
+      <c r="E1402" s="5">
+        <v>49</v>
+      </c>
+      <c r="F1402" s="5">
+        <v>10</v>
+      </c>
+      <c r="G1402" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1403" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1403" s="5" t="s">
+        <v>516</v>
+      </c>
+      <c r="B1403" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="C1403" s="5" t="s">
+        <v>297</v>
+      </c>
+      <c r="D1403" s="5">
+        <v>10.1</v>
+      </c>
+      <c r="E1403" s="5">
+        <v>48</v>
+      </c>
+      <c r="F1403" s="5">
+        <v>10</v>
+      </c>
+      <c r="G1403" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1404" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1404" s="5" t="s">
+        <v>516</v>
+      </c>
+      <c r="B1404" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1404" s="5" t="s">
+        <v>297</v>
+      </c>
+      <c r="D1404" s="5">
+        <v>10.2</v>
+      </c>
+      <c r="E1404" s="5">
+        <v>48</v>
+      </c>
+      <c r="F1404" s="5">
+        <v>10</v>
+      </c>
+      <c r="G1404" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1405" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1405" s="5" t="s">
+        <v>516</v>
+      </c>
+      <c r="B1405" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="C1405" s="5" t="s">
+        <v>297</v>
+      </c>
+      <c r="D1405" s="5">
+        <v>10.1</v>
+      </c>
+      <c r="E1405" s="5">
+        <v>49</v>
+      </c>
+      <c r="F1405" s="5">
+        <v>10</v>
+      </c>
+      <c r="G1405" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>

</xml_diff>

<commit_message>
📊 체감온도 기록: 2026-10-30 11:08 KST
</commit_message>
<xml_diff>
--- a/data/체감온도기록_2026.xlsx
+++ b/data/체감온도기록_2026.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5640" uniqueCount="518">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5656" uniqueCount="519">
   <si>
     <t>성동자이리버뷰 체감온도 기록</t>
   </si>
@@ -1568,6 +1568,9 @@
   </si>
   <si>
     <t>10:56</t>
+  </si>
+  <si>
+    <t>2026-10-30</t>
   </si>
 </sst>
 </file>
@@ -1988,7 +1991,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G1405"/>
+  <dimension ref="A1:G1409"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
@@ -34300,6 +34303,98 @@
         <v>11</v>
       </c>
     </row>
+    <row r="1406" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1406" s="5" t="s">
+        <v>518</v>
+      </c>
+      <c r="B1406" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1406" s="5" t="s">
+        <v>311</v>
+      </c>
+      <c r="D1406" s="5">
+        <v>7.9</v>
+      </c>
+      <c r="E1406" s="5">
+        <v>88</v>
+      </c>
+      <c r="F1406" s="5">
+        <v>10</v>
+      </c>
+      <c r="G1406" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1407" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1407" s="5" t="s">
+        <v>518</v>
+      </c>
+      <c r="B1407" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="C1407" s="5" t="s">
+        <v>311</v>
+      </c>
+      <c r="D1407" s="5">
+        <v>8.8</v>
+      </c>
+      <c r="E1407" s="5">
+        <v>87</v>
+      </c>
+      <c r="F1407" s="5">
+        <v>11</v>
+      </c>
+      <c r="G1407" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1408" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1408" s="5" t="s">
+        <v>518</v>
+      </c>
+      <c r="B1408" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="C1408" s="5" t="s">
+        <v>311</v>
+      </c>
+      <c r="D1408" s="5">
+        <v>10.4</v>
+      </c>
+      <c r="E1408" s="5">
+        <v>79</v>
+      </c>
+      <c r="F1408" s="5">
+        <v>12</v>
+      </c>
+      <c r="G1408" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1409" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1409" s="5" t="s">
+        <v>518</v>
+      </c>
+      <c r="B1409" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1409" s="5" t="s">
+        <v>311</v>
+      </c>
+      <c r="D1409" s="5">
+        <v>12.5</v>
+      </c>
+      <c r="E1409" s="5">
+        <v>73</v>
+      </c>
+      <c r="F1409" s="5">
+        <v>14</v>
+      </c>
+      <c r="G1409" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>

</xml_diff>

<commit_message>
📊 체감온도 기록: 2026-10-30 17:59 KST
</commit_message>
<xml_diff>
--- a/data/체감온도기록_2026.xlsx
+++ b/data/체감온도기록_2026.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5656" uniqueCount="519">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5684" uniqueCount="519">
   <si>
     <t>성동자이리버뷰 체감온도 기록</t>
   </si>
@@ -1991,7 +1991,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G1409"/>
+  <dimension ref="A1:G1416"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
@@ -34395,6 +34395,167 @@
         <v>11</v>
       </c>
     </row>
+    <row r="1410" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1410" s="5" t="s">
+        <v>518</v>
+      </c>
+      <c r="B1410" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="C1410" s="5" t="s">
+        <v>238</v>
+      </c>
+      <c r="D1410" s="5">
+        <v>14.9</v>
+      </c>
+      <c r="E1410" s="5">
+        <v>66</v>
+      </c>
+      <c r="F1410" s="5">
+        <v>16</v>
+      </c>
+      <c r="G1410" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1411" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1411" s="5" t="s">
+        <v>518</v>
+      </c>
+      <c r="B1411" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="C1411" s="5" t="s">
+        <v>238</v>
+      </c>
+      <c r="D1411" s="5">
+        <v>16.1</v>
+      </c>
+      <c r="E1411" s="5">
+        <v>60</v>
+      </c>
+      <c r="F1411" s="5">
+        <v>17</v>
+      </c>
+      <c r="G1411" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1412" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1412" s="5" t="s">
+        <v>518</v>
+      </c>
+      <c r="B1412" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1412" s="5" t="s">
+        <v>238</v>
+      </c>
+      <c r="D1412" s="5">
+        <v>17.7</v>
+      </c>
+      <c r="E1412" s="5">
+        <v>46</v>
+      </c>
+      <c r="F1412" s="5">
+        <v>17</v>
+      </c>
+      <c r="G1412" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1413" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1413" s="5" t="s">
+        <v>518</v>
+      </c>
+      <c r="B1413" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="C1413" s="5" t="s">
+        <v>238</v>
+      </c>
+      <c r="D1413" s="5">
+        <v>17.7</v>
+      </c>
+      <c r="E1413" s="5">
+        <v>43</v>
+      </c>
+      <c r="F1413" s="5">
+        <v>17</v>
+      </c>
+      <c r="G1413" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1414" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1414" s="5" t="s">
+        <v>518</v>
+      </c>
+      <c r="B1414" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="C1414" s="5" t="s">
+        <v>238</v>
+      </c>
+      <c r="D1414" s="5">
+        <v>18.2</v>
+      </c>
+      <c r="E1414" s="5">
+        <v>45</v>
+      </c>
+      <c r="F1414" s="5">
+        <v>18</v>
+      </c>
+      <c r="G1414" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1415" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1415" s="5" t="s">
+        <v>518</v>
+      </c>
+      <c r="B1415" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1415" s="5" t="s">
+        <v>238</v>
+      </c>
+      <c r="D1415" s="5">
+        <v>17.8</v>
+      </c>
+      <c r="E1415" s="5">
+        <v>38</v>
+      </c>
+      <c r="F1415" s="5">
+        <v>17</v>
+      </c>
+      <c r="G1415" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1416" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1416" s="5" t="s">
+        <v>518</v>
+      </c>
+      <c r="B1416" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="C1416" s="5" t="s">
+        <v>238</v>
+      </c>
+      <c r="D1416" s="5">
+        <v>17.1</v>
+      </c>
+      <c r="E1416" s="5">
+        <v>43</v>
+      </c>
+      <c r="F1416" s="5">
+        <v>17</v>
+      </c>
+      <c r="G1416" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>

</xml_diff>

<commit_message>
📊 체감온도 기록: 2026-10-31 10:48 KST
</commit_message>
<xml_diff>
--- a/data/체감온도기록_2026.xlsx
+++ b/data/체감온도기록_2026.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5684" uniqueCount="519">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5700" uniqueCount="520">
   <si>
     <t>성동자이리버뷰 체감온도 기록</t>
   </si>
@@ -1571,6 +1571,9 @@
   </si>
   <si>
     <t>2026-10-30</t>
+  </si>
+  <si>
+    <t>2026-10-31</t>
   </si>
 </sst>
 </file>
@@ -1991,7 +1994,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G1416"/>
+  <dimension ref="A1:G1420"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
@@ -34556,6 +34559,98 @@
         <v>11</v>
       </c>
     </row>
+    <row r="1417" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1417" s="5" t="s">
+        <v>519</v>
+      </c>
+      <c r="B1417" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1417" s="5" t="s">
+        <v>450</v>
+      </c>
+      <c r="D1417" s="5">
+        <v>12.7</v>
+      </c>
+      <c r="E1417" s="5">
+        <v>85</v>
+      </c>
+      <c r="F1417" s="5">
+        <v>15</v>
+      </c>
+      <c r="G1417" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1418" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1418" s="5" t="s">
+        <v>519</v>
+      </c>
+      <c r="B1418" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="C1418" s="5" t="s">
+        <v>450</v>
+      </c>
+      <c r="D1418" s="5">
+        <v>13.2</v>
+      </c>
+      <c r="E1418" s="5">
+        <v>79</v>
+      </c>
+      <c r="F1418" s="5">
+        <v>15</v>
+      </c>
+      <c r="G1418" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1419" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1419" s="5" t="s">
+        <v>519</v>
+      </c>
+      <c r="B1419" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="C1419" s="5" t="s">
+        <v>450</v>
+      </c>
+      <c r="D1419" s="5">
+        <v>14.1</v>
+      </c>
+      <c r="E1419" s="5">
+        <v>62</v>
+      </c>
+      <c r="F1419" s="5">
+        <v>15</v>
+      </c>
+      <c r="G1419" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1420" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1420" s="5" t="s">
+        <v>519</v>
+      </c>
+      <c r="B1420" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1420" s="5" t="s">
+        <v>450</v>
+      </c>
+      <c r="D1420" s="5">
+        <v>14.2</v>
+      </c>
+      <c r="E1420" s="5">
+        <v>58</v>
+      </c>
+      <c r="F1420" s="5">
+        <v>15</v>
+      </c>
+      <c r="G1420" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>

</xml_diff>

<commit_message>
📊 체감온도 기록: 2026-10-31 17:52 KST
</commit_message>
<xml_diff>
--- a/data/체감온도기록_2026.xlsx
+++ b/data/체감온도기록_2026.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5700" uniqueCount="520">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5728" uniqueCount="521">
   <si>
     <t>성동자이리버뷰 체감온도 기록</t>
   </si>
@@ -1574,6 +1574,9 @@
   </si>
   <si>
     <t>2026-10-31</t>
+  </si>
+  <si>
+    <t>17:52</t>
   </si>
 </sst>
 </file>
@@ -1994,7 +1997,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G1420"/>
+  <dimension ref="A1:G1427"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
@@ -34651,6 +34654,167 @@
         <v>11</v>
       </c>
     </row>
+    <row r="1421" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1421" s="5" t="s">
+        <v>519</v>
+      </c>
+      <c r="B1421" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="C1421" s="5" t="s">
+        <v>520</v>
+      </c>
+      <c r="D1421" s="5">
+        <v>15.6</v>
+      </c>
+      <c r="E1421" s="5">
+        <v>39</v>
+      </c>
+      <c r="F1421" s="5">
+        <v>15</v>
+      </c>
+      <c r="G1421" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1422" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1422" s="5" t="s">
+        <v>519</v>
+      </c>
+      <c r="B1422" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="C1422" s="5" t="s">
+        <v>520</v>
+      </c>
+      <c r="D1422" s="5">
+        <v>16.4</v>
+      </c>
+      <c r="E1422" s="5">
+        <v>33</v>
+      </c>
+      <c r="F1422" s="5">
+        <v>15</v>
+      </c>
+      <c r="G1422" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1423" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1423" s="5" t="s">
+        <v>519</v>
+      </c>
+      <c r="B1423" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1423" s="5" t="s">
+        <v>520</v>
+      </c>
+      <c r="D1423" s="5">
+        <v>16.1</v>
+      </c>
+      <c r="E1423" s="5">
+        <v>31</v>
+      </c>
+      <c r="F1423" s="5">
+        <v>15</v>
+      </c>
+      <c r="G1423" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1424" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1424" s="5" t="s">
+        <v>519</v>
+      </c>
+      <c r="B1424" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="C1424" s="5" t="s">
+        <v>520</v>
+      </c>
+      <c r="D1424" s="5">
+        <v>16</v>
+      </c>
+      <c r="E1424" s="5">
+        <v>21</v>
+      </c>
+      <c r="F1424" s="5">
+        <v>14</v>
+      </c>
+      <c r="G1424" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1425" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1425" s="5" t="s">
+        <v>519</v>
+      </c>
+      <c r="B1425" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="C1425" s="5" t="s">
+        <v>520</v>
+      </c>
+      <c r="D1425" s="5">
+        <v>16.4</v>
+      </c>
+      <c r="E1425" s="5">
+        <v>20</v>
+      </c>
+      <c r="F1425" s="5">
+        <v>14</v>
+      </c>
+      <c r="G1425" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1426" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1426" s="5" t="s">
+        <v>519</v>
+      </c>
+      <c r="B1426" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1426" s="5" t="s">
+        <v>520</v>
+      </c>
+      <c r="D1426" s="5">
+        <v>15.9</v>
+      </c>
+      <c r="E1426" s="5">
+        <v>14</v>
+      </c>
+      <c r="F1426" s="5">
+        <v>13</v>
+      </c>
+      <c r="G1426" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1427" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1427" s="5" t="s">
+        <v>519</v>
+      </c>
+      <c r="B1427" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="C1427" s="5" t="s">
+        <v>520</v>
+      </c>
+      <c r="D1427" s="5">
+        <v>14.5</v>
+      </c>
+      <c r="E1427" s="5">
+        <v>18</v>
+      </c>
+      <c r="F1427" s="5">
+        <v>12</v>
+      </c>
+      <c r="G1427" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>

</xml_diff>